<commit_message>
chore: weekly briefing 2026-09-08 11:57Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-08 19:46 KST</t>
+          <t>2026-09-08 20:57 KST</t>
         </is>
       </c>
     </row>
@@ -791,7 +791,7 @@
       </c>
       <c r="C4" s="16" t="inlineStr">
         <is>
-          <t>AI 반도체 주도 랠리와 경기 둔화 우려의 교차</t>
+          <t>반도체 주도 랠리와 금리 인상 우려 사이의 변동성 장세</t>
         </is>
       </c>
     </row>
@@ -1278,7 +1278,7 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수의 3.37% 급등이 국내 반도체 소부장 및 대형주로 이어지며, 미국 지수 약세에도 불구하고 외국인과 기관의 강력한 매수세를 유도함.</t>
+          <t>필라델피아 반도체 지수의 3.37% 급등과 마이크론 상승세가 국내 반도체 소부장 및 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도함.</t>
         </is>
       </c>
     </row>
@@ -1311,7 +1311,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>미국 국채 금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담을 가중시켰고, 국내 GDP 성장률 둔화와 맞물려 지수 하락을 견인함.</t>
+          <t>미국 국채금리 급등과 UBS의 금리 인상 전망 제기로 인한 투자 심리 위축이 국내 증시의 밸류에이션 부담을 가중시키며 지수 하락을 유발함.</t>
         </is>
       </c>
     </row>
@@ -1351,21 +1351,21 @@
     <row r="30" ht="31" customHeight="1" s="15">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>- 매크로 환경: 미국 비농업 고용지수(162K)가 예상치(55K)를 상회하며 금리 인하 경로 불확실성이 커졌고, 국내 2분기 GDP 성장률(0.6%)은 이전치(1.8%)를 하회하며 경기 둔화 신호가 뚜렷함.</t>
+          <t>- 미국 비농업 고용지표(162K)가 예상치를 상회하고 국내 2분기 GDP(0.6%)가 이전치(1.8%)를 하회하며 매크로 환경의 불확실성이 커짐.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31" customHeight="1" s="15">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>- 수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되었으나, 개인은 전 섹터에서 매도 우위를 보이며 차익 실현에 집중함.</t>
+          <t>- 수급 측면에서는 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되었으나, 개인은 전반적인 차익 실현 매도를 지속함.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="31" customHeight="1" s="15">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>- 종합 관점: AI 반도체 모멘텀이 시장을 견인했으나, 매크로 불확실성과 경기 둔화 우려가 상존하며 수급 쏠림 현상이 심화된 한 주였음.</t>
+          <t>- 반도체 중심의 수급 쏠림이 뚜렷한 가운데, 금리 인상 우려와 경기 둔화 신호가 맞물리며 지수 상단이 제한되는 흐름을 보임.</t>
         </is>
       </c>
     </row>
@@ -1461,25 +1461,25 @@
         </is>
       </c>
       <c r="D36" s="28" t="n">
-        <v>43839</v>
+        <v>45121</v>
       </c>
       <c r="E36" s="28" t="n">
-        <v>20501</v>
+        <v>21100</v>
       </c>
       <c r="F36" s="28" t="n">
-        <v>23338</v>
+        <v>24020</v>
       </c>
       <c r="G36" s="27" t="n">
-        <v>-53897</v>
+        <v>-55192</v>
       </c>
       <c r="H36" s="29" t="n">
         <v>1816.7</v>
       </c>
       <c r="I36" s="29" t="n">
-        <v>247447.2</v>
+        <v>240284.8</v>
       </c>
       <c r="J36" s="29" t="n">
-        <v>0</v>
+        <v>-7162.4</v>
       </c>
     </row>
     <row r="37">
@@ -1497,25 +1497,25 @@
         </is>
       </c>
       <c r="D37" s="28" t="n">
-        <v>28819</v>
+        <v>29092</v>
       </c>
       <c r="E37" s="28" t="n">
-        <v>19070</v>
+        <v>19197</v>
       </c>
       <c r="F37" s="28" t="n">
-        <v>9749</v>
+        <v>9895</v>
       </c>
       <c r="G37" s="27" t="n">
-        <v>-51831</v>
+        <v>-52130</v>
       </c>
       <c r="H37" s="29" t="n">
         <v>3364.2</v>
       </c>
       <c r="I37" s="29" t="n">
-        <v>225804.3</v>
+        <v>223759.5</v>
       </c>
       <c r="J37" s="29" t="n">
-        <v>0</v>
+        <v>-2044.8</v>
       </c>
     </row>
     <row r="38">
@@ -1533,25 +1533,25 @@
         </is>
       </c>
       <c r="D38" s="28" t="n">
-        <v>5236</v>
+        <v>5294</v>
       </c>
       <c r="E38" s="28" t="n">
-        <v>3060</v>
+        <v>3070</v>
       </c>
       <c r="F38" s="28" t="n">
-        <v>2175</v>
+        <v>2223</v>
       </c>
       <c r="G38" s="27" t="n">
-        <v>-5105</v>
+        <v>-5184</v>
       </c>
       <c r="H38" s="29" t="n">
         <v>365.7</v>
       </c>
       <c r="I38" s="29" t="n">
-        <v>32812</v>
+        <v>32891.8</v>
       </c>
       <c r="J38" s="29" t="n">
-        <v>0</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="39">
@@ -1584,10 +1584,10 @@
         <v>206.2</v>
       </c>
       <c r="I39" s="29" t="n">
-        <v>29143.8</v>
+        <v>28477.7</v>
       </c>
       <c r="J39" s="29" t="n">
-        <v>0</v>
+        <v>-666.1</v>
       </c>
     </row>
     <row r="40">
@@ -1605,25 +1605,25 @@
         </is>
       </c>
       <c r="D40" s="28" t="n">
-        <v>2266</v>
-      </c>
-      <c r="E40" s="28" t="n">
-        <v>58</v>
+        <v>2138</v>
+      </c>
+      <c r="E40" s="27" t="n">
+        <v>-81</v>
       </c>
       <c r="F40" s="28" t="n">
-        <v>2208</v>
+        <v>2220</v>
       </c>
       <c r="G40" s="27" t="n">
-        <v>-2304</v>
+        <v>-2125</v>
       </c>
       <c r="H40" s="29" t="n">
         <v>900.5</v>
       </c>
       <c r="I40" s="29" t="n">
-        <v>19475.5</v>
+        <v>19469.6</v>
       </c>
       <c r="J40" s="29" t="n">
-        <v>0</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="41">
@@ -1641,25 +1641,25 @@
         </is>
       </c>
       <c r="D41" s="28" t="n">
-        <v>1369</v>
+        <v>1581</v>
       </c>
       <c r="E41" s="28" t="n">
-        <v>816</v>
+        <v>1000</v>
       </c>
       <c r="F41" s="28" t="n">
-        <v>553</v>
+        <v>581</v>
       </c>
       <c r="G41" s="27" t="n">
-        <v>-1351</v>
+        <v>-1560</v>
       </c>
       <c r="H41" s="29" t="n">
         <v>485.3</v>
       </c>
       <c r="I41" s="29" t="n">
-        <v>44346.7</v>
+        <v>43511.4</v>
       </c>
       <c r="J41" s="29" t="n">
-        <v>0</v>
+        <v>-835.3</v>
       </c>
     </row>
     <row r="42">
@@ -1677,25 +1677,25 @@
         </is>
       </c>
       <c r="D42" s="28" t="n">
-        <v>1309</v>
+        <v>1182</v>
       </c>
       <c r="E42" s="28" t="n">
-        <v>765</v>
+        <v>640</v>
       </c>
       <c r="F42" s="28" t="n">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="G42" s="27" t="n">
-        <v>-1290</v>
+        <v>-1175</v>
       </c>
       <c r="H42" s="29" t="n">
         <v>422.1</v>
       </c>
       <c r="I42" s="29" t="n">
-        <v>10675.8</v>
+        <v>10178.7</v>
       </c>
       <c r="J42" s="29" t="n">
-        <v>0</v>
+        <v>-497.1</v>
       </c>
     </row>
     <row r="43">
@@ -1713,25 +1713,25 @@
         </is>
       </c>
       <c r="D43" s="28" t="n">
-        <v>867</v>
+        <v>852</v>
       </c>
       <c r="E43" s="28" t="n">
-        <v>702</v>
+        <v>687</v>
       </c>
       <c r="F43" s="28" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G43" s="27" t="n">
-        <v>-880</v>
+        <v>-863</v>
       </c>
       <c r="H43" s="29" t="n">
         <v>144</v>
       </c>
       <c r="I43" s="29" t="n">
-        <v>6126.4</v>
+        <v>5502.2</v>
       </c>
       <c r="J43" s="29" t="n">
-        <v>0</v>
+        <v>-624.2</v>
       </c>
     </row>
     <row r="44">
@@ -1764,10 +1764,10 @@
         <v>164.4</v>
       </c>
       <c r="I44" s="29" t="n">
-        <v>5739.7</v>
+        <v>6222.6</v>
       </c>
       <c r="J44" s="29" t="n">
-        <v>0</v>
+        <v>482.9</v>
       </c>
     </row>
     <row r="45">
@@ -1785,25 +1785,25 @@
         </is>
       </c>
       <c r="D45" s="28" t="n">
-        <v>720</v>
+        <v>754</v>
       </c>
       <c r="E45" s="27" t="n">
-        <v>-287</v>
+        <v>-258</v>
       </c>
       <c r="F45" s="28" t="n">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="G45" s="27" t="n">
-        <v>-724</v>
+        <v>-760</v>
       </c>
       <c r="H45" s="29" t="n">
         <v>292.4</v>
       </c>
       <c r="I45" s="29" t="n">
-        <v>8468.6</v>
+        <v>8765.6</v>
       </c>
       <c r="J45" s="29" t="n">
-        <v>0</v>
+        <v>297</v>
       </c>
     </row>
     <row r="46">
@@ -1821,25 +1821,25 @@
         </is>
       </c>
       <c r="D46" s="27" t="n">
-        <v>-1900</v>
+        <v>-3070</v>
       </c>
       <c r="E46" s="27" t="n">
-        <v>-1420</v>
+        <v>-2520</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>-480</v>
+        <v>-550</v>
       </c>
       <c r="G46" s="28" t="n">
-        <v>1869</v>
+        <v>3076</v>
       </c>
       <c r="H46" s="29" t="n">
         <v>686.4</v>
       </c>
       <c r="I46" s="29" t="n">
-        <v>38810</v>
+        <v>36009</v>
       </c>
       <c r="J46" s="29" t="n">
-        <v>0</v>
+        <v>-2801</v>
       </c>
     </row>
     <row r="47">
@@ -1857,25 +1857,25 @@
         </is>
       </c>
       <c r="D47" s="27" t="n">
-        <v>-1526</v>
+        <v>-1568</v>
       </c>
       <c r="E47" s="27" t="n">
-        <v>-657</v>
+        <v>-695</v>
       </c>
       <c r="F47" s="27" t="n">
-        <v>-870</v>
+        <v>-873</v>
       </c>
       <c r="G47" s="28" t="n">
-        <v>1555</v>
+        <v>1591</v>
       </c>
       <c r="H47" s="29" t="n">
         <v>284</v>
       </c>
       <c r="I47" s="29" t="n">
-        <v>13527.9</v>
+        <v>13231</v>
       </c>
       <c r="J47" s="29" t="n">
-        <v>0</v>
+        <v>-296.9</v>
       </c>
     </row>
     <row r="48">
@@ -1893,25 +1893,25 @@
         </is>
       </c>
       <c r="D48" s="27" t="n">
-        <v>-944</v>
+        <v>-968</v>
       </c>
       <c r="E48" s="27" t="n">
-        <v>-113</v>
+        <v>-135</v>
       </c>
       <c r="F48" s="27" t="n">
-        <v>-831</v>
+        <v>-833</v>
       </c>
       <c r="G48" s="28" t="n">
-        <v>942</v>
+        <v>966</v>
       </c>
       <c r="H48" s="29" t="n">
         <v>96.5</v>
       </c>
       <c r="I48" s="29" t="n">
-        <v>8359.200000000001</v>
+        <v>8138.3</v>
       </c>
       <c r="J48" s="29" t="n">
-        <v>0</v>
+        <v>-220.9</v>
       </c>
     </row>
     <row r="49">
@@ -1929,25 +1929,25 @@
         </is>
       </c>
       <c r="D49" s="27" t="n">
-        <v>-751</v>
+        <v>-783</v>
       </c>
       <c r="E49" s="27" t="n">
-        <v>-528</v>
+        <v>-551</v>
       </c>
       <c r="F49" s="27" t="n">
-        <v>-223</v>
+        <v>-232</v>
       </c>
       <c r="G49" s="28" t="n">
-        <v>564</v>
+        <v>626</v>
       </c>
       <c r="H49" s="29" t="n">
         <v>125.5</v>
       </c>
       <c r="I49" s="29" t="n">
-        <v>12830.3</v>
+        <v>12546.7</v>
       </c>
       <c r="J49" s="29" t="n">
-        <v>0</v>
+        <v>-283.6</v>
       </c>
     </row>
     <row r="50">
@@ -1961,29 +1961,29 @@
       </c>
       <c r="C50" s="29" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D50" s="27" t="n">
-        <v>-588</v>
+        <v>-679</v>
       </c>
       <c r="E50" s="27" t="n">
-        <v>-3</v>
+        <v>-292</v>
       </c>
       <c r="F50" s="27" t="n">
-        <v>-585</v>
+        <v>-386</v>
       </c>
       <c r="G50" s="28" t="n">
-        <v>590</v>
+        <v>764</v>
       </c>
       <c r="H50" s="29" t="n">
-        <v>133.3</v>
+        <v>419.2</v>
       </c>
       <c r="I50" s="29" t="n">
-        <v>14894.9</v>
+        <v>31440</v>
       </c>
       <c r="J50" s="29" t="n">
-        <v>0</v>
+        <v>-1186.9</v>
       </c>
     </row>
     <row r="51">
@@ -1997,29 +1997,29 @@
       </c>
       <c r="C51" s="29" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="D51" s="27" t="n">
-        <v>-572</v>
+        <v>-629</v>
       </c>
       <c r="E51" s="27" t="n">
-        <v>-204</v>
+        <v>-46</v>
       </c>
       <c r="F51" s="27" t="n">
-        <v>-368</v>
+        <v>-583</v>
       </c>
       <c r="G51" s="28" t="n">
-        <v>658</v>
+        <v>634</v>
       </c>
       <c r="H51" s="29" t="n">
-        <v>419.2</v>
+        <v>133.3</v>
       </c>
       <c r="I51" s="29" t="n">
-        <v>32626.9</v>
+        <v>14504.2</v>
       </c>
       <c r="J51" s="29" t="n">
-        <v>0</v>
+        <v>-390.7</v>
       </c>
     </row>
     <row r="52">
@@ -2033,29 +2033,29 @@
       </c>
       <c r="C52" s="29" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="D52" s="27" t="n">
-        <v>-535</v>
+        <v>-593</v>
       </c>
       <c r="E52" s="27" t="n">
-        <v>-555</v>
-      </c>
-      <c r="F52" s="28" t="n">
-        <v>20</v>
+        <v>-468</v>
+      </c>
+      <c r="F52" s="27" t="n">
+        <v>-125</v>
       </c>
       <c r="G52" s="28" t="n">
-        <v>537</v>
+        <v>588</v>
       </c>
       <c r="H52" s="29" t="n">
-        <v>146.9</v>
+        <v>222.6</v>
       </c>
       <c r="I52" s="29" t="n">
-        <v>12094.3</v>
+        <v>6895.6</v>
       </c>
       <c r="J52" s="29" t="n">
-        <v>0</v>
+        <v>-292.3</v>
       </c>
     </row>
     <row r="53">
@@ -2069,29 +2069,29 @@
       </c>
       <c r="C53" s="29" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D53" s="27" t="n">
-        <v>-530</v>
-      </c>
-      <c r="E53" s="28" t="n">
-        <v>108</v>
+        <v>-582</v>
+      </c>
+      <c r="E53" s="27" t="n">
+        <v>-195</v>
       </c>
       <c r="F53" s="27" t="n">
-        <v>-638</v>
+        <v>-386</v>
       </c>
       <c r="G53" s="28" t="n">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="H53" s="29" t="n">
-        <v>314.6</v>
+        <v>563.7</v>
       </c>
       <c r="I53" s="29" t="n">
-        <v>14493.4</v>
+        <v>9333.9</v>
       </c>
       <c r="J53" s="29" t="n">
-        <v>0</v>
+        <v>-1092.4</v>
       </c>
     </row>
     <row r="54">
@@ -2105,29 +2105,29 @@
       </c>
       <c r="C54" s="29" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D54" s="27" t="n">
-        <v>-503</v>
+        <v>-524</v>
       </c>
       <c r="E54" s="27" t="n">
-        <v>-385</v>
-      </c>
-      <c r="F54" s="27" t="n">
-        <v>-118</v>
+        <v>-559</v>
+      </c>
+      <c r="F54" s="28" t="n">
+        <v>35</v>
       </c>
       <c r="G54" s="28" t="n">
-        <v>494</v>
+        <v>528</v>
       </c>
       <c r="H54" s="29" t="n">
-        <v>222.6</v>
+        <v>146.9</v>
       </c>
       <c r="I54" s="29" t="n">
-        <v>7187.9</v>
+        <v>11659.9</v>
       </c>
       <c r="J54" s="29" t="n">
-        <v>0</v>
+        <v>-434.4</v>
       </c>
     </row>
     <row r="55">
@@ -2141,29 +2141,29 @@
       </c>
       <c r="C55" s="29" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D55" s="27" t="n">
-        <v>-465</v>
-      </c>
-      <c r="E55" s="27" t="n">
-        <v>-29</v>
+        <v>-511</v>
+      </c>
+      <c r="E55" s="28" t="n">
+        <v>132</v>
       </c>
       <c r="F55" s="27" t="n">
-        <v>-436</v>
+        <v>-643</v>
       </c>
       <c r="G55" s="28" t="n">
-        <v>497</v>
+        <v>559</v>
       </c>
       <c r="H55" s="29" t="n">
-        <v>37.7</v>
+        <v>314.6</v>
       </c>
       <c r="I55" s="29" t="n">
-        <v>3613.5</v>
+        <v>13946.5</v>
       </c>
       <c r="J55" s="29" t="n">
-        <v>0</v>
+        <v>-546.9</v>
       </c>
     </row>
     <row r="56"/>
@@ -2212,12 +2212,12 @@
       </c>
       <c r="B59" s="29" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>주간 순매수 43,839억 원으로 수급 집중도가 가장 높음.</t>
+          <t>주가 상승에도 대차잔고가 2,044.8억 감소하며 숏커버링 여지 확인됨.</t>
         </is>
       </c>
     </row>
@@ -2229,12 +2229,12 @@
       </c>
       <c r="B60" s="29" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>주간 순매수 28,819억 원으로 AI 메모리 모멘텀 지속.</t>
+          <t>기관 순매수 2,220억이 집중되었으며 원전 수주 기대감이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>주간 순매수 -1,900억 원으로 수급 이탈이 뚜렷함.</t>
+          <t>주간 순매도 -3,070억을 기록하며 수급 이탈이 관찰됨.</t>
         </is>
       </c>
     </row>
@@ -2263,12 +2263,12 @@
       </c>
       <c r="B62" s="29" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>주간 순매수 -1,526억 원으로 수급 약세 지속.</t>
+          <t>주가 급등에 따른 대차잔고 482.9억 증가로 하방 압력 관찰됨.</t>
         </is>
       </c>
     </row>
@@ -2308,28 +2308,28 @@
     <row r="66" ht="15" customHeight="1" s="15">
       <c r="A66" s="17" t="inlineStr">
         <is>
-          <t>- AI 반도체 중심의 강력한 외국인·기관 매수세가 유입되며 주초 시장 급등을 견인함.</t>
+          <t>- 주초 외국인과 기관의 강력한 동반 매수세로 KOSPI가 4.61% 급등하며 Risk-On 국면을 연출함.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="15">
       <c r="A67" s="17" t="inlineStr">
         <is>
-          <t>- 미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 상승이 시장 상단을 제한함.</t>
+          <t>- 미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장 상단을 제한함.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="15">
       <c r="A68" s="17" t="inlineStr">
         <is>
-          <t>- 국내 2분기 GDP 성장률(0.6%)이 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>- 주 후반 국내 2분기 GDP 성장률이 0.6%로 둔화하며 경기 우려가 부각됨.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>- 개인의 대규모 차익 실현 매도세가 지수 하락 압력으로 작용하며 변동성이 확대됨.</t>
+          <t>- 반도체 섹터는 미국 모멘텀을 이어받았으나, 금리 인상 우려와 밸류에이션 부담으로 지수 변동성이 확대됨.</t>
         </is>
       </c>
     </row>
@@ -2357,21 +2357,21 @@
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>- 전기·전자 및 기계·장비 섹터가 AI 반도체와 원전 모멘텀을 바탕으로 시장 상승을 주도함.</t>
+          <t>- 전기·전자 및 기계·장비 섹터가 반도체와 원전 모멘텀을 바탕으로 주간 상승률 상위를 기록함.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="15">
       <c r="A73" s="17" t="inlineStr">
         <is>
-          <t>- 건설 섹터는 대형 원전 건설 협의 기대감으로 주간 7.86% 상승하며 강세를 지속함.</t>
+          <t>- 건설 및 전기·가스 섹터는 대형 원전 수주 기대감으로 주 후반 강세를 보임.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="15">
       <c r="A74" s="17" t="inlineStr">
         <is>
-          <t>- 음식료·담배 및 IT 서비스 섹터는 차익 실현 매물 출회로 약세 전환함.</t>
+          <t>- IT 서비스 및 음식료·담배 섹터는 차익 실현 매물과 경기 둔화 우려로 약세를 보임.</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="31" customHeight="1" s="15">
+    <row r="77" ht="15" customHeight="1" s="15">
       <c r="A77" s="29" t="inlineStr">
         <is>
           <t>2026-09-07</t>
@@ -2416,7 +2416,7 @@
       <c r="E77" s="28" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
+          <t>외국인·기관 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       <c r="E86" s="28" t="inlineStr"/>
       <c r="F86" s="17" t="inlineStr">
         <is>
-          <t>2분기 GDP 성장률 0.6% 발표 및 경기 둔화 우려 부각으로 KOSPI 0.58% 하락.</t>
+          <t>국내 2분기 GDP 성장률 0.6% 발표 및 금리 인상 우려로 KOSPI 0.58% 하락</t>
         </is>
       </c>
     </row>
@@ -2901,19 +2901,19 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>미국 PPI 및 CPI 발표 결과에 따라 금리 인상 우려가 완화되면 반도체 중심의 상승세가 재개될 것.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="15" customHeight="1" s="15">
-      <c r="A97" s="10" t="inlineStr">
-        <is>
-          <t>하방 시나리오</t>
+          <t>미국 PPI 및 CPI 발표 결과에 따라 금리 인상 우려가 완화되면 반도체 중심의 상승세가 재개될 것임.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="31" customHeight="1" s="15">
+      <c r="A97" s="8" t="inlineStr">
+        <is>
+          <t>상승 시나리오</t>
         </is>
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>물가 지표가 예상치를 상회하여 국채 금리가 추가 상승하면 경기 둔화 우려가 부각되며 지수 조정이 심화될 것.</t>
+          <t>물가 지표가 예상치를 상회하여 금리 인상 압력이 지속될 경우, 경기 방어주 및 원전 관련주로의 수급 로테이션이 강화될 것임.</t>
         </is>
       </c>
     </row>
@@ -2925,11 +2925,11 @@
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>판별 신호: 9월 11일 발표되는 미국 소비자물가지수(CPI)의 전월 대비 증감률.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="31" customHeight="1" s="15">
+          <t>판별 신호: 미국 생산자물가지수(PPI) 및 소비자물가지수(CPI)의 전월 대비 등락폭.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="15" customHeight="1" s="15">
       <c r="A99" s="3" t="inlineStr">
         <is>
           <t>핵심 이벤트</t>
@@ -2937,7 +2937,7 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>핵심 이벤트: 9월 10일 미국 생산자물가지수(PPI), 9월 11일 미국 소비자물가지수(CPI), 9월 15일 국내 무역수지.</t>
+          <t>핵심 이벤트: 9월 10일 미국 PPI, 9월 11일 미국 CPI, 9월 15일 국내 무역수지.</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 19:46 KST</t>
+          <t>2026-09-08 20:57 KST</t>
         </is>
       </c>
     </row>
@@ -3042,7 +3042,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AI 반도체 주도 랠리와 경기 둔화 우려의 교차</t>
+          <t>반도체 주도 랠리와 금리 인상 우려 사이의 변동성 장세</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수의 3.37% 급등이 국내 반도체 소부장 및 대형주로 이어지며, 미국 지수 약세에도 불구하고 외국인과 기관의 강력한 매수세를 유도함.</t>
+          <t>필라델피아 반도체 지수의 3.37% 급등과 마이크론 상승세가 국내 반도체 소부장 및 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도함.</t>
         </is>
       </c>
     </row>
@@ -3281,7 +3281,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>미국 국채 금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담을 가중시켰고, 국내 GDP 성장률 둔화와 맞물려 지수 하락을 견인함.</t>
+          <t>미국 국채금리 급등과 UBS의 금리 인상 전망 제기로 인한 투자 심리 위축이 국내 증시의 밸류에이션 부담을 가중시키며 지수 하락을 유발함.</t>
         </is>
       </c>
     </row>
@@ -3301,7 +3301,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>매크로 환경: 미국 비농업 고용지수(162K)가 예상치(55K)를 상회하며 금리 인하 경로 불확실성이 커졌고, 국내 2분기 GDP 성장률(0.6%)은 이전치(1.8%)를 하회하며 경기 둔화 신호가 뚜렷함.</t>
+          <t>미국 비농업 고용지표(162K)가 예상치를 상회하고 국내 2분기 GDP(0.6%)가 이전치(1.8%)를 하회하며 매크로 환경의 불확실성이 커짐.</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3313,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되었으나, 개인은 전 섹터에서 매도 우위를 보이며 차익 실현에 집중함.</t>
+          <t>수급 측면에서는 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되었으나, 개인은 전반적인 차익 실현 매도를 지속함.</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>종합 관점: AI 반도체 모멘텀이 시장을 견인했으나, 매크로 불확실성과 경기 둔화 우려가 상존하며 수급 쏠림 현상이 심화된 한 주였음.</t>
+          <t>반도체 중심의 수급 쏠림이 뚜렷한 가운데, 금리 인상 우려와 경기 둔화 신호가 맞물리며 지수 상단이 제한되는 흐름을 보임.</t>
         </is>
       </c>
     </row>
@@ -3351,25 +3351,25 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>43839</v>
+        <v>45121</v>
       </c>
       <c r="E31" t="n">
-        <v>20501</v>
+        <v>21100</v>
       </c>
       <c r="F31" t="n">
-        <v>23338</v>
+        <v>24020</v>
       </c>
       <c r="G31" t="n">
-        <v>-53897</v>
+        <v>-55192</v>
       </c>
       <c r="H31" t="n">
         <v>1816.7</v>
       </c>
       <c r="I31" t="n">
-        <v>247447.2</v>
+        <v>240284.8</v>
       </c>
       <c r="J31" t="n">
-        <v>0</v>
+        <v>-7162.4</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="15">
@@ -3387,25 +3387,25 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>28819</v>
+        <v>29092</v>
       </c>
       <c r="E32" t="n">
-        <v>19070</v>
+        <v>19197</v>
       </c>
       <c r="F32" t="n">
-        <v>9749</v>
+        <v>9895</v>
       </c>
       <c r="G32" t="n">
-        <v>-51831</v>
+        <v>-52130</v>
       </c>
       <c r="H32" t="n">
         <v>3364.2</v>
       </c>
       <c r="I32" t="n">
-        <v>225804.3</v>
+        <v>223759.5</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>-2044.8</v>
       </c>
     </row>
     <row r="33">
@@ -3423,25 +3423,25 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>5236</v>
+        <v>5294</v>
       </c>
       <c r="E33" t="n">
-        <v>3060</v>
+        <v>3070</v>
       </c>
       <c r="F33" t="n">
-        <v>2175</v>
+        <v>2223</v>
       </c>
       <c r="G33" t="n">
-        <v>-5105</v>
+        <v>-5184</v>
       </c>
       <c r="H33" t="n">
         <v>365.7</v>
       </c>
       <c r="I33" t="n">
-        <v>32812</v>
+        <v>32891.8</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>79.8</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="15">
@@ -3474,10 +3474,10 @@
         <v>206.2</v>
       </c>
       <c r="I34" t="n">
-        <v>29143.8</v>
+        <v>28477.7</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>-666.1</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="15">
@@ -3495,25 +3495,25 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>2266</v>
+        <v>2138</v>
       </c>
       <c r="E35" t="n">
-        <v>58</v>
+        <v>-81</v>
       </c>
       <c r="F35" t="n">
-        <v>2208</v>
+        <v>2220</v>
       </c>
       <c r="G35" t="n">
-        <v>-2304</v>
+        <v>-2125</v>
       </c>
       <c r="H35" t="n">
         <v>900.5</v>
       </c>
       <c r="I35" t="n">
-        <v>19475.5</v>
+        <v>19469.6</v>
       </c>
       <c r="J35" t="n">
-        <v>0</v>
+        <v>-5.9</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="15">
@@ -3531,25 +3531,25 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>1369</v>
+        <v>1581</v>
       </c>
       <c r="E36" t="n">
-        <v>816</v>
+        <v>1000</v>
       </c>
       <c r="F36" t="n">
-        <v>553</v>
+        <v>581</v>
       </c>
       <c r="G36" t="n">
-        <v>-1351</v>
+        <v>-1560</v>
       </c>
       <c r="H36" t="n">
         <v>485.3</v>
       </c>
       <c r="I36" t="n">
-        <v>44346.7</v>
+        <v>43511.4</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>-835.3</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1" s="15">
@@ -3567,25 +3567,25 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1309</v>
+        <v>1182</v>
       </c>
       <c r="E37" t="n">
-        <v>765</v>
+        <v>640</v>
       </c>
       <c r="F37" t="n">
-        <v>543</v>
+        <v>541</v>
       </c>
       <c r="G37" t="n">
-        <v>-1290</v>
+        <v>-1175</v>
       </c>
       <c r="H37" t="n">
         <v>422.1</v>
       </c>
       <c r="I37" t="n">
-        <v>10675.8</v>
+        <v>10178.7</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>-497.1</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1" s="15">
@@ -3603,25 +3603,25 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>867</v>
+        <v>852</v>
       </c>
       <c r="E38" t="n">
-        <v>702</v>
+        <v>687</v>
       </c>
       <c r="F38" t="n">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="G38" t="n">
-        <v>-880</v>
+        <v>-863</v>
       </c>
       <c r="H38" t="n">
         <v>144</v>
       </c>
       <c r="I38" t="n">
-        <v>6126.4</v>
+        <v>5502.2</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>-624.2</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="15">
@@ -3654,10 +3654,10 @@
         <v>164.4</v>
       </c>
       <c r="I39" t="n">
-        <v>5739.7</v>
+        <v>6222.6</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>482.9</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="15">
@@ -3675,25 +3675,25 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>720</v>
+        <v>754</v>
       </c>
       <c r="E40" t="n">
-        <v>-287</v>
+        <v>-258</v>
       </c>
       <c r="F40" t="n">
-        <v>1007</v>
+        <v>1011</v>
       </c>
       <c r="G40" t="n">
-        <v>-724</v>
+        <v>-760</v>
       </c>
       <c r="H40" t="n">
         <v>292.4</v>
       </c>
       <c r="I40" t="n">
-        <v>8468.6</v>
+        <v>8765.6</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>297</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="15">
@@ -3711,25 +3711,25 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>-1900</v>
+        <v>-3070</v>
       </c>
       <c r="E41" t="n">
-        <v>-1420</v>
+        <v>-2520</v>
       </c>
       <c r="F41" t="n">
-        <v>-480</v>
+        <v>-550</v>
       </c>
       <c r="G41" t="n">
-        <v>1869</v>
+        <v>3076</v>
       </c>
       <c r="H41" t="n">
         <v>686.4</v>
       </c>
       <c r="I41" t="n">
-        <v>38810</v>
+        <v>36009</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>-2801</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="15">
@@ -3747,25 +3747,25 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-1526</v>
+        <v>-1568</v>
       </c>
       <c r="E42" t="n">
-        <v>-657</v>
+        <v>-695</v>
       </c>
       <c r="F42" t="n">
-        <v>-870</v>
+        <v>-873</v>
       </c>
       <c r="G42" t="n">
-        <v>1555</v>
+        <v>1591</v>
       </c>
       <c r="H42" t="n">
         <v>284</v>
       </c>
       <c r="I42" t="n">
-        <v>13527.9</v>
+        <v>13231</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>-296.9</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
@@ -3783,25 +3783,25 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>-944</v>
+        <v>-968</v>
       </c>
       <c r="E43" t="n">
-        <v>-113</v>
+        <v>-135</v>
       </c>
       <c r="F43" t="n">
-        <v>-831</v>
+        <v>-833</v>
       </c>
       <c r="G43" t="n">
-        <v>942</v>
+        <v>966</v>
       </c>
       <c r="H43" t="n">
         <v>96.5</v>
       </c>
       <c r="I43" t="n">
-        <v>8359.200000000001</v>
+        <v>8138.3</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>-220.9</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="15">
@@ -3819,25 +3819,25 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>-751</v>
+        <v>-783</v>
       </c>
       <c r="E44" t="n">
-        <v>-528</v>
+        <v>-551</v>
       </c>
       <c r="F44" t="n">
-        <v>-223</v>
+        <v>-232</v>
       </c>
       <c r="G44" t="n">
-        <v>564</v>
+        <v>626</v>
       </c>
       <c r="H44" t="n">
         <v>125.5</v>
       </c>
       <c r="I44" t="n">
-        <v>12830.3</v>
+        <v>12546.7</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>-283.6</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="15">
@@ -3851,29 +3851,29 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>-588</v>
+        <v>-679</v>
       </c>
       <c r="E45" t="n">
-        <v>-3</v>
+        <v>-292</v>
       </c>
       <c r="F45" t="n">
-        <v>-585</v>
+        <v>-386</v>
       </c>
       <c r="G45" t="n">
-        <v>590</v>
+        <v>764</v>
       </c>
       <c r="H45" t="n">
-        <v>133.3</v>
+        <v>419.2</v>
       </c>
       <c r="I45" t="n">
-        <v>14894.9</v>
+        <v>31440</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>-1186.9</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
@@ -3887,29 +3887,29 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>-572</v>
+        <v>-629</v>
       </c>
       <c r="E46" t="n">
-        <v>-204</v>
+        <v>-46</v>
       </c>
       <c r="F46" t="n">
-        <v>-368</v>
+        <v>-583</v>
       </c>
       <c r="G46" t="n">
-        <v>658</v>
+        <v>634</v>
       </c>
       <c r="H46" t="n">
-        <v>419.2</v>
+        <v>133.3</v>
       </c>
       <c r="I46" t="n">
-        <v>32626.9</v>
+        <v>14504.2</v>
       </c>
       <c r="J46" t="n">
-        <v>0</v>
+        <v>-390.7</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">
@@ -3923,29 +3923,29 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-535</v>
+        <v>-593</v>
       </c>
       <c r="E47" t="n">
-        <v>-555</v>
+        <v>-468</v>
       </c>
       <c r="F47" t="n">
-        <v>20</v>
+        <v>-125</v>
       </c>
       <c r="G47" t="n">
-        <v>537</v>
+        <v>588</v>
       </c>
       <c r="H47" t="n">
-        <v>146.9</v>
+        <v>222.6</v>
       </c>
       <c r="I47" t="n">
-        <v>12094.3</v>
+        <v>6895.6</v>
       </c>
       <c r="J47" t="n">
-        <v>0</v>
+        <v>-292.3</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="15">
@@ -3959,29 +3959,29 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-530</v>
+        <v>-582</v>
       </c>
       <c r="E48" t="n">
-        <v>108</v>
+        <v>-195</v>
       </c>
       <c r="F48" t="n">
-        <v>-638</v>
+        <v>-386</v>
       </c>
       <c r="G48" t="n">
-        <v>575</v>
+        <v>571</v>
       </c>
       <c r="H48" t="n">
-        <v>314.6</v>
+        <v>563.7</v>
       </c>
       <c r="I48" t="n">
-        <v>14493.4</v>
+        <v>9333.9</v>
       </c>
       <c r="J48" t="n">
-        <v>0</v>
+        <v>-1092.4</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="15">
@@ -3995,29 +3995,29 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-503</v>
+        <v>-524</v>
       </c>
       <c r="E49" t="n">
-        <v>-385</v>
+        <v>-559</v>
       </c>
       <c r="F49" t="n">
-        <v>-118</v>
+        <v>35</v>
       </c>
       <c r="G49" t="n">
-        <v>494</v>
+        <v>528</v>
       </c>
       <c r="H49" t="n">
-        <v>222.6</v>
+        <v>146.9</v>
       </c>
       <c r="I49" t="n">
-        <v>7187.9</v>
+        <v>11659.9</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>-434.4</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="15">
@@ -4031,29 +4031,29 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>-465</v>
+        <v>-511</v>
       </c>
       <c r="E50" t="n">
-        <v>-29</v>
+        <v>132</v>
       </c>
       <c r="F50" t="n">
-        <v>-436</v>
+        <v>-643</v>
       </c>
       <c r="G50" t="n">
-        <v>497</v>
+        <v>559</v>
       </c>
       <c r="H50" t="n">
-        <v>37.7</v>
+        <v>314.6</v>
       </c>
       <c r="I50" t="n">
-        <v>3613.5</v>
+        <v>13946.5</v>
       </c>
       <c r="J50" t="n">
-        <v>0</v>
+        <v>-546.9</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="15">
@@ -4071,12 +4071,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>주간 순매수 43,839억 원으로 수급 집중도가 가장 높음.</t>
+          <t>주가 상승에도 대차잔고가 2,044.8억 감소하며 숏커버링 여지 확인됨.</t>
         </is>
       </c>
     </row>
@@ -4088,12 +4088,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>주간 순매수 28,819억 원으로 AI 메모리 모멘텀 지속.</t>
+          <t>기관 순매수 2,220억이 집중되었으며 원전 수주 기대감이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>주간 순매수 -1,900억 원으로 수급 이탈이 뚜렷함.</t>
+          <t>주간 순매도 -3,070억을 기록하며 수급 이탈이 관찰됨.</t>
         </is>
       </c>
     </row>
@@ -4122,12 +4122,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>주간 순매수 -1,526억 원으로 수급 약세 지속.</t>
+          <t>주가 급등에 따른 대차잔고 482.9억 증가로 하방 압력 관찰됨.</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4146,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AI 반도체 중심의 강력한 외국인·기관 매수세가 유입되며 주초 시장 급등을 견인함.</t>
+          <t>주초 외국인과 기관의 강력한 동반 매수세로 KOSPI가 4.61% 급등하며 Risk-On 국면을 연출함.</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 상승이 시장 상단을 제한함.</t>
+          <t>미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장 상단을 제한함.</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>국내 2분기 GDP 성장률(0.6%)이 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>주 후반 국내 2분기 GDP 성장률이 0.6%로 둔화하며 경기 우려가 부각됨.</t>
         </is>
       </c>
     </row>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>개인의 대규모 차익 실현 매도세가 지수 하락 압력으로 작용하며 변동성이 확대됨.</t>
+          <t>반도체 섹터는 미국 모멘텀을 이어받았으나, 금리 인상 우려와 밸류에이션 부담으로 지수 변동성이 확대됨.</t>
         </is>
       </c>
     </row>
@@ -4201,7 +4201,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>전기·전자 및 기계·장비 섹터가 AI 반도체와 원전 모멘텀을 바탕으로 시장 상승을 주도함.</t>
+          <t>전기·전자 및 기계·장비 섹터가 반도체와 원전 모멘텀을 바탕으로 주간 상승률 상위를 기록함.</t>
         </is>
       </c>
     </row>
@@ -4213,7 +4213,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>건설 섹터는 대형 원전 건설 협의 기대감으로 주간 7.86% 상승하며 강세를 지속함.</t>
+          <t>건설 및 전기·가스 섹터는 대형 원전 수주 기대감으로 주 후반 강세를 보임.</t>
         </is>
       </c>
     </row>
@@ -4225,7 +4225,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>음식료·담배 및 IT 서비스 섹터는 차익 실현 매물 출회로 약세 전환함.</t>
+          <t>IT 서비스 및 음식료·담배 섹터는 차익 실현 매물과 경기 둔화 우려로 약세를 보임.</t>
         </is>
       </c>
     </row>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
+          <t>외국인·기관 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4490,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>2분기 GDP 성장률 0.6% 발표 및 경기 둔화 우려 부각으로 KOSPI 0.58% 하락.</t>
+          <t>국내 2분기 GDP 성장률 0.6% 발표 및 금리 인상 우려로 KOSPI 0.58% 하락</t>
         </is>
       </c>
     </row>
@@ -4677,19 +4677,19 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>미국 PPI 및 CPI 발표 결과에 따라 금리 인상 우려가 완화되면 반도체 중심의 상승세가 재개될 것.</t>
+          <t>미국 PPI 및 CPI 발표 결과에 따라 금리 인상 우려가 완화되면 반도체 중심의 상승세가 재개될 것임.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="15">
       <c r="A84" t="inlineStr">
         <is>
-          <t>하방 시나리오</t>
+          <t>상승 시나리오</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>물가 지표가 예상치를 상회하여 국채 금리가 추가 상승하면 경기 둔화 우려가 부각되며 지수 조정이 심화될 것.</t>
+          <t>물가 지표가 예상치를 상회하여 금리 인상 압력이 지속될 경우, 경기 방어주 및 원전 관련주로의 수급 로테이션이 강화될 것임.</t>
         </is>
       </c>
     </row>
@@ -4701,7 +4701,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>판별 신호: 9월 11일 발표되는 미국 소비자물가지수(CPI)의 전월 대비 증감률.</t>
+          <t>판별 신호: 미국 생산자물가지수(PPI) 및 소비자물가지수(CPI)의 전월 대비 등락폭.</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4713,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>핵심 이벤트: 9월 10일 미국 생산자물가지수(PPI), 9월 11일 미국 소비자물가지수(CPI), 9월 15일 국내 무역수지.</t>
+          <t>핵심 이벤트: 9월 10일 미국 PPI, 9월 11일 미국 CPI, 9월 15일 국내 무역수지.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-09-08 12:22Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -747,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12.9" customWidth="1" style="15" min="1" max="1"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-08 20:57 KST</t>
+          <t>2026-09-08 21:22 KST</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>반도체 주도 랠리와 금리 인상 우려 사이의 변동성 장세</t>
+          <t>반도체 주도 급등 후 매크로 경계감에 따른 숨 고르기</t>
         </is>
       </c>
     </row>
@@ -1303,11 +1303,11 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수의 3.37% 급등과 마이크론 상승세가 국내 반도체 소부장 및 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1" s="15">
+          <t>미국 필라델피아 반도체 지수의 3.37% 급등이 국내 반도체 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도해 지수 급등을 견인함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44.5" customHeight="1" s="15">
       <c r="A26" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 UBS의 금리 인상 전망 제기로 인한 투자 심리 위축이 국내 증시의 밸류에이션 부담을 가중시키며 지수 하락을 유발함.</t>
+          <t>미국 국채금리 급등과 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, GDP 성장률 둔화까지 겹쳐 지수 하락을 유발함.</t>
         </is>
       </c>
     </row>
@@ -1376,21 +1376,21 @@
     <row r="30" ht="31" customHeight="1" s="15">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>- 미국 비농업 고용지표(162K)가 예상치를 상회하고 국내 2분기 GDP(0.6%)가 이전치(1.8%)를 하회하며 매크로 환경의 불확실성이 커짐.</t>
+          <t>- 매크로 환경: 미국 비농업고용지수(162K)가 예상치(55K)를 상회하며 금리 인하 기대가 후퇴했고, 국내 2분기 GDP 성장률(0.6%)이 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31" customHeight="1" s="15">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>- 수급 측면에서는 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되었으나, 개인은 전반적인 차익 실현 매도를 지속함.</t>
+          <t>- 수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되며 주가를 견인했으나, 개인은 전기·전자에서 91,202억을 순매도하며 차익 실현에 집중함.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="31" customHeight="1" s="15">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>- 반도체 중심의 수급 쏠림이 뚜렷한 가운데, 금리 인상 우려와 경기 둔화 신호가 맞물리며 지수 상단이 제한되는 흐름을 보임.</t>
+          <t>- 종합 관점: 반도체 중심의 수급 쏠림이 뚜렷했으나, 매크로 불확실성과 경기 둔화 신호가 지수 상단을 제한하는 국면으로 전환됨.</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>주가 상승에도 대차잔고가 2,044.8억 감소하며 숏커버링 여지 확인됨.</t>
+          <t>주가 상승세에도 대차잔고가 2,044.8억 감소하여 숏커버링 여지가 존재함.</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>기관 순매수 2,220억이 집중되었으며 원전 수주 기대감이 지속됨.</t>
+          <t>기관 순매수(2,220억)가 집중되며 원전 모멘텀이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>주간 순매도 -3,070억을 기록하며 수급 이탈이 관찰됨.</t>
+          <t>주가 하락세 속에서 외국인(-2,520억)과 기관(-550억)의 동반 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -2288,12 +2288,12 @@
       </c>
       <c r="B62" s="30" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>주가 급등에 따른 대차잔고 482.9억 증가로 하방 압력 관찰됨.</t>
+          <t>주가 하락세 속에서 기관(-833억)의 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -2330,31 +2330,31 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="15" customHeight="1" s="15">
+    <row r="66" ht="31" customHeight="1" s="15">
       <c r="A66" s="17" t="inlineStr">
         <is>
-          <t>- 주초 외국인과 기관의 강력한 동반 매수세로 KOSPI가 4.61% 급등하며 Risk-On 국면을 연출함.</t>
+          <t>- KOSPI는 외국인과 기관의 강력한 반도체 매수세에 힘입어 6995.39까지 급등했으나, 이후 매크로 경계감으로 6954.52로 조정됨.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="15">
       <c r="A67" s="17" t="inlineStr">
         <is>
-          <t>- 미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장 상단을 제한함.</t>
+          <t>- 미국 비농업고용지표 호조에 따른 금리 인하 기대 후퇴가 시장의 상승 동력을 제한함.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="15">
       <c r="A68" s="17" t="inlineStr">
         <is>
-          <t>- 주 후반 국내 2분기 GDP 성장률이 0.6%로 둔화하며 경기 우려가 부각됨.</t>
+          <t>- 국내 2분기 GDP 성장률이 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>- 반도체 섹터는 미국 모멘텀을 이어받았으나, 금리 인상 우려와 밸류에이션 부담으로 지수 변동성이 확대됨.</t>
+          <t>- 개인은 전기·전자 섹터에서 91,202억을 순매도하며 대규모 차익 실현에 집중함.</t>
         </is>
       </c>
     </row>
@@ -2382,21 +2382,21 @@
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>- 전기·전자 및 기계·장비 섹터가 반도체와 원전 모멘텀을 바탕으로 주간 상승률 상위를 기록함.</t>
+          <t>- 전기·전자 섹터는 외국인과 기관의 수급 집중으로 강세 지속.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="15">
       <c r="A73" s="17" t="inlineStr">
         <is>
-          <t>- 건설 및 전기·가스 섹터는 대형 원전 수주 기대감으로 주 후반 강세를 보임.</t>
+          <t>- 원전 및 건설 관련주(기계·장비, 전기·가스)는 대형 수주 기대감으로 순환매 흐름.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="15">
       <c r="A74" s="17" t="inlineStr">
         <is>
-          <t>- IT 서비스 및 음식료·담배 섹터는 차익 실현 매물과 경기 둔화 우려로 약세를 보임.</t>
+          <t>- 음식료 및 IT 서비스 섹터는 실적 우려와 차익 실현 매물로 약세 전환.</t>
         </is>
       </c>
     </row>
@@ -2425,7 +2425,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="15" customHeight="1" s="15">
+    <row r="77" ht="31" customHeight="1" s="15">
       <c r="A77" s="30" t="inlineStr">
         <is>
           <t>2026-09-07</t>
@@ -2441,7 +2441,7 @@
       <c r="E77" s="29" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>외국인·기관 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
+          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       <c r="E86" s="29" t="inlineStr"/>
       <c r="F86" s="17" t="inlineStr">
         <is>
-          <t>국내 2분기 GDP 성장률 0.6% 발표 및 금리 인상 우려로 KOSPI 0.58% 하락</t>
+          <t>국내 2분기 GDP 성장률 0.6% 발표 및 국채금리 상승 여파로 KOSPI 0.58% 하락.</t>
         </is>
       </c>
     </row>
@@ -2926,43 +2926,43 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>미국 PPI 및 CPI 발표 결과에 따라 금리 인상 우려가 완화되면 반도체 중심의 상승세가 재개될 것임.</t>
+          <t>미국 물가 지표가 예상치에 부합하거나 하회하면 반도체 중심의 기술주 반등세 재개</t>
         </is>
       </c>
     </row>
     <row r="97" ht="31" customHeight="1" s="15">
-      <c r="A97" s="31" t="inlineStr">
-        <is>
-          <t>상승 시나리오</t>
+      <c r="A97" s="32" t="inlineStr">
+        <is>
+          <t>하방 시나리오</t>
         </is>
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>물가 지표가 예상치를 상회하여 금리 인상 압력이 지속될 경우, 경기 방어주 및 원전 관련주로의 수급 로테이션이 강화될 것임.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="31" customHeight="1" s="15">
-      <c r="A98" s="32" t="inlineStr">
-        <is>
-          <t>하방 시나리오</t>
+          <t>물가 지표가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 연장</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15" customHeight="1" s="15">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>9월 10일 발표될 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="15">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>판별 신호</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>판별 신호: 미국 생산자물가지수(PPI) 및 소비자물가지수(CPI)의 전월 대비 등락폭.</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -2974,12 +2974,24 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>핵심 이벤트: 9월 10일 미국 PPI, 9월 11일 미국 CPI, 9월 15일 국내 무역수지.</t>
+          <t>미국 소비자물가지수(CPI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="15">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>핵심 이벤트</t>
+        </is>
+      </c>
+      <c r="B101" s="17" t="inlineStr">
+        <is>
+          <t>국내 무역수지</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="48">
     <mergeCell ref="A32:J32"/>
     <mergeCell ref="F78:J78"/>
     <mergeCell ref="B98:J98"/>
@@ -2987,6 +2999,7 @@
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="F87:J87"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="B101:J101"/>
     <mergeCell ref="C62:J62"/>
     <mergeCell ref="C58:J58"/>
     <mergeCell ref="G25:J25"/>
@@ -3038,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" outlineLevelCol="0"/>
   <cols>
     <col width="30.85546875" customWidth="1" style="15" min="1" max="1"/>
@@ -3070,7 +3083,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 20:57 KST</t>
+          <t>2026-09-08 21:22 KST</t>
         </is>
       </c>
     </row>
@@ -3082,7 +3095,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>반도체 주도 랠리와 금리 인상 우려 사이의 변동성 장세</t>
+          <t>반도체 주도 급등 후 매크로 경계감에 따른 숨 고르기</t>
         </is>
       </c>
     </row>
@@ -3306,7 +3319,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>필라델피아 반도체 지수의 3.37% 급등과 마이크론 상승세가 국내 반도체 소부장 및 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도함.</t>
+          <t>미국 필라델피아 반도체 지수의 3.37% 급등이 국내 반도체 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도해 지수 급등을 견인함.</t>
         </is>
       </c>
     </row>
@@ -3321,7 +3334,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 UBS의 금리 인상 전망 제기로 인한 투자 심리 위축이 국내 증시의 밸류에이션 부담을 가중시키며 지수 하락을 유발함.</t>
+          <t>미국 국채금리 급등과 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, GDP 성장률 둔화까지 겹쳐 지수 하락을 유발함.</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3354,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미국 비농업 고용지표(162K)가 예상치를 상회하고 국내 2분기 GDP(0.6%)가 이전치(1.8%)를 하회하며 매크로 환경의 불확실성이 커짐.</t>
+          <t>매크로 환경: 미국 비농업고용지수(162K)가 예상치(55K)를 상회하며 금리 인하 기대가 후퇴했고, 국내 2분기 GDP 성장률(0.6%)이 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
         </is>
       </c>
     </row>
@@ -3353,7 +3366,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>수급 측면에서는 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되었으나, 개인은 전반적인 차익 실현 매도를 지속함.</t>
+          <t>수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되며 주가를 견인했으나, 개인은 전기·전자에서 91,202억을 순매도하며 차익 실현에 집중함.</t>
         </is>
       </c>
     </row>
@@ -3365,7 +3378,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>반도체 중심의 수급 쏠림이 뚜렷한 가운데, 금리 인상 우려와 경기 둔화 신호가 맞물리며 지수 상단이 제한되는 흐름을 보임.</t>
+          <t>종합 관점: 반도체 중심의 수급 쏠림이 뚜렷했으나, 매크로 불확실성과 경기 둔화 신호가 지수 상단을 제한하는 국면으로 전환됨.</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4129,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>주가 상승에도 대차잔고가 2,044.8억 감소하며 숏커버링 여지 확인됨.</t>
+          <t>주가 상승세에도 대차잔고가 2,044.8억 감소하여 숏커버링 여지가 존재함.</t>
         </is>
       </c>
     </row>
@@ -4133,7 +4146,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>기관 순매수 2,220억이 집중되었으며 원전 수주 기대감이 지속됨.</t>
+          <t>기관 순매수(2,220억)가 집중되며 원전 모멘텀이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -4150,7 +4163,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>주간 순매도 -3,070억을 기록하며 수급 이탈이 관찰됨.</t>
+          <t>주가 하락세 속에서 외국인(-2,520억)과 기관(-550억)의 동반 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -4162,12 +4175,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>주가 급등에 따른 대차잔고 482.9억 증가로 하방 압력 관찰됨.</t>
+          <t>주가 하락세 속에서 기관(-833억)의 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -4186,7 +4199,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>주초 외국인과 기관의 강력한 동반 매수세로 KOSPI가 4.61% 급등하며 Risk-On 국면을 연출함.</t>
+          <t>KOSPI는 외국인과 기관의 강력한 반도체 매수세에 힘입어 6995.39까지 급등했으나, 이후 매크로 경계감으로 6954.52로 조정됨.</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4211,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장 상단을 제한함.</t>
+          <t>미국 비농업고용지표 호조에 따른 금리 인하 기대 후퇴가 시장의 상승 동력을 제한함.</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4223,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>주 후반 국내 2분기 GDP 성장률이 0.6%로 둔화하며 경기 우려가 부각됨.</t>
+          <t>국내 2분기 GDP 성장률이 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4235,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>반도체 섹터는 미국 모멘텀을 이어받았으나, 금리 인상 우려와 밸류에이션 부담으로 지수 변동성이 확대됨.</t>
+          <t>개인은 전기·전자 섹터에서 91,202억을 순매도하며 대규모 차익 실현에 집중함.</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4254,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>전기·전자 및 기계·장비 섹터가 반도체와 원전 모멘텀을 바탕으로 주간 상승률 상위를 기록함.</t>
+          <t>전기·전자 섹터는 외국인과 기관의 수급 집중으로 강세 지속.</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4266,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>건설 및 전기·가스 섹터는 대형 원전 수주 기대감으로 주 후반 강세를 보임.</t>
+          <t>원전 및 건설 관련주(기계·장비, 전기·가스)는 대형 수주 기대감으로 순환매 흐름.</t>
         </is>
       </c>
     </row>
@@ -4265,7 +4278,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>IT 서비스 및 음식료·담배 섹터는 차익 실현 매물과 경기 둔화 우려로 약세를 보임.</t>
+          <t>음식료 및 IT 서비스 섹터는 실적 우려와 차익 실현 매물로 약세 전환.</t>
         </is>
       </c>
     </row>
@@ -4289,7 +4302,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>외국인·기관 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
+          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4543,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>국내 2분기 GDP 성장률 0.6% 발표 및 금리 인상 우려로 KOSPI 0.58% 하락</t>
+          <t>국내 2분기 GDP 성장률 0.6% 발표 및 국채금리 상승 여파로 KOSPI 0.58% 하락.</t>
         </is>
       </c>
     </row>
@@ -4717,43 +4730,43 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>미국 PPI 및 CPI 발표 결과에 따라 금리 인상 우려가 완화되면 반도체 중심의 상승세가 재개될 것임.</t>
+          <t>미국 물가 지표가 예상치에 부합하거나 하회하면 반도체 중심의 기술주 반등세 재개</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="15">
       <c r="A84" t="inlineStr">
         <is>
-          <t>상승 시나리오</t>
+          <t>하방 시나리오</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>물가 지표가 예상치를 상회하여 금리 인상 압력이 지속될 경우, 경기 방어주 및 원전 관련주로의 수급 로테이션이 강화될 것임.</t>
+          <t>물가 지표가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 연장</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="15">
       <c r="A85" t="inlineStr">
         <is>
-          <t>하방 시나리오</t>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
+          <t>9월 10일 발표될 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="15">
       <c r="A86" t="inlineStr">
         <is>
-          <t>판별 신호</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>판별 신호: 미국 생산자물가지수(PPI) 및 소비자물가지수(CPI)의 전월 대비 등락폭.</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -4765,11 +4778,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>핵심 이벤트: 9월 10일 미국 PPI, 9월 11일 미국 CPI, 9월 15일 국내 무역수지.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15" customHeight="1" s="15"/>
+          <t>미국 소비자물가지수(CPI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1" s="15">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>핵심 이벤트</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>국내 무역수지</t>
+        </is>
+      </c>
+    </row>
     <row r="89" ht="15" customHeight="1" s="15"/>
     <row r="90" ht="15" customHeight="1" s="15"/>
     <row r="91" ht="15" customHeight="1" s="15"/>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-09-08 12:31Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -747,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J101"/>
+  <dimension ref="A1:J100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12.9" customWidth="1" style="15" min="1" max="1"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-08 21:22 KST</t>
+          <t>2026-09-08 21:31 KST</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>반도체 주도 급등 후 매크로 경계감에 따른 숨 고르기</t>
+          <t>반도체 주도 랠리와 매크로 불확실성 사이의 줄타기</t>
         </is>
       </c>
     </row>
@@ -1303,11 +1303,11 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>미국 필라델피아 반도체 지수의 3.37% 급등이 국내 반도체 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도해 지수 급등을 견인함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="44.5" customHeight="1" s="15">
+          <t>미국 반도체 지수 급등과 마이크론 강세가 국내 반도체 대형주로 이어지며 외국인·기관의 대규모 매수세와 함께 KOSPI 4.61% 급등을 견인함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1" s="15">
       <c r="A26" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, GDP 성장률 둔화까지 겹쳐 지수 하락을 유발함.</t>
+          <t>미국 국채 금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 둔화까지 겹쳐 지수가 0.58% 하락함.</t>
         </is>
       </c>
     </row>
@@ -1376,21 +1376,21 @@
     <row r="30" ht="31" customHeight="1" s="15">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>- 매크로 환경: 미국 비농업고용지수(162K)가 예상치(55K)를 상회하며 금리 인하 기대가 후퇴했고, 국내 2분기 GDP 성장률(0.6%)이 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>- 미국 비농업 고용지표가 16만 2천 명 증가하며 예상치를 상회해 금리 인하 경로의 불확실성이 커졌고, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 매크로 환경을 압박함.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31" customHeight="1" s="15">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>- 수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되며 주가를 견인했으나, 개인은 전기·전자에서 91,202억을 순매도하며 차익 실현에 집중함.</t>
+          <t>- 수급 측면에서 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되며 주간 5.93% 상승했고, 기계·장비 섹터 역시 기관(2,736억) 매수와 함께 7.43% 상승하며 주도 섹터로 자리매김함.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="31" customHeight="1" s="15">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>- 종합 관점: 반도체 중심의 수급 쏠림이 뚜렷했으나, 매크로 불확실성과 경기 둔화 신호가 지수 상단을 제한하는 국면으로 전환됨.</t>
+          <t>- 매크로 지표의 둔화 신호에도 불구하고 반도체와 원전 등 특정 섹터로의 수급 쏠림이 뚜렷해, 향후 지수 방향성은 매크로 데이터의 추가 확인과 주도 섹터의 수급 연속성에 좌우될 전망임.</t>
         </is>
       </c>
     </row>
@@ -1842,29 +1842,29 @@
       </c>
       <c r="C46" s="30" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D46" s="28" t="n">
-        <v>-3070</v>
+        <v>-1568</v>
       </c>
       <c r="E46" s="28" t="n">
-        <v>-2520</v>
+        <v>-695</v>
       </c>
       <c r="F46" s="28" t="n">
-        <v>-550</v>
+        <v>-873</v>
       </c>
       <c r="G46" s="29" t="n">
-        <v>3076</v>
+        <v>1591</v>
       </c>
       <c r="H46" s="30" t="n">
-        <v>686.4</v>
+        <v>284</v>
       </c>
       <c r="I46" s="30" t="n">
-        <v>36009</v>
+        <v>13231</v>
       </c>
       <c r="J46" s="30" t="n">
-        <v>-2801</v>
+        <v>-296.9</v>
       </c>
     </row>
     <row r="47">
@@ -1878,29 +1878,29 @@
       </c>
       <c r="C47" s="30" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="D47" s="28" t="n">
-        <v>-1568</v>
+        <v>-968</v>
       </c>
       <c r="E47" s="28" t="n">
-        <v>-695</v>
+        <v>-135</v>
       </c>
       <c r="F47" s="28" t="n">
-        <v>-873</v>
+        <v>-833</v>
       </c>
       <c r="G47" s="29" t="n">
-        <v>1591</v>
+        <v>966</v>
       </c>
       <c r="H47" s="30" t="n">
-        <v>284</v>
+        <v>96.5</v>
       </c>
       <c r="I47" s="30" t="n">
-        <v>13231</v>
+        <v>8138.3</v>
       </c>
       <c r="J47" s="30" t="n">
-        <v>-296.9</v>
+        <v>-220.9</v>
       </c>
     </row>
     <row r="48">
@@ -1914,32 +1914,32 @@
       </c>
       <c r="C48" s="30" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D48" s="28" t="n">
-        <v>-968</v>
+        <v>-783</v>
       </c>
       <c r="E48" s="28" t="n">
-        <v>-135</v>
+        <v>-551</v>
       </c>
       <c r="F48" s="28" t="n">
-        <v>-833</v>
+        <v>-232</v>
       </c>
       <c r="G48" s="29" t="n">
-        <v>966</v>
+        <v>626</v>
       </c>
       <c r="H48" s="30" t="n">
-        <v>96.5</v>
+        <v>125.5</v>
       </c>
       <c r="I48" s="30" t="n">
-        <v>8138.3</v>
+        <v>12546.7</v>
       </c>
       <c r="J48" s="30" t="n">
-        <v>-220.9</v>
-      </c>
-    </row>
-    <row r="49">
+        <v>-283.6</v>
+      </c>
+    </row>
+    <row r="49" ht="31" customHeight="1" s="15">
       <c r="A49" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -1948,34 +1948,34 @@
       <c r="B49" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="C49" s="30" t="inlineStr">
-        <is>
-          <t>셀트리온</t>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D49" s="28" t="n">
-        <v>-783</v>
+        <v>-679</v>
       </c>
       <c r="E49" s="28" t="n">
-        <v>-551</v>
+        <v>-292</v>
       </c>
       <c r="F49" s="28" t="n">
-        <v>-232</v>
+        <v>-386</v>
       </c>
       <c r="G49" s="29" t="n">
-        <v>626</v>
+        <v>764</v>
       </c>
       <c r="H49" s="30" t="n">
-        <v>125.5</v>
+        <v>419.2</v>
       </c>
       <c r="I49" s="30" t="n">
-        <v>12546.7</v>
+        <v>31440</v>
       </c>
       <c r="J49" s="30" t="n">
-        <v>-283.6</v>
-      </c>
-    </row>
-    <row r="50" ht="31" customHeight="1" s="15">
+        <v>-1186.9</v>
+      </c>
+    </row>
+    <row r="50">
       <c r="A50" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -1984,34 +1984,34 @@
       <c r="B50" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C50" s="17" t="inlineStr">
-        <is>
-          <t>LG에너지솔루션</t>
+      <c r="C50" s="30" t="inlineStr">
+        <is>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="D50" s="28" t="n">
-        <v>-679</v>
+        <v>-629</v>
       </c>
       <c r="E50" s="28" t="n">
-        <v>-292</v>
+        <v>-46</v>
       </c>
       <c r="F50" s="28" t="n">
-        <v>-386</v>
+        <v>-583</v>
       </c>
       <c r="G50" s="29" t="n">
-        <v>764</v>
+        <v>634</v>
       </c>
       <c r="H50" s="30" t="n">
-        <v>419.2</v>
+        <v>133.3</v>
       </c>
       <c r="I50" s="30" t="n">
-        <v>31440</v>
+        <v>14504.2</v>
       </c>
       <c r="J50" s="30" t="n">
-        <v>-1186.9</v>
-      </c>
-    </row>
-    <row r="51">
+        <v>-390.7</v>
+      </c>
+    </row>
+    <row r="51" ht="31" customHeight="1" s="15">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2020,34 +2020,34 @@
       <c r="B51" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="C51" s="30" t="inlineStr">
-        <is>
-          <t>에이피알</t>
+      <c r="C51" s="17" t="inlineStr">
+        <is>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="D51" s="28" t="n">
-        <v>-629</v>
+        <v>-593</v>
       </c>
       <c r="E51" s="28" t="n">
-        <v>-46</v>
+        <v>-468</v>
       </c>
       <c r="F51" s="28" t="n">
-        <v>-583</v>
+        <v>-125</v>
       </c>
       <c r="G51" s="29" t="n">
-        <v>634</v>
+        <v>588</v>
       </c>
       <c r="H51" s="30" t="n">
-        <v>133.3</v>
+        <v>222.6</v>
       </c>
       <c r="I51" s="30" t="n">
-        <v>14504.2</v>
+        <v>6895.6</v>
       </c>
       <c r="J51" s="30" t="n">
-        <v>-390.7</v>
-      </c>
-    </row>
-    <row r="52" ht="31" customHeight="1" s="15">
+        <v>-292.3</v>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2056,34 +2056,34 @@
       <c r="B52" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="C52" s="17" t="inlineStr">
-        <is>
-          <t>레인보우로보틱스</t>
+      <c r="C52" s="30" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D52" s="28" t="n">
-        <v>-593</v>
+        <v>-582</v>
       </c>
       <c r="E52" s="28" t="n">
-        <v>-468</v>
+        <v>-195</v>
       </c>
       <c r="F52" s="28" t="n">
-        <v>-125</v>
+        <v>-386</v>
       </c>
       <c r="G52" s="29" t="n">
-        <v>588</v>
+        <v>571</v>
       </c>
       <c r="H52" s="30" t="n">
-        <v>222.6</v>
+        <v>563.7</v>
       </c>
       <c r="I52" s="30" t="n">
-        <v>6895.6</v>
+        <v>9333.9</v>
       </c>
       <c r="J52" s="30" t="n">
-        <v>-292.3</v>
-      </c>
-    </row>
-    <row r="53">
+        <v>-1092.4</v>
+      </c>
+    </row>
+    <row r="53" ht="31" customHeight="1" s="15">
       <c r="A53" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2092,34 +2092,34 @@
       <c r="B53" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="C53" s="30" t="inlineStr">
-        <is>
-          <t>LG이노텍</t>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D53" s="28" t="n">
-        <v>-582</v>
+        <v>-524</v>
       </c>
       <c r="E53" s="28" t="n">
-        <v>-195</v>
-      </c>
-      <c r="F53" s="28" t="n">
-        <v>-386</v>
+        <v>-559</v>
+      </c>
+      <c r="F53" s="29" t="n">
+        <v>35</v>
       </c>
       <c r="G53" s="29" t="n">
-        <v>571</v>
+        <v>528</v>
       </c>
       <c r="H53" s="30" t="n">
-        <v>563.7</v>
+        <v>146.9</v>
       </c>
       <c r="I53" s="30" t="n">
-        <v>9333.9</v>
+        <v>11659.9</v>
       </c>
       <c r="J53" s="30" t="n">
-        <v>-1092.4</v>
-      </c>
-    </row>
-    <row r="54" ht="31" customHeight="1" s="15">
+        <v>-434.4</v>
+      </c>
+    </row>
+    <row r="54">
       <c r="A54" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2128,31 +2128,31 @@
       <c r="B54" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="C54" s="17" t="inlineStr">
-        <is>
-          <t>한화에어로스페이스</t>
+      <c r="C54" s="30" t="inlineStr">
+        <is>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D54" s="28" t="n">
-        <v>-524</v>
-      </c>
-      <c r="E54" s="28" t="n">
-        <v>-559</v>
-      </c>
-      <c r="F54" s="29" t="n">
-        <v>35</v>
+        <v>-511</v>
+      </c>
+      <c r="E54" s="29" t="n">
+        <v>132</v>
+      </c>
+      <c r="F54" s="28" t="n">
+        <v>-643</v>
       </c>
       <c r="G54" s="29" t="n">
-        <v>528</v>
+        <v>559</v>
       </c>
       <c r="H54" s="30" t="n">
-        <v>146.9</v>
+        <v>314.6</v>
       </c>
       <c r="I54" s="30" t="n">
-        <v>11659.9</v>
+        <v>13946.5</v>
       </c>
       <c r="J54" s="30" t="n">
-        <v>-434.4</v>
+        <v>-546.9</v>
       </c>
     </row>
     <row r="55">
@@ -2166,29 +2166,29 @@
       </c>
       <c r="C55" s="30" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>OCI홀딩스</t>
         </is>
       </c>
       <c r="D55" s="28" t="n">
-        <v>-511</v>
-      </c>
-      <c r="E55" s="29" t="n">
-        <v>132</v>
+        <v>-478</v>
+      </c>
+      <c r="E55" s="28" t="n">
+        <v>-42</v>
       </c>
       <c r="F55" s="28" t="n">
-        <v>-643</v>
+        <v>-437</v>
       </c>
       <c r="G55" s="29" t="n">
-        <v>559</v>
+        <v>507</v>
       </c>
       <c r="H55" s="30" t="n">
-        <v>314.6</v>
+        <v>37.7</v>
       </c>
       <c r="I55" s="30" t="n">
-        <v>13946.5</v>
+        <v>3421.8</v>
       </c>
       <c r="J55" s="30" t="n">
-        <v>-546.9</v>
+        <v>-191.7</v>
       </c>
     </row>
     <row r="56"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>주가 상승세에도 대차잔고가 2,044.8억 감소하여 숏커버링 여지가 존재함.</t>
+          <t>주간 순매수 상위 종목이며 대차잔고가 2,044.8억 감소하여 숏커버 여지가 있음.</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>기관 순매수(2,220억)가 집중되며 원전 모멘텀이 지속됨.</t>
+          <t>기관 순매수 2,220억이 집중되었으며 원전 모멘텀이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -2271,12 +2271,12 @@
       </c>
       <c r="B61" s="30" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>주가 하락세 속에서 외국인(-2,520억)과 기관(-550억)의 동반 순매도가 집중됨.</t>
+          <t>주간 순매도 1,568억으로 수급 이탈이 뚜렷함.</t>
         </is>
       </c>
     </row>
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>주가 하락세 속에서 기관(-833억)의 순매도가 집중됨.</t>
+          <t>주간 순매도 968억으로 수급이 악화됨.</t>
         </is>
       </c>
     </row>
@@ -2333,28 +2333,28 @@
     <row r="66" ht="31" customHeight="1" s="15">
       <c r="A66" s="17" t="inlineStr">
         <is>
-          <t>- KOSPI는 외국인과 기관의 강력한 반도체 매수세에 힘입어 6995.39까지 급등했으나, 이후 매크로 경계감으로 6954.52로 조정됨.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" s="15">
+          <t>- 주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 국면을 연출함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="31" customHeight="1" s="15">
       <c r="A67" s="17" t="inlineStr">
         <is>
-          <t>- 미국 비농업고용지표 호조에 따른 금리 인하 기대 후퇴가 시장의 상승 동력을 제한함.</t>
+          <t>- 반도체 및 기계·장비 섹터가 지수 상승을 견인했으나, 주 후반 경기 둔화 우려와 금리 인상 경계감이 부각되며 상승분을 일부 반납함.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="15">
       <c r="A68" s="17" t="inlineStr">
         <is>
-          <t>- 국내 2분기 GDP 성장률이 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>- 미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장의 밸류에이션 부담을 가중시킴.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>- 개인은 전기·전자 섹터에서 91,202억을 순매도하며 대규모 차익 실현에 집중함.</t>
+          <t>- 개인 투자자는 주간 내내 차익 실현 매물을 쏟아내며 외국인·기관의 매수 물량을 받아내는 양상을 보임.</t>
         </is>
       </c>
     </row>
@@ -2382,46 +2382,59 @@
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>- 전기·전자 섹터는 외국인과 기관의 수급 집중으로 강세 지속.</t>
+          <t>- 반도체 및 기계·장비 섹터는 AI 모멘텀과 원전 수주 기대감으로 주간 내내 강세를 유지하며 시장 주도력을 확보함.</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1" s="15">
       <c r="A73" s="17" t="inlineStr">
         <is>
-          <t>- 원전 및 건설 관련주(기계·장비, 전기·가스)는 대형 수주 기대감으로 순환매 흐름.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="15" customHeight="1" s="15">
-      <c r="A74" s="17" t="inlineStr">
-        <is>
-          <t>- 음식료 및 IT 서비스 섹터는 실적 우려와 차익 실현 매물로 약세 전환.</t>
-        </is>
-      </c>
-    </row>
-    <row r="75"/>
-    <row r="76">
-      <c r="A76" s="2" t="inlineStr">
+          <t>- 음식료·담배 및 부동산 섹터는 환율 하락에 따른 수출 우려와 고금리 부담으로 인해 약세 흐름이 지속됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74"/>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B75" s="3" t="inlineStr">
         <is>
           <t>주간 촉매 타임라인</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr"/>
-      <c r="D76" s="3" t="inlineStr"/>
-      <c r="E76" s="3" t="inlineStr"/>
-      <c r="F76" s="3" t="inlineStr"/>
-      <c r="G76" s="3" t="inlineStr"/>
-      <c r="H76" s="3" t="inlineStr"/>
-      <c r="I76" s="3" t="inlineStr"/>
-      <c r="J76" s="18" t="inlineStr">
+      <c r="C75" s="3" t="inlineStr"/>
+      <c r="D75" s="3" t="inlineStr"/>
+      <c r="E75" s="3" t="inlineStr"/>
+      <c r="F75" s="3" t="inlineStr"/>
+      <c r="G75" s="3" t="inlineStr"/>
+      <c r="H75" s="3" t="inlineStr"/>
+      <c r="I75" s="3" t="inlineStr"/>
+      <c r="J75" s="18" t="inlineStr">
         <is>
           <t>등락률 = 주간 누적</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="31" customHeight="1" s="15">
+      <c r="A76" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B76" s="30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="inlineStr"/>
+      <c r="D76" s="14" t="inlineStr"/>
+      <c r="E76" s="29" t="inlineStr"/>
+      <c r="F76" s="17" t="inlineStr">
+        <is>
+          <t>외국인과 기관의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
         </is>
       </c>
     </row>
@@ -2433,15 +2446,25 @@
       </c>
       <c r="B77" s="30" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C77" s="30" t="inlineStr"/>
-      <c r="D77" s="14" t="inlineStr"/>
-      <c r="E77" s="29" t="inlineStr"/>
+          <t>네오오토</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D77" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="E77" s="29" t="n">
+        <v>40.59</v>
+      </c>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
+          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
         </is>
       </c>
     </row>
@@ -2453,7 +2476,7 @@
       </c>
       <c r="B78" s="30" t="inlineStr">
         <is>
-          <t>네오오토</t>
+          <t>필옵틱스</t>
         </is>
       </c>
       <c r="C78" s="30" t="inlineStr">
@@ -2467,11 +2490,11 @@
         </is>
       </c>
       <c r="E78" s="29" t="n">
-        <v>40.59</v>
+        <v>37.21</v>
       </c>
       <c r="F78" s="17" t="inlineStr">
         <is>
-          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
+          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
         </is>
       </c>
     </row>
@@ -2483,7 +2506,7 @@
       </c>
       <c r="B79" s="30" t="inlineStr">
         <is>
-          <t>필옵틱스</t>
+          <t>나무가</t>
         </is>
       </c>
       <c r="C79" s="30" t="inlineStr">
@@ -2497,11 +2520,11 @@
         </is>
       </c>
       <c r="E79" s="29" t="n">
-        <v>37.21</v>
+        <v>10.23</v>
       </c>
       <c r="F79" s="17" t="inlineStr">
         <is>
-          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
+          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -2513,12 +2536,12 @@
       </c>
       <c r="B80" s="30" t="inlineStr">
         <is>
-          <t>나무가</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="C80" s="30" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
@@ -2527,11 +2550,11 @@
         </is>
       </c>
       <c r="E80" s="29" t="n">
-        <v>10.23</v>
+        <v>12.31</v>
       </c>
       <c r="F80" s="17" t="inlineStr">
         <is>
-          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
+          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2566,7 @@
       </c>
       <c r="B81" s="30" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C81" s="30" t="inlineStr">
@@ -2553,15 +2576,15 @@
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="E81" s="29" t="n">
-        <v>12.31</v>
+        <v>15.02</v>
       </c>
       <c r="F81" s="17" t="inlineStr">
         <is>
-          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
+          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2596,7 @@
       </c>
       <c r="B82" s="30" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C82" s="30" t="inlineStr">
@@ -2587,11 +2610,11 @@
         </is>
       </c>
       <c r="E82" s="29" t="n">
-        <v>15.02</v>
+        <v>13.01</v>
       </c>
       <c r="F82" s="17" t="inlineStr">
         <is>
-          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
+          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
         </is>
       </c>
     </row>
@@ -2603,7 +2626,7 @@
       </c>
       <c r="B83" s="30" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C83" s="30" t="inlineStr">
@@ -2617,11 +2640,11 @@
         </is>
       </c>
       <c r="E83" s="29" t="n">
-        <v>13.01</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F83" s="17" t="inlineStr">
         <is>
-          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
+          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -2633,7 +2656,7 @@
       </c>
       <c r="B84" s="30" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="C84" s="30" t="inlineStr">
@@ -2647,45 +2670,35 @@
         </is>
       </c>
       <c r="E84" s="29" t="n">
-        <v>8.859999999999999</v>
+        <v>5.48</v>
       </c>
       <c r="F84" s="17" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
+          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="31" customHeight="1" s="15">
       <c r="A85" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B85" s="30" t="inlineStr">
         <is>
-          <t>삼성전자</t>
-        </is>
-      </c>
-      <c r="C85" s="30" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D85" s="14" t="inlineStr">
-        <is>
-          <t>★★★★</t>
-        </is>
-      </c>
-      <c r="E85" s="29" t="n">
-        <v>5.48</v>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C85" s="30" t="inlineStr"/>
+      <c r="D85" s="14" t="inlineStr"/>
+      <c r="E85" s="29" t="inlineStr"/>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="31" customHeight="1" s="15">
+          <t>2분기 GDP 성장률 0.6%로 둔화 및 국채 금리 급등에 따른 투자 심리 위축으로 KOSPI 0.58% 하락</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="15" customHeight="1" s="15">
       <c r="A86" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -2693,15 +2706,25 @@
       </c>
       <c r="B86" s="30" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C86" s="30" t="inlineStr"/>
-      <c r="D86" s="14" t="inlineStr"/>
-      <c r="E86" s="29" t="inlineStr"/>
+          <t>빛과전자</t>
+        </is>
+      </c>
+      <c r="C86" s="30" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D86" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="E86" s="29" t="n">
+        <v>34.07</v>
+      </c>
       <c r="F86" s="17" t="inlineStr">
         <is>
-          <t>국내 2분기 GDP 성장률 0.6% 발표 및 국채금리 상승 여파로 KOSPI 0.58% 하락.</t>
+          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2736,7 @@
       </c>
       <c r="B87" s="30" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>오르비텍</t>
         </is>
       </c>
       <c r="C87" s="30" t="inlineStr">
@@ -2727,15 +2750,15 @@
         </is>
       </c>
       <c r="E87" s="29" t="n">
-        <v>34.07</v>
+        <v>39.88</v>
       </c>
       <c r="F87" s="17" t="inlineStr">
         <is>
-          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15" customHeight="1" s="15">
+          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="31" customHeight="1" s="15">
       <c r="A88" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -2743,7 +2766,7 @@
       </c>
       <c r="B88" s="30" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>서전기전</t>
         </is>
       </c>
       <c r="C88" s="30" t="inlineStr">
@@ -2757,15 +2780,15 @@
         </is>
       </c>
       <c r="E88" s="29" t="n">
-        <v>39.88</v>
+        <v>37.07</v>
       </c>
       <c r="F88" s="17" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="31" customHeight="1" s="15">
+          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="15" customHeight="1" s="15">
       <c r="A89" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -2773,12 +2796,12 @@
       </c>
       <c r="B89" s="30" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="C89" s="30" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D89" s="14" t="inlineStr">
@@ -2787,11 +2810,11 @@
         </is>
       </c>
       <c r="E89" s="29" t="n">
-        <v>37.07</v>
+        <v>32.53</v>
       </c>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -2803,7 +2826,7 @@
       </c>
       <c r="B90" s="30" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="C90" s="30" t="inlineStr">
@@ -2813,15 +2836,15 @@
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="E90" s="29" t="n">
-        <v>32.53</v>
+        <v>31.32</v>
       </c>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
+          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2856,7 @@
       </c>
       <c r="B91" s="30" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="C91" s="30" t="inlineStr">
@@ -2847,110 +2870,92 @@
         </is>
       </c>
       <c r="E91" s="29" t="n">
-        <v>31.32</v>
+        <v>18.52</v>
       </c>
       <c r="F91" s="17" t="inlineStr">
         <is>
-          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15" customHeight="1" s="15">
-      <c r="A92" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B92" s="30" t="inlineStr">
-        <is>
-          <t>대우건설</t>
-        </is>
-      </c>
-      <c r="C92" s="30" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D92" s="14" t="inlineStr">
-        <is>
-          <t>★★★★</t>
-        </is>
-      </c>
-      <c r="E92" s="29" t="n">
-        <v>18.52</v>
-      </c>
-      <c r="F92" s="17" t="inlineStr">
-        <is>
           <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
         </is>
       </c>
     </row>
-    <row r="93"/>
+    <row r="92"/>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="inlineStr">
+        <is>
+          <t>다음 주 프리뷰</t>
+        </is>
+      </c>
+      <c r="C93" s="3" t="inlineStr"/>
+      <c r="D93" s="3" t="inlineStr"/>
+      <c r="E93" s="3" t="inlineStr"/>
+      <c r="F93" s="3" t="inlineStr"/>
+      <c r="G93" s="3" t="inlineStr"/>
+      <c r="H93" s="3" t="inlineStr"/>
+      <c r="I93" s="3" t="inlineStr"/>
+      <c r="J93" s="3" t="inlineStr"/>
+    </row>
     <row r="94">
-      <c r="A94" s="2" t="inlineStr">
-        <is>
-          <t>11</t>
-        </is>
-      </c>
-      <c r="B94" s="3" t="inlineStr">
-        <is>
-          <t>다음 주 프리뷰</t>
-        </is>
-      </c>
-      <c r="C94" s="3" t="inlineStr"/>
-      <c r="D94" s="3" t="inlineStr"/>
-      <c r="E94" s="3" t="inlineStr"/>
-      <c r="F94" s="3" t="inlineStr"/>
-      <c r="G94" s="3" t="inlineStr"/>
-      <c r="H94" s="3" t="inlineStr"/>
-      <c r="I94" s="3" t="inlineStr"/>
-      <c r="J94" s="3" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="4" t="inlineStr">
+      <c r="A94" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="B94" s="4" t="inlineStr">
         <is>
           <t>내용</t>
         </is>
       </c>
     </row>
+    <row r="95" ht="31" customHeight="1" s="15">
+      <c r="A95" s="31" t="inlineStr">
+        <is>
+          <t>상승 시나리오</t>
+        </is>
+      </c>
+      <c r="B95" s="17" t="inlineStr">
+        <is>
+          <t>반도체 및 원전 관련주가 외국인 수급을 유지하면 지수 하방 경직성 확보 및 완만한 상승세 지속</t>
+        </is>
+      </c>
+    </row>
     <row r="96" ht="31" customHeight="1" s="15">
-      <c r="A96" s="31" t="inlineStr">
-        <is>
-          <t>상승 시나리오</t>
+      <c r="A96" s="32" t="inlineStr">
+        <is>
+          <t>하방 시나리오</t>
         </is>
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>미국 물가 지표가 예상치에 부합하거나 하회하면 반도체 중심의 기술주 반등세 재개</t>
+          <t>미국 물가지표(PPI, CPI)가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 압력 확대</t>
         </is>
       </c>
     </row>
     <row r="97" ht="31" customHeight="1" s="15">
-      <c r="A97" s="32" t="inlineStr">
-        <is>
-          <t>하방 시나리오</t>
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>물가 지표가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 연장</t>
+          <t>9월 10일 발표되는 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과가 금리 경로에 미칠 영향</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="15">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>판별 신호</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>9월 10일 발표될 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2967,7 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>미국 생산자물가지수(PPI)</t>
+          <t>미국 소비자물가지수(CPI)</t>
         </is>
       </c>
     </row>
@@ -2974,24 +2979,12 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>미국 소비자물가지수(CPI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="15" customHeight="1" s="15">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B101" s="17" t="inlineStr">
-        <is>
           <t>국내 무역수지</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="48">
+  <mergeCells count="47">
     <mergeCell ref="A32:J32"/>
     <mergeCell ref="F78:J78"/>
     <mergeCell ref="B98:J98"/>
@@ -2999,7 +2992,6 @@
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="F87:J87"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="B101:J101"/>
     <mergeCell ref="C62:J62"/>
     <mergeCell ref="C58:J58"/>
     <mergeCell ref="G25:J25"/>
@@ -3016,6 +3008,7 @@
     <mergeCell ref="F86:J86"/>
     <mergeCell ref="A30:J30"/>
     <mergeCell ref="F80:J80"/>
+    <mergeCell ref="F76:J76"/>
     <mergeCell ref="B65:J65"/>
     <mergeCell ref="A73:J73"/>
     <mergeCell ref="F79:J79"/>
@@ -3027,15 +3020,14 @@
     <mergeCell ref="F90:J90"/>
     <mergeCell ref="C60:J60"/>
     <mergeCell ref="A69:J69"/>
+    <mergeCell ref="B94:J94"/>
     <mergeCell ref="B97:J97"/>
     <mergeCell ref="C61:J61"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="B100:J100"/>
     <mergeCell ref="A66:J66"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="F92:J92"/>
     <mergeCell ref="F77:J77"/>
-    <mergeCell ref="A74:J74"/>
     <mergeCell ref="F82:J82"/>
     <mergeCell ref="G24:J24"/>
     <mergeCell ref="B96:J96"/>
@@ -3051,7 +3043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J88"/>
+  <dimension ref="A1:J87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" outlineLevelCol="0"/>
   <cols>
     <col width="30.85546875" customWidth="1" style="15" min="1" max="1"/>
@@ -3083,7 +3075,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 21:22 KST</t>
+          <t>2026-09-08 21:31 KST</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3087,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>반도체 주도 급등 후 매크로 경계감에 따른 숨 고르기</t>
+          <t>반도체 주도 랠리와 매크로 불확실성 사이의 줄타기</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3311,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>미국 필라델피아 반도체 지수의 3.37% 급등이 국내 반도체 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도해 지수 급등을 견인함.</t>
+          <t>미국 반도체 지수 급등과 마이크론 강세가 국내 반도체 대형주로 이어지며 외국인·기관의 대규모 매수세와 함께 KOSPI 4.61% 급등을 견인함.</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3326,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, GDP 성장률 둔화까지 겹쳐 지수 하락을 유발함.</t>
+          <t>미국 국채 금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 둔화까지 겹쳐 지수가 0.58% 하락함.</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3346,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>매크로 환경: 미국 비농업고용지수(162K)가 예상치(55K)를 상회하며 금리 인하 기대가 후퇴했고, 국내 2분기 GDP 성장률(0.6%)이 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>미국 비농업 고용지표가 16만 2천 명 증가하며 예상치를 상회해 금리 인하 경로의 불확실성이 커졌고, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 매크로 환경을 압박함.</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3358,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수가 집중되며 주가를 견인했으나, 개인은 전기·전자에서 91,202억을 순매도하며 차익 실현에 집중함.</t>
+          <t>수급 측면에서 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되며 주간 5.93% 상승했고, 기계·장비 섹터 역시 기관(2,736억) 매수와 함께 7.43% 상승하며 주도 섹터로 자리매김함.</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3370,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>종합 관점: 반도체 중심의 수급 쏠림이 뚜렷했으나, 매크로 불확실성과 경기 둔화 신호가 지수 상단을 제한하는 국면으로 전환됨.</t>
+          <t>매크로 지표의 둔화 신호에도 불구하고 반도체와 원전 등 특정 섹터로의 수급 쏠림이 뚜렷해, 향후 지수 방향성은 매크로 데이터의 추가 확인과 주도 섹터의 수급 연속성에 좌우될 전망임.</t>
         </is>
       </c>
     </row>
@@ -3760,29 +3752,29 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>-3070</v>
+        <v>-1568</v>
       </c>
       <c r="E41" t="n">
-        <v>-2520</v>
+        <v>-695</v>
       </c>
       <c r="F41" t="n">
-        <v>-550</v>
+        <v>-873</v>
       </c>
       <c r="G41" t="n">
-        <v>3076</v>
+        <v>1591</v>
       </c>
       <c r="H41" t="n">
-        <v>686.4</v>
+        <v>284</v>
       </c>
       <c r="I41" t="n">
-        <v>36009</v>
+        <v>13231</v>
       </c>
       <c r="J41" t="n">
-        <v>-2801</v>
+        <v>-296.9</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="15">
@@ -3796,29 +3788,29 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-1568</v>
+        <v>-968</v>
       </c>
       <c r="E42" t="n">
-        <v>-695</v>
+        <v>-135</v>
       </c>
       <c r="F42" t="n">
-        <v>-873</v>
+        <v>-833</v>
       </c>
       <c r="G42" t="n">
-        <v>1591</v>
+        <v>966</v>
       </c>
       <c r="H42" t="n">
-        <v>284</v>
+        <v>96.5</v>
       </c>
       <c r="I42" t="n">
-        <v>13231</v>
+        <v>8138.3</v>
       </c>
       <c r="J42" t="n">
-        <v>-296.9</v>
+        <v>-220.9</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
@@ -3832,29 +3824,29 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>-968</v>
+        <v>-783</v>
       </c>
       <c r="E43" t="n">
-        <v>-135</v>
+        <v>-551</v>
       </c>
       <c r="F43" t="n">
-        <v>-833</v>
+        <v>-232</v>
       </c>
       <c r="G43" t="n">
-        <v>966</v>
+        <v>626</v>
       </c>
       <c r="H43" t="n">
-        <v>96.5</v>
+        <v>125.5</v>
       </c>
       <c r="I43" t="n">
-        <v>8138.3</v>
+        <v>12546.7</v>
       </c>
       <c r="J43" t="n">
-        <v>-220.9</v>
+        <v>-283.6</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="15">
@@ -3868,29 +3860,29 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>-783</v>
+        <v>-679</v>
       </c>
       <c r="E44" t="n">
-        <v>-551</v>
+        <v>-292</v>
       </c>
       <c r="F44" t="n">
-        <v>-232</v>
+        <v>-386</v>
       </c>
       <c r="G44" t="n">
-        <v>626</v>
+        <v>764</v>
       </c>
       <c r="H44" t="n">
-        <v>125.5</v>
+        <v>419.2</v>
       </c>
       <c r="I44" t="n">
-        <v>12546.7</v>
+        <v>31440</v>
       </c>
       <c r="J44" t="n">
-        <v>-283.6</v>
+        <v>-1186.9</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="15">
@@ -3904,29 +3896,29 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>-679</v>
+        <v>-629</v>
       </c>
       <c r="E45" t="n">
-        <v>-292</v>
+        <v>-46</v>
       </c>
       <c r="F45" t="n">
-        <v>-386</v>
+        <v>-583</v>
       </c>
       <c r="G45" t="n">
-        <v>764</v>
+        <v>634</v>
       </c>
       <c r="H45" t="n">
-        <v>419.2</v>
+        <v>133.3</v>
       </c>
       <c r="I45" t="n">
-        <v>31440</v>
+        <v>14504.2</v>
       </c>
       <c r="J45" t="n">
-        <v>-1186.9</v>
+        <v>-390.7</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
@@ -3940,29 +3932,29 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>-629</v>
+        <v>-593</v>
       </c>
       <c r="E46" t="n">
-        <v>-46</v>
+        <v>-468</v>
       </c>
       <c r="F46" t="n">
-        <v>-583</v>
+        <v>-125</v>
       </c>
       <c r="G46" t="n">
-        <v>634</v>
+        <v>588</v>
       </c>
       <c r="H46" t="n">
-        <v>133.3</v>
+        <v>222.6</v>
       </c>
       <c r="I46" t="n">
-        <v>14504.2</v>
+        <v>6895.6</v>
       </c>
       <c r="J46" t="n">
-        <v>-390.7</v>
+        <v>-292.3</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">
@@ -3976,29 +3968,29 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-593</v>
+        <v>-582</v>
       </c>
       <c r="E47" t="n">
-        <v>-468</v>
+        <v>-195</v>
       </c>
       <c r="F47" t="n">
-        <v>-125</v>
+        <v>-386</v>
       </c>
       <c r="G47" t="n">
-        <v>588</v>
+        <v>571</v>
       </c>
       <c r="H47" t="n">
-        <v>222.6</v>
+        <v>563.7</v>
       </c>
       <c r="I47" t="n">
-        <v>6895.6</v>
+        <v>9333.9</v>
       </c>
       <c r="J47" t="n">
-        <v>-292.3</v>
+        <v>-1092.4</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="15">
@@ -4012,29 +4004,29 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-582</v>
+        <v>-524</v>
       </c>
       <c r="E48" t="n">
-        <v>-195</v>
+        <v>-559</v>
       </c>
       <c r="F48" t="n">
-        <v>-386</v>
+        <v>35</v>
       </c>
       <c r="G48" t="n">
-        <v>571</v>
+        <v>528</v>
       </c>
       <c r="H48" t="n">
-        <v>563.7</v>
+        <v>146.9</v>
       </c>
       <c r="I48" t="n">
-        <v>9333.9</v>
+        <v>11659.9</v>
       </c>
       <c r="J48" t="n">
-        <v>-1092.4</v>
+        <v>-434.4</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="15">
@@ -4048,29 +4040,29 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-524</v>
+        <v>-511</v>
       </c>
       <c r="E49" t="n">
-        <v>-559</v>
+        <v>132</v>
       </c>
       <c r="F49" t="n">
-        <v>35</v>
+        <v>-643</v>
       </c>
       <c r="G49" t="n">
-        <v>528</v>
+        <v>559</v>
       </c>
       <c r="H49" t="n">
-        <v>146.9</v>
+        <v>314.6</v>
       </c>
       <c r="I49" t="n">
-        <v>11659.9</v>
+        <v>13946.5</v>
       </c>
       <c r="J49" t="n">
-        <v>-434.4</v>
+        <v>-546.9</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="15">
@@ -4084,29 +4076,29 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>OCI홀딩스</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>-511</v>
+        <v>-478</v>
       </c>
       <c r="E50" t="n">
-        <v>132</v>
+        <v>-42</v>
       </c>
       <c r="F50" t="n">
-        <v>-643</v>
+        <v>-437</v>
       </c>
       <c r="G50" t="n">
-        <v>559</v>
+        <v>507</v>
       </c>
       <c r="H50" t="n">
-        <v>314.6</v>
+        <v>37.7</v>
       </c>
       <c r="I50" t="n">
-        <v>13946.5</v>
+        <v>3421.8</v>
       </c>
       <c r="J50" t="n">
-        <v>-546.9</v>
+        <v>-191.7</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="15">
@@ -4129,7 +4121,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>주가 상승세에도 대차잔고가 2,044.8억 감소하여 숏커버링 여지가 존재함.</t>
+          <t>주간 순매수 상위 종목이며 대차잔고가 2,044.8억 감소하여 숏커버 여지가 있음.</t>
         </is>
       </c>
     </row>
@@ -4146,7 +4138,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>기관 순매수(2,220억)가 집중되며 원전 모멘텀이 지속됨.</t>
+          <t>기관 순매수 2,220억이 집중되었으며 원전 모멘텀이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -4158,12 +4150,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>삼성전기</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>주가 하락세 속에서 외국인(-2,520억)과 기관(-550억)의 동반 순매도가 집중됨.</t>
+          <t>주간 순매도 1,568억으로 수급 이탈이 뚜렷함.</t>
         </is>
       </c>
     </row>
@@ -4180,7 +4172,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>주가 하락세 속에서 기관(-833억)의 순매도가 집중됨.</t>
+          <t>주간 순매도 968억으로 수급이 악화됨.</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4191,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>KOSPI는 외국인과 기관의 강력한 반도체 매수세에 힘입어 6995.39까지 급등했으나, 이후 매크로 경계감으로 6954.52로 조정됨.</t>
+          <t>주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 국면을 연출함.</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4203,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>미국 비농업고용지표 호조에 따른 금리 인하 기대 후퇴가 시장의 상승 동력을 제한함.</t>
+          <t>반도체 및 기계·장비 섹터가 지수 상승을 견인했으나, 주 후반 경기 둔화 우려와 금리 인상 경계감이 부각되며 상승분을 일부 반납함.</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4215,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>국내 2분기 GDP 성장률이 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장의 밸류에이션 부담을 가중시킴.</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4227,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>개인은 전기·전자 섹터에서 91,202억을 순매도하며 대규모 차익 실현에 집중함.</t>
+          <t>개인 투자자는 주간 내내 차익 실현 매물을 쏟아내며 외국인·기관의 매수 물량을 받아내는 양상을 보임.</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4246,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>전기·전자 섹터는 외국인과 기관의 수급 집중으로 강세 지속.</t>
+          <t>반도체 및 기계·장비 섹터는 AI 모멘텀과 원전 수주 기대감으로 주간 내내 강세를 유지하며 시장 주도력을 확보함.</t>
         </is>
       </c>
     </row>
@@ -4266,26 +4258,31 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>원전 및 건설 관련주(기계·장비, 전기·가스)는 대형 수주 기대감으로 순환매 흐름.</t>
+          <t>음식료·담배 및 부동산 섹터는 환율 하락에 따른 수출 우려와 고금리 부담으로 인해 약세 흐름이 지속됨.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="15">
       <c r="A64" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>음식료 및 IT 서비스 섹터는 실적 우려와 차익 실현 매물로 약세 전환.</t>
+          <t>10. 촉매 타임라인</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="15">
       <c r="A65" t="inlineStr">
         <is>
-          <t>10. 촉매 타임라인</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>외국인과 기관의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
         </is>
       </c>
     </row>
@@ -4297,12 +4294,23 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>네오오토</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" t="n">
+        <v>40.59</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
+          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
         </is>
       </c>
     </row>
@@ -4314,7 +4322,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>네오오토</t>
+          <t>필옵틱스</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4326,11 +4334,11 @@
         <v>5</v>
       </c>
       <c r="E67" t="n">
-        <v>40.59</v>
+        <v>37.21</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
+          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
         </is>
       </c>
     </row>
@@ -4342,7 +4350,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>필옵틱스</t>
+          <t>나무가</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4354,11 +4362,11 @@
         <v>5</v>
       </c>
       <c r="E68" t="n">
-        <v>37.21</v>
+        <v>10.23</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
+          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -4370,23 +4378,23 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>나무가</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>5</v>
       </c>
       <c r="E69" t="n">
-        <v>10.23</v>
+        <v>12.31</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
+          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -4398,7 +4406,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4407,14 +4415,14 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E70" t="n">
-        <v>12.31</v>
+        <v>15.02</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
+          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4434,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4438,11 +4446,11 @@
         <v>4</v>
       </c>
       <c r="E71" t="n">
-        <v>15.02</v>
+        <v>13.01</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
+          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4462,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4466,11 +4474,11 @@
         <v>4</v>
       </c>
       <c r="E72" t="n">
-        <v>13.01</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
+          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -4482,7 +4490,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4494,39 +4502,28 @@
         <v>4</v>
       </c>
       <c r="E73" t="n">
-        <v>8.859999999999999</v>
+        <v>5.48</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
+          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="15">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>삼성전자</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D74" t="n">
-        <v>4</v>
-      </c>
-      <c r="E74" t="n">
-        <v>5.48</v>
+          <t>—</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
+          <t>2분기 GDP 성장률 0.6%로 둔화 및 국채 금리 급등에 따른 투자 심리 위축으로 KOSPI 0.58% 하락</t>
         </is>
       </c>
     </row>
@@ -4538,12 +4535,23 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>빛과전자</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>5</v>
+      </c>
+      <c r="E75" t="n">
+        <v>34.07</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>국내 2분기 GDP 성장률 0.6% 발표 및 국채금리 상승 여파로 KOSPI 0.58% 하락.</t>
+          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
         </is>
       </c>
     </row>
@@ -4555,7 +4563,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>오르비텍</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4567,11 +4575,11 @@
         <v>5</v>
       </c>
       <c r="E76" t="n">
-        <v>34.07</v>
+        <v>39.88</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
+          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4591,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>서전기전</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4595,11 +4603,11 @@
         <v>5</v>
       </c>
       <c r="E77" t="n">
-        <v>39.88</v>
+        <v>37.07</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
+          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
         </is>
       </c>
     </row>
@@ -4611,23 +4619,23 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D78" t="n">
         <v>5</v>
       </c>
       <c r="E78" t="n">
-        <v>37.07</v>
+        <v>32.53</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -4639,7 +4647,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4648,14 +4656,14 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E79" t="n">
-        <v>32.53</v>
+        <v>31.32</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
+          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
         </is>
       </c>
     </row>
@@ -4667,7 +4675,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4679,82 +4687,66 @@
         <v>4</v>
       </c>
       <c r="E80" t="n">
-        <v>31.32</v>
+        <v>18.52</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
+          <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="15">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>대우건설</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D81" t="n">
-        <v>4</v>
-      </c>
-      <c r="E81" t="n">
-        <v>18.52</v>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
+          <t>11. 다음 주 프리뷰</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="15">
       <c r="A82" t="inlineStr">
         <is>
-          <t>11. 다음 주 프리뷰</t>
+          <t>상승 시나리오</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>반도체 및 원전 관련주가 외국인 수급을 유지하면 지수 하방 경직성 확보 및 완만한 상승세 지속</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="15">
       <c r="A83" t="inlineStr">
         <is>
-          <t>상승 시나리오</t>
+          <t>하방 시나리오</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>미국 물가 지표가 예상치에 부합하거나 하회하면 반도체 중심의 기술주 반등세 재개</t>
+          <t>미국 물가지표(PPI, CPI)가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 압력 확대</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="15">
       <c r="A84" t="inlineStr">
         <is>
-          <t>하방 시나리오</t>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>물가 지표가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 연장</t>
+          <t>9월 10일 발표되는 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과가 금리 경로에 미칠 영향</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="15">
       <c r="A85" t="inlineStr">
         <is>
-          <t>판별 신호</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>9월 10일 발표될 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4758,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>미국 생산자물가지수(PPI)</t>
+          <t>미국 소비자물가지수(CPI)</t>
         </is>
       </c>
     </row>
@@ -4778,22 +4770,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>미국 소비자물가지수(CPI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15" customHeight="1" s="15">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
           <t>국내 무역수지</t>
         </is>
       </c>
     </row>
+    <row r="88" ht="15" customHeight="1" s="15"/>
     <row r="89" ht="15" customHeight="1" s="15"/>
     <row r="90" ht="15" customHeight="1" s="15"/>
     <row r="91" ht="15" customHeight="1" s="15"/>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-09-08 12:43Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -747,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J100"/>
+  <dimension ref="A1:J101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12.9" customWidth="1" style="15" min="1" max="1"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-08 21:31 KST</t>
+          <t>2026-09-08 21:43 KST</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>반도체 주도 랠리와 매크로 불확실성 사이의 줄타기</t>
+          <t>반도체 주도 수급 쏠림과 매크로 불확실성 사이의 줄타기</t>
         </is>
       </c>
     </row>
@@ -1303,7 +1303,7 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>미국 반도체 지수 급등과 마이크론 강세가 국내 반도체 대형주로 이어지며 외국인·기관의 대규모 매수세와 함께 KOSPI 4.61% 급등을 견인함.</t>
+          <t>미국 필라델피아 반도체 지수 3.37% 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 기대 후퇴로 지수 상단은 제한됨.</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>미국 국채 금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 둔화까지 겹쳐 지수가 0.58% 하락함.</t>
+          <t>미국 국채금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 0.6% 발표와 맞물려 지수 하락을 견인함.</t>
         </is>
       </c>
     </row>
@@ -1376,21 +1376,21 @@
     <row r="30" ht="31" customHeight="1" s="15">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>- 미국 비농업 고용지표가 16만 2천 명 증가하며 예상치를 상회해 금리 인하 경로의 불확실성이 커졌고, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 매크로 환경을 압박함.</t>
+          <t>- 매크로 환경은 미국 고용지표가 16만 2천 명 증가하며 견조함을 보였으나, 국내 2분기 GDP 성장률이 0.6%로 이전치 1.8%를 하회하며 경기 둔화 우려가 상존함.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31" customHeight="1" s="15">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>- 수급 측면에서 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되며 주간 5.93% 상승했고, 기계·장비 섹터 역시 기관(2,736억) 매수와 함께 7.43% 상승하며 주도 섹터로 자리매김함.</t>
+          <t>- 수급 구도는 전기·전자 섹터에 외국인 32,305억, 기관 25,821억의 대규모 순매수가 집중되며 반도체 쏠림 현상이 뚜렷했음.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="31" customHeight="1" s="15">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>- 매크로 지표의 둔화 신호에도 불구하고 반도체와 원전 등 특정 섹터로의 수급 쏠림이 뚜렷해, 향후 지수 방향성은 매크로 데이터의 추가 확인과 주도 섹터의 수급 연속성에 좌우될 전망임.</t>
+          <t>- 종합적으로 반도체 중심의 수급 주도력은 강력하나, 매크로 지표의 엇박자와 개인의 차익 실현 매물이 지수 변동성을 키우는 국면임.</t>
         </is>
       </c>
     </row>
@@ -1842,29 +1842,29 @@
       </c>
       <c r="C46" s="30" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D46" s="28" t="n">
-        <v>-1568</v>
+        <v>-3070</v>
       </c>
       <c r="E46" s="28" t="n">
-        <v>-695</v>
+        <v>-2520</v>
       </c>
       <c r="F46" s="28" t="n">
-        <v>-873</v>
+        <v>-550</v>
       </c>
       <c r="G46" s="29" t="n">
-        <v>1591</v>
+        <v>3076</v>
       </c>
       <c r="H46" s="30" t="n">
-        <v>284</v>
+        <v>686.4</v>
       </c>
       <c r="I46" s="30" t="n">
-        <v>13231</v>
+        <v>36009</v>
       </c>
       <c r="J46" s="30" t="n">
-        <v>-296.9</v>
+        <v>-2801</v>
       </c>
     </row>
     <row r="47">
@@ -1878,29 +1878,29 @@
       </c>
       <c r="C47" s="30" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D47" s="28" t="n">
-        <v>-968</v>
+        <v>-1568</v>
       </c>
       <c r="E47" s="28" t="n">
-        <v>-135</v>
+        <v>-695</v>
       </c>
       <c r="F47" s="28" t="n">
-        <v>-833</v>
+        <v>-873</v>
       </c>
       <c r="G47" s="29" t="n">
-        <v>966</v>
+        <v>1591</v>
       </c>
       <c r="H47" s="30" t="n">
-        <v>96.5</v>
+        <v>284</v>
       </c>
       <c r="I47" s="30" t="n">
-        <v>8138.3</v>
+        <v>13231</v>
       </c>
       <c r="J47" s="30" t="n">
-        <v>-220.9</v>
+        <v>-296.9</v>
       </c>
     </row>
     <row r="48">
@@ -1914,32 +1914,32 @@
       </c>
       <c r="C48" s="30" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="D48" s="28" t="n">
-        <v>-783</v>
+        <v>-968</v>
       </c>
       <c r="E48" s="28" t="n">
-        <v>-551</v>
+        <v>-135</v>
       </c>
       <c r="F48" s="28" t="n">
-        <v>-232</v>
+        <v>-833</v>
       </c>
       <c r="G48" s="29" t="n">
-        <v>626</v>
+        <v>966</v>
       </c>
       <c r="H48" s="30" t="n">
-        <v>125.5</v>
+        <v>96.5</v>
       </c>
       <c r="I48" s="30" t="n">
-        <v>12546.7</v>
+        <v>8138.3</v>
       </c>
       <c r="J48" s="30" t="n">
-        <v>-283.6</v>
-      </c>
-    </row>
-    <row r="49" ht="31" customHeight="1" s="15">
+        <v>-220.9</v>
+      </c>
+    </row>
+    <row r="49">
       <c r="A49" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -1948,34 +1948,34 @@
       <c r="B49" s="30" t="n">
         <v>4</v>
       </c>
-      <c r="C49" s="17" t="inlineStr">
-        <is>
-          <t>LG에너지솔루션</t>
+      <c r="C49" s="30" t="inlineStr">
+        <is>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D49" s="28" t="n">
-        <v>-679</v>
+        <v>-783</v>
       </c>
       <c r="E49" s="28" t="n">
-        <v>-292</v>
+        <v>-551</v>
       </c>
       <c r="F49" s="28" t="n">
-        <v>-386</v>
+        <v>-232</v>
       </c>
       <c r="G49" s="29" t="n">
-        <v>764</v>
+        <v>626</v>
       </c>
       <c r="H49" s="30" t="n">
-        <v>419.2</v>
+        <v>125.5</v>
       </c>
       <c r="I49" s="30" t="n">
-        <v>31440</v>
+        <v>12546.7</v>
       </c>
       <c r="J49" s="30" t="n">
-        <v>-1186.9</v>
-      </c>
-    </row>
-    <row r="50">
+        <v>-283.6</v>
+      </c>
+    </row>
+    <row r="50" ht="31" customHeight="1" s="15">
       <c r="A50" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -1984,34 +1984,34 @@
       <c r="B50" s="30" t="n">
         <v>5</v>
       </c>
-      <c r="C50" s="30" t="inlineStr">
-        <is>
-          <t>에이피알</t>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D50" s="28" t="n">
-        <v>-629</v>
+        <v>-679</v>
       </c>
       <c r="E50" s="28" t="n">
-        <v>-46</v>
+        <v>-292</v>
       </c>
       <c r="F50" s="28" t="n">
-        <v>-583</v>
+        <v>-386</v>
       </c>
       <c r="G50" s="29" t="n">
-        <v>634</v>
+        <v>764</v>
       </c>
       <c r="H50" s="30" t="n">
-        <v>133.3</v>
+        <v>419.2</v>
       </c>
       <c r="I50" s="30" t="n">
-        <v>14504.2</v>
+        <v>31440</v>
       </c>
       <c r="J50" s="30" t="n">
-        <v>-390.7</v>
-      </c>
-    </row>
-    <row r="51" ht="31" customHeight="1" s="15">
+        <v>-1186.9</v>
+      </c>
+    </row>
+    <row r="51">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2020,34 +2020,34 @@
       <c r="B51" s="30" t="n">
         <v>6</v>
       </c>
-      <c r="C51" s="17" t="inlineStr">
-        <is>
-          <t>레인보우로보틱스</t>
+      <c r="C51" s="30" t="inlineStr">
+        <is>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="D51" s="28" t="n">
-        <v>-593</v>
+        <v>-629</v>
       </c>
       <c r="E51" s="28" t="n">
-        <v>-468</v>
+        <v>-46</v>
       </c>
       <c r="F51" s="28" t="n">
-        <v>-125</v>
+        <v>-583</v>
       </c>
       <c r="G51" s="29" t="n">
-        <v>588</v>
+        <v>634</v>
       </c>
       <c r="H51" s="30" t="n">
-        <v>222.6</v>
+        <v>133.3</v>
       </c>
       <c r="I51" s="30" t="n">
-        <v>6895.6</v>
+        <v>14504.2</v>
       </c>
       <c r="J51" s="30" t="n">
-        <v>-292.3</v>
-      </c>
-    </row>
-    <row r="52">
+        <v>-390.7</v>
+      </c>
+    </row>
+    <row r="52" ht="31" customHeight="1" s="15">
       <c r="A52" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2056,34 +2056,34 @@
       <c r="B52" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="C52" s="30" t="inlineStr">
-        <is>
-          <t>LG이노텍</t>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="D52" s="28" t="n">
-        <v>-582</v>
+        <v>-593</v>
       </c>
       <c r="E52" s="28" t="n">
-        <v>-195</v>
+        <v>-468</v>
       </c>
       <c r="F52" s="28" t="n">
-        <v>-386</v>
+        <v>-125</v>
       </c>
       <c r="G52" s="29" t="n">
-        <v>571</v>
+        <v>588</v>
       </c>
       <c r="H52" s="30" t="n">
-        <v>563.7</v>
+        <v>222.6</v>
       </c>
       <c r="I52" s="30" t="n">
-        <v>9333.9</v>
+        <v>6895.6</v>
       </c>
       <c r="J52" s="30" t="n">
-        <v>-1092.4</v>
-      </c>
-    </row>
-    <row r="53" ht="31" customHeight="1" s="15">
+        <v>-292.3</v>
+      </c>
+    </row>
+    <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2092,34 +2092,34 @@
       <c r="B53" s="30" t="n">
         <v>8</v>
       </c>
-      <c r="C53" s="17" t="inlineStr">
-        <is>
-          <t>한화에어로스페이스</t>
+      <c r="C53" s="30" t="inlineStr">
+        <is>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D53" s="28" t="n">
-        <v>-524</v>
+        <v>-582</v>
       </c>
       <c r="E53" s="28" t="n">
-        <v>-559</v>
-      </c>
-      <c r="F53" s="29" t="n">
-        <v>35</v>
+        <v>-195</v>
+      </c>
+      <c r="F53" s="28" t="n">
+        <v>-386</v>
       </c>
       <c r="G53" s="29" t="n">
-        <v>528</v>
+        <v>571</v>
       </c>
       <c r="H53" s="30" t="n">
-        <v>146.9</v>
+        <v>563.7</v>
       </c>
       <c r="I53" s="30" t="n">
-        <v>11659.9</v>
+        <v>9333.9</v>
       </c>
       <c r="J53" s="30" t="n">
-        <v>-434.4</v>
-      </c>
-    </row>
-    <row r="54">
+        <v>-1092.4</v>
+      </c>
+    </row>
+    <row r="54" ht="31" customHeight="1" s="15">
       <c r="A54" s="10" t="inlineStr">
         <is>
           <t>순매도 상위</t>
@@ -2128,31 +2128,31 @@
       <c r="B54" s="30" t="n">
         <v>9</v>
       </c>
-      <c r="C54" s="30" t="inlineStr">
-        <is>
-          <t>알테오젠</t>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D54" s="28" t="n">
-        <v>-511</v>
-      </c>
-      <c r="E54" s="29" t="n">
-        <v>132</v>
-      </c>
-      <c r="F54" s="28" t="n">
-        <v>-643</v>
+        <v>-524</v>
+      </c>
+      <c r="E54" s="28" t="n">
+        <v>-559</v>
+      </c>
+      <c r="F54" s="29" t="n">
+        <v>35</v>
       </c>
       <c r="G54" s="29" t="n">
-        <v>559</v>
+        <v>528</v>
       </c>
       <c r="H54" s="30" t="n">
-        <v>314.6</v>
+        <v>146.9</v>
       </c>
       <c r="I54" s="30" t="n">
-        <v>13946.5</v>
+        <v>11659.9</v>
       </c>
       <c r="J54" s="30" t="n">
-        <v>-546.9</v>
+        <v>-434.4</v>
       </c>
     </row>
     <row r="55">
@@ -2166,29 +2166,29 @@
       </c>
       <c r="C55" s="30" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D55" s="28" t="n">
-        <v>-478</v>
-      </c>
-      <c r="E55" s="28" t="n">
-        <v>-42</v>
+        <v>-511</v>
+      </c>
+      <c r="E55" s="29" t="n">
+        <v>132</v>
       </c>
       <c r="F55" s="28" t="n">
-        <v>-437</v>
+        <v>-643</v>
       </c>
       <c r="G55" s="29" t="n">
-        <v>507</v>
+        <v>559</v>
       </c>
       <c r="H55" s="30" t="n">
-        <v>37.7</v>
+        <v>314.6</v>
       </c>
       <c r="I55" s="30" t="n">
-        <v>3421.8</v>
+        <v>13946.5</v>
       </c>
       <c r="J55" s="30" t="n">
-        <v>-191.7</v>
+        <v>-546.9</v>
       </c>
     </row>
     <row r="56"/>
@@ -2242,7 +2242,7 @@
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>주간 순매수 상위 종목이며 대차잔고가 2,044.8억 감소하여 숏커버 여지가 있음.</t>
+          <t>주가 상승에도 대차잔고 감소로 숏커버 여지가 있으며, 외국인과 기관의 순매수가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>기관 순매수 2,220억이 집중되었으며 원전 모멘텀이 지속됨.</t>
+          <t>원전 수주 기대감과 함께 기관 순매수 2,220억이 유입됨.</t>
         </is>
       </c>
     </row>
@@ -2271,12 +2271,12 @@
       </c>
       <c r="B61" s="30" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>주간 순매도 1,568억으로 수급 이탈이 뚜렷함.</t>
+          <t>주가 하락세 속 외국인 -2,520억, 기관 -550억의 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -2293,7 +2293,7 @@
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>주간 순매도 968억으로 수급이 악화됨.</t>
+          <t>주가 하락세 속 기관 -833억의 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -2333,28 +2333,28 @@
     <row r="66" ht="31" customHeight="1" s="15">
       <c r="A66" s="17" t="inlineStr">
         <is>
-          <t>- 주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 국면을 연출함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="31" customHeight="1" s="15">
+          <t>- 주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 장세가 연출됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="15" customHeight="1" s="15">
       <c r="A67" s="17" t="inlineStr">
         <is>
-          <t>- 반도체 및 기계·장비 섹터가 지수 상승을 견인했으나, 주 후반 경기 둔화 우려와 금리 인상 경계감이 부각되며 상승분을 일부 반납함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="15" customHeight="1" s="15">
+          <t>- 반도체 섹터로의 수급 쏠림이 극대화되며 삼성전자와 SK하이닉스가 지수 상승을 견인함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="31" customHeight="1" s="15">
       <c r="A68" s="17" t="inlineStr">
         <is>
-          <t>- 미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장의 밸류에이션 부담을 가중시킴.</t>
+          <t>- 주 후반 미국발 금리 인상 우려와 국내 2분기 GDP 성장률 0.6% 기록에 따른 경기 둔화 우려가 부각되며 상승분 일부를 반납함.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>- 개인 투자자는 주간 내내 차익 실현 매물을 쏟아내며 외국인·기관의 매수 물량을 받아내는 양상을 보임.</t>
+          <t>- 개인 투자자의 대규모 차익 실현 매물이 출회되는 가운데, 원/달러 환율은 1,340원대에서 등락하며 변동성이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -2382,59 +2382,46 @@
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>- 반도체 및 기계·장비 섹터는 AI 모멘텀과 원전 수주 기대감으로 주간 내내 강세를 유지하며 시장 주도력을 확보함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="15" customHeight="1" s="15">
+          <t>- 반도체·AI: 삼성전자와 SK하이닉스 중심의 수급 쏠림이 지속되며 주도 섹터 지위 공고화.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="31" customHeight="1" s="15">
       <c r="A73" s="17" t="inlineStr">
         <is>
-          <t>- 음식료·담배 및 부동산 섹터는 환율 하락에 따른 수출 우려와 고금리 부담으로 인해 약세 흐름이 지속됨.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74"/>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+          <t>- 건설·원전: 미국 내 대형 원전 8기 건설 협의 및 가덕도 신공항 이슈로 건설 및 기계·장비 섹터가 강한 순환매 흐름 형성.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="15" customHeight="1" s="15">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>- 소비재·IT서비스: 환율 하락에 따른 수출 우려와 차익 실현 매물로 음식료 및 IT 서비스 섹터는 약세 전환.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75"/>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>주간 촉매 타임라인</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr"/>
-      <c r="D75" s="3" t="inlineStr"/>
-      <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr"/>
-      <c r="G75" s="3" t="inlineStr"/>
-      <c r="H75" s="3" t="inlineStr"/>
-      <c r="I75" s="3" t="inlineStr"/>
-      <c r="J75" s="18" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr"/>
+      <c r="D76" s="3" t="inlineStr"/>
+      <c r="E76" s="3" t="inlineStr"/>
+      <c r="F76" s="3" t="inlineStr"/>
+      <c r="G76" s="3" t="inlineStr"/>
+      <c r="H76" s="3" t="inlineStr"/>
+      <c r="I76" s="3" t="inlineStr"/>
+      <c r="J76" s="18" t="inlineStr">
         <is>
           <t>등락률 = 주간 누적</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="31" customHeight="1" s="15">
-      <c r="A76" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="B76" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C76" s="30" t="inlineStr"/>
-      <c r="D76" s="14" t="inlineStr"/>
-      <c r="E76" s="29" t="inlineStr"/>
-      <c r="F76" s="17" t="inlineStr">
-        <is>
-          <t>외국인과 기관의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
         </is>
       </c>
     </row>
@@ -2446,25 +2433,15 @@
       </c>
       <c r="B77" s="30" t="inlineStr">
         <is>
-          <t>네오오토</t>
-        </is>
-      </c>
-      <c r="C77" s="30" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="inlineStr">
-        <is>
-          <t>★★★★★</t>
-        </is>
-      </c>
-      <c r="E77" s="29" t="n">
-        <v>40.59</v>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C77" s="30" t="inlineStr"/>
+      <c r="D77" s="14" t="inlineStr"/>
+      <c r="E77" s="29" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
+          <t>KOSPI 4.61% 급등, 외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -2476,7 +2453,7 @@
       </c>
       <c r="B78" s="30" t="inlineStr">
         <is>
-          <t>필옵틱스</t>
+          <t>네오오토</t>
         </is>
       </c>
       <c r="C78" s="30" t="inlineStr">
@@ -2490,11 +2467,11 @@
         </is>
       </c>
       <c r="E78" s="29" t="n">
-        <v>37.21</v>
+        <v>40.59</v>
       </c>
       <c r="F78" s="17" t="inlineStr">
         <is>
-          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
+          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2483,7 @@
       </c>
       <c r="B79" s="30" t="inlineStr">
         <is>
-          <t>나무가</t>
+          <t>필옵틱스</t>
         </is>
       </c>
       <c r="C79" s="30" t="inlineStr">
@@ -2520,11 +2497,11 @@
         </is>
       </c>
       <c r="E79" s="29" t="n">
-        <v>10.23</v>
+        <v>37.21</v>
       </c>
       <c r="F79" s="17" t="inlineStr">
         <is>
-          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
+          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
         </is>
       </c>
     </row>
@@ -2536,12 +2513,12 @@
       </c>
       <c r="B80" s="30" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>나무가</t>
         </is>
       </c>
       <c r="C80" s="30" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D80" s="14" t="inlineStr">
@@ -2550,11 +2527,11 @@
         </is>
       </c>
       <c r="E80" s="29" t="n">
-        <v>12.31</v>
+        <v>10.23</v>
       </c>
       <c r="F80" s="17" t="inlineStr">
         <is>
-          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
+          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -2566,7 +2543,7 @@
       </c>
       <c r="B81" s="30" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="C81" s="30" t="inlineStr">
@@ -2576,15 +2553,15 @@
       </c>
       <c r="D81" s="14" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="E81" s="29" t="n">
-        <v>15.02</v>
+        <v>12.31</v>
       </c>
       <c r="F81" s="17" t="inlineStr">
         <is>
-          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
+          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2573,7 @@
       </c>
       <c r="B82" s="30" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C82" s="30" t="inlineStr">
@@ -2610,11 +2587,11 @@
         </is>
       </c>
       <c r="E82" s="29" t="n">
-        <v>13.01</v>
+        <v>15.02</v>
       </c>
       <c r="F82" s="17" t="inlineStr">
         <is>
-          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
+          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2603,7 @@
       </c>
       <c r="B83" s="30" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C83" s="30" t="inlineStr">
@@ -2640,11 +2617,11 @@
         </is>
       </c>
       <c r="E83" s="29" t="n">
-        <v>8.859999999999999</v>
+        <v>13.01</v>
       </c>
       <c r="F83" s="17" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
+          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
         </is>
       </c>
     </row>
@@ -2656,7 +2633,7 @@
       </c>
       <c r="B84" s="30" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C84" s="30" t="inlineStr">
@@ -2670,61 +2647,61 @@
         </is>
       </c>
       <c r="E84" s="29" t="n">
-        <v>5.48</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F84" s="17" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
+          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="31" customHeight="1" s="15">
       <c r="A85" s="30" t="inlineStr">
         <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B85" s="30" t="inlineStr">
+        <is>
+          <t>삼성전자</t>
+        </is>
+      </c>
+      <c r="C85" s="30" t="inlineStr">
+        <is>
+          <t>KOSPI</t>
+        </is>
+      </c>
+      <c r="D85" s="14" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="E85" s="29" t="n">
+        <v>5.48</v>
+      </c>
+      <c r="F85" s="17" t="inlineStr">
+        <is>
+          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="31" customHeight="1" s="15">
+      <c r="A86" s="30" t="inlineStr">
+        <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B85" s="30" t="inlineStr">
+      <c r="B86" s="30" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C85" s="30" t="inlineStr"/>
-      <c r="D85" s="14" t="inlineStr"/>
-      <c r="E85" s="29" t="inlineStr"/>
-      <c r="F85" s="17" t="inlineStr">
-        <is>
-          <t>2분기 GDP 성장률 0.6%로 둔화 및 국채 금리 급등에 따른 투자 심리 위축으로 KOSPI 0.58% 하락</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="15" customHeight="1" s="15">
-      <c r="A86" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B86" s="30" t="inlineStr">
-        <is>
-          <t>빛과전자</t>
-        </is>
-      </c>
-      <c r="C86" s="30" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D86" s="14" t="inlineStr">
-        <is>
-          <t>★★★★★</t>
-        </is>
-      </c>
-      <c r="E86" s="29" t="n">
-        <v>34.07</v>
-      </c>
+      <c r="C86" s="30" t="inlineStr"/>
+      <c r="D86" s="14" t="inlineStr"/>
+      <c r="E86" s="29" t="inlineStr"/>
       <c r="F86" s="17" t="inlineStr">
         <is>
-          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
+          <t>KOSPI 0.58% 하락, 2분기 GDP 성장률 0.6% 발표에 따른 경기 둔화 우려 부각.</t>
         </is>
       </c>
     </row>
@@ -2736,85 +2713,85 @@
       </c>
       <c r="B87" s="30" t="inlineStr">
         <is>
+          <t>빛과전자</t>
+        </is>
+      </c>
+      <c r="C87" s="30" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D87" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="E87" s="29" t="n">
+        <v>34.07</v>
+      </c>
+      <c r="F87" s="17" t="inlineStr">
+        <is>
+          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1" s="15">
+      <c r="A88" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B88" s="30" t="inlineStr">
+        <is>
           <t>오르비텍</t>
         </is>
       </c>
-      <c r="C87" s="30" t="inlineStr">
+      <c r="C88" s="30" t="inlineStr">
         <is>
           <t>KOSDAQ</t>
         </is>
       </c>
-      <c r="D87" s="14" t="inlineStr">
+      <c r="D88" s="14" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="E87" s="29" t="n">
+      <c r="E88" s="29" t="n">
         <v>39.88</v>
       </c>
-      <c r="F87" s="17" t="inlineStr">
+      <c r="F88" s="17" t="inlineStr">
         <is>
           <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
-    <row r="88" ht="31" customHeight="1" s="15">
-      <c r="A88" s="30" t="inlineStr">
+    <row r="89" ht="31" customHeight="1" s="15">
+      <c r="A89" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B88" s="30" t="inlineStr">
+      <c r="B89" s="30" t="inlineStr">
         <is>
           <t>서전기전</t>
         </is>
       </c>
-      <c r="C88" s="30" t="inlineStr">
+      <c r="C89" s="30" t="inlineStr">
         <is>
           <t>KOSDAQ</t>
         </is>
       </c>
-      <c r="D88" s="14" t="inlineStr">
+      <c r="D89" s="14" t="inlineStr">
         <is>
           <t>★★★★★</t>
         </is>
       </c>
-      <c r="E88" s="29" t="n">
+      <c r="E89" s="29" t="n">
         <v>37.07</v>
       </c>
-      <c r="F88" s="17" t="inlineStr">
+      <c r="F89" s="17" t="inlineStr">
         <is>
           <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="15" customHeight="1" s="15">
-      <c r="A89" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B89" s="30" t="inlineStr">
-        <is>
-          <t>한전기술</t>
-        </is>
-      </c>
-      <c r="C89" s="30" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D89" s="14" t="inlineStr">
-        <is>
-          <t>★★★★★</t>
-        </is>
-      </c>
-      <c r="E89" s="29" t="n">
-        <v>32.53</v>
-      </c>
-      <c r="F89" s="17" t="inlineStr">
-        <is>
-          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -2826,7 +2803,7 @@
       </c>
       <c r="B90" s="30" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="C90" s="30" t="inlineStr">
@@ -2836,15 +2813,15 @@
       </c>
       <c r="D90" s="14" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="E90" s="29" t="n">
-        <v>31.32</v>
+        <v>32.53</v>
       </c>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
+          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -2856,106 +2833,124 @@
       </c>
       <c r="B91" s="30" t="inlineStr">
         <is>
+          <t>현대약품</t>
+        </is>
+      </c>
+      <c r="C91" s="30" t="inlineStr">
+        <is>
+          <t>KOSPI</t>
+        </is>
+      </c>
+      <c r="D91" s="14" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="E91" s="29" t="n">
+        <v>31.32</v>
+      </c>
+      <c r="F91" s="17" t="inlineStr">
+        <is>
+          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="15" customHeight="1" s="15">
+      <c r="A92" s="30" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B92" s="30" t="inlineStr">
+        <is>
           <t>대우건설</t>
         </is>
       </c>
-      <c r="C91" s="30" t="inlineStr">
+      <c r="C92" s="30" t="inlineStr">
         <is>
           <t>KOSPI</t>
         </is>
       </c>
-      <c r="D91" s="14" t="inlineStr">
+      <c r="D92" s="14" t="inlineStr">
         <is>
           <t>★★★★</t>
         </is>
       </c>
-      <c r="E91" s="29" t="n">
+      <c r="E92" s="29" t="n">
         <v>18.52</v>
       </c>
-      <c r="F91" s="17" t="inlineStr">
+      <c r="F92" s="17" t="inlineStr">
         <is>
           <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
         </is>
       </c>
     </row>
-    <row r="92"/>
-    <row r="93">
-      <c r="A93" s="2" t="inlineStr">
+    <row r="93"/>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B93" s="3" t="inlineStr">
+      <c r="B94" s="3" t="inlineStr">
         <is>
           <t>다음 주 프리뷰</t>
         </is>
       </c>
-      <c r="C93" s="3" t="inlineStr"/>
-      <c r="D93" s="3" t="inlineStr"/>
-      <c r="E93" s="3" t="inlineStr"/>
-      <c r="F93" s="3" t="inlineStr"/>
-      <c r="G93" s="3" t="inlineStr"/>
-      <c r="H93" s="3" t="inlineStr"/>
-      <c r="I93" s="3" t="inlineStr"/>
-      <c r="J93" s="3" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="4" t="inlineStr">
+      <c r="C94" s="3" t="inlineStr"/>
+      <c r="D94" s="3" t="inlineStr"/>
+      <c r="E94" s="3" t="inlineStr"/>
+      <c r="F94" s="3" t="inlineStr"/>
+      <c r="G94" s="3" t="inlineStr"/>
+      <c r="H94" s="3" t="inlineStr"/>
+      <c r="I94" s="3" t="inlineStr"/>
+      <c r="J94" s="3" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>내용</t>
         </is>
       </c>
     </row>
-    <row r="95" ht="31" customHeight="1" s="15">
-      <c r="A95" s="31" t="inlineStr">
+    <row r="96" ht="31" customHeight="1" s="15">
+      <c r="A96" s="31" t="inlineStr">
         <is>
           <t>상승 시나리오</t>
         </is>
       </c>
-      <c r="B95" s="17" t="inlineStr">
-        <is>
-          <t>반도체 및 원전 관련주가 외국인 수급을 유지하면 지수 하방 경직성 확보 및 완만한 상승세 지속</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="31" customHeight="1" s="15">
-      <c r="A96" s="32" t="inlineStr">
+      <c r="B96" s="17" t="inlineStr">
+        <is>
+          <t>반도체 수급이 지속되고 미국 물가 지표가 안정적이면 지수 반등 시도</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="31" customHeight="1" s="15">
+      <c r="A97" s="32" t="inlineStr">
         <is>
           <t>하방 시나리오</t>
         </is>
       </c>
-      <c r="B96" s="17" t="inlineStr">
-        <is>
-          <t>미국 물가지표(PPI, CPI)가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 압력 확대</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="31" customHeight="1" s="15">
-      <c r="A97" s="3" t="inlineStr">
-        <is>
-          <t>판별 신호</t>
-        </is>
-      </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>9월 10일 발표되는 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과가 금리 경로에 미칠 영향</t>
+          <t>미국 물가 지표가 예상치를 상회하여 금리 인상 우려가 재점화되면 지수 조정</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="15">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>핵심 이벤트</t>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>미국 생산자물가지수(PPI)</t>
+          <t>9월 10일 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2962,7 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>미국 소비자물가지수(CPI)</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -2979,12 +2974,24 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>국내 무역수지</t>
+          <t>미국 소비자물가지수(CPI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="15">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>핵심 이벤트</t>
+        </is>
+      </c>
+      <c r="B101" s="17" t="inlineStr">
+        <is>
+          <t>한국 무역수지</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="47">
+  <mergeCells count="48">
     <mergeCell ref="A32:J32"/>
     <mergeCell ref="F78:J78"/>
     <mergeCell ref="B98:J98"/>
@@ -2992,6 +2999,7 @@
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="F87:J87"/>
     <mergeCell ref="I2:J2"/>
+    <mergeCell ref="B101:J101"/>
     <mergeCell ref="C62:J62"/>
     <mergeCell ref="C58:J58"/>
     <mergeCell ref="G25:J25"/>
@@ -3008,7 +3016,6 @@
     <mergeCell ref="F86:J86"/>
     <mergeCell ref="A30:J30"/>
     <mergeCell ref="F80:J80"/>
-    <mergeCell ref="F76:J76"/>
     <mergeCell ref="B65:J65"/>
     <mergeCell ref="A73:J73"/>
     <mergeCell ref="F79:J79"/>
@@ -3020,14 +3027,15 @@
     <mergeCell ref="F90:J90"/>
     <mergeCell ref="C60:J60"/>
     <mergeCell ref="A69:J69"/>
-    <mergeCell ref="B94:J94"/>
     <mergeCell ref="B97:J97"/>
     <mergeCell ref="C61:J61"/>
     <mergeCell ref="I1:J1"/>
     <mergeCell ref="B100:J100"/>
     <mergeCell ref="A66:J66"/>
     <mergeCell ref="A4:B4"/>
+    <mergeCell ref="F92:J92"/>
     <mergeCell ref="F77:J77"/>
+    <mergeCell ref="A74:J74"/>
     <mergeCell ref="F82:J82"/>
     <mergeCell ref="G24:J24"/>
     <mergeCell ref="B96:J96"/>
@@ -3043,7 +3051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J87"/>
+  <dimension ref="A1:J88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" outlineLevelCol="0"/>
   <cols>
     <col width="30.85546875" customWidth="1" style="15" min="1" max="1"/>
@@ -3075,7 +3083,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 21:31 KST</t>
+          <t>2026-09-08 21:43 KST</t>
         </is>
       </c>
     </row>
@@ -3087,7 +3095,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>반도체 주도 랠리와 매크로 불확실성 사이의 줄타기</t>
+          <t>반도체 주도 수급 쏠림과 매크로 불확실성 사이의 줄타기</t>
         </is>
       </c>
     </row>
@@ -3311,7 +3319,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>미국 반도체 지수 급등과 마이크론 강세가 국내 반도체 대형주로 이어지며 외국인·기관의 대규모 매수세와 함께 KOSPI 4.61% 급등을 견인함.</t>
+          <t>미국 필라델피아 반도체 지수 3.37% 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 기대 후퇴로 지수 상단은 제한됨.</t>
         </is>
       </c>
     </row>
@@ -3326,7 +3334,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>미국 국채 금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 둔화까지 겹쳐 지수가 0.58% 하락함.</t>
+          <t>미국 국채금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 0.6% 발표와 맞물려 지수 하락을 견인함.</t>
         </is>
       </c>
     </row>
@@ -3346,7 +3354,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>미국 비농업 고용지표가 16만 2천 명 증가하며 예상치를 상회해 금리 인하 경로의 불확실성이 커졌고, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 매크로 환경을 압박함.</t>
+          <t>매크로 환경은 미국 고용지표가 16만 2천 명 증가하며 견조함을 보였으나, 국내 2분기 GDP 성장률이 0.6%로 이전치 1.8%를 하회하며 경기 둔화 우려가 상존함.</t>
         </is>
       </c>
     </row>
@@ -3358,7 +3366,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>수급 측면에서 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되며 주간 5.93% 상승했고, 기계·장비 섹터 역시 기관(2,736억) 매수와 함께 7.43% 상승하며 주도 섹터로 자리매김함.</t>
+          <t>수급 구도는 전기·전자 섹터에 외국인 32,305억, 기관 25,821억의 대규모 순매수가 집중되며 반도체 쏠림 현상이 뚜렷했음.</t>
         </is>
       </c>
     </row>
@@ -3370,7 +3378,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>매크로 지표의 둔화 신호에도 불구하고 반도체와 원전 등 특정 섹터로의 수급 쏠림이 뚜렷해, 향후 지수 방향성은 매크로 데이터의 추가 확인과 주도 섹터의 수급 연속성에 좌우될 전망임.</t>
+          <t>종합적으로 반도체 중심의 수급 주도력은 강력하나, 매크로 지표의 엇박자와 개인의 차익 실현 매물이 지수 변동성을 키우는 국면임.</t>
         </is>
       </c>
     </row>
@@ -3752,29 +3760,29 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>-1568</v>
+        <v>-3070</v>
       </c>
       <c r="E41" t="n">
-        <v>-695</v>
+        <v>-2520</v>
       </c>
       <c r="F41" t="n">
-        <v>-873</v>
+        <v>-550</v>
       </c>
       <c r="G41" t="n">
-        <v>1591</v>
+        <v>3076</v>
       </c>
       <c r="H41" t="n">
-        <v>284</v>
+        <v>686.4</v>
       </c>
       <c r="I41" t="n">
-        <v>13231</v>
+        <v>36009</v>
       </c>
       <c r="J41" t="n">
-        <v>-296.9</v>
+        <v>-2801</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="15">
@@ -3788,29 +3796,29 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>-968</v>
+        <v>-1568</v>
       </c>
       <c r="E42" t="n">
-        <v>-135</v>
+        <v>-695</v>
       </c>
       <c r="F42" t="n">
-        <v>-833</v>
+        <v>-873</v>
       </c>
       <c r="G42" t="n">
-        <v>966</v>
+        <v>1591</v>
       </c>
       <c r="H42" t="n">
-        <v>96.5</v>
+        <v>284</v>
       </c>
       <c r="I42" t="n">
-        <v>8138.3</v>
+        <v>13231</v>
       </c>
       <c r="J42" t="n">
-        <v>-220.9</v>
+        <v>-296.9</v>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="15">
@@ -3824,29 +3832,29 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>셀트리온</t>
+          <t>삼양식품</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>-783</v>
+        <v>-968</v>
       </c>
       <c r="E43" t="n">
-        <v>-551</v>
+        <v>-135</v>
       </c>
       <c r="F43" t="n">
-        <v>-232</v>
+        <v>-833</v>
       </c>
       <c r="G43" t="n">
-        <v>626</v>
+        <v>966</v>
       </c>
       <c r="H43" t="n">
-        <v>125.5</v>
+        <v>96.5</v>
       </c>
       <c r="I43" t="n">
-        <v>12546.7</v>
+        <v>8138.3</v>
       </c>
       <c r="J43" t="n">
-        <v>-283.6</v>
+        <v>-220.9</v>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="15">
@@ -3860,29 +3868,29 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LG에너지솔루션</t>
+          <t>셀트리온</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>-679</v>
+        <v>-783</v>
       </c>
       <c r="E44" t="n">
-        <v>-292</v>
+        <v>-551</v>
       </c>
       <c r="F44" t="n">
-        <v>-386</v>
+        <v>-232</v>
       </c>
       <c r="G44" t="n">
-        <v>764</v>
+        <v>626</v>
       </c>
       <c r="H44" t="n">
-        <v>419.2</v>
+        <v>125.5</v>
       </c>
       <c r="I44" t="n">
-        <v>31440</v>
+        <v>12546.7</v>
       </c>
       <c r="J44" t="n">
-        <v>-1186.9</v>
+        <v>-283.6</v>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="15">
@@ -3896,29 +3904,29 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>에이피알</t>
+          <t>LG에너지솔루션</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>-629</v>
+        <v>-679</v>
       </c>
       <c r="E45" t="n">
-        <v>-46</v>
+        <v>-292</v>
       </c>
       <c r="F45" t="n">
-        <v>-583</v>
+        <v>-386</v>
       </c>
       <c r="G45" t="n">
-        <v>634</v>
+        <v>764</v>
       </c>
       <c r="H45" t="n">
-        <v>133.3</v>
+        <v>419.2</v>
       </c>
       <c r="I45" t="n">
-        <v>14504.2</v>
+        <v>31440</v>
       </c>
       <c r="J45" t="n">
-        <v>-390.7</v>
+        <v>-1186.9</v>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1" s="15">
@@ -3932,29 +3940,29 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>레인보우로보틱스</t>
+          <t>에이피알</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>-593</v>
+        <v>-629</v>
       </c>
       <c r="E46" t="n">
-        <v>-468</v>
+        <v>-46</v>
       </c>
       <c r="F46" t="n">
-        <v>-125</v>
+        <v>-583</v>
       </c>
       <c r="G46" t="n">
-        <v>588</v>
+        <v>634</v>
       </c>
       <c r="H46" t="n">
-        <v>222.6</v>
+        <v>133.3</v>
       </c>
       <c r="I46" t="n">
-        <v>6895.6</v>
+        <v>14504.2</v>
       </c>
       <c r="J46" t="n">
-        <v>-292.3</v>
+        <v>-390.7</v>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1" s="15">
@@ -3968,29 +3976,29 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LG이노텍</t>
+          <t>레인보우로보틱스</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>-582</v>
+        <v>-593</v>
       </c>
       <c r="E47" t="n">
-        <v>-195</v>
+        <v>-468</v>
       </c>
       <c r="F47" t="n">
-        <v>-386</v>
+        <v>-125</v>
       </c>
       <c r="G47" t="n">
-        <v>571</v>
+        <v>588</v>
       </c>
       <c r="H47" t="n">
-        <v>563.7</v>
+        <v>222.6</v>
       </c>
       <c r="I47" t="n">
-        <v>9333.9</v>
+        <v>6895.6</v>
       </c>
       <c r="J47" t="n">
-        <v>-1092.4</v>
+        <v>-292.3</v>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="15">
@@ -4004,29 +4012,29 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>한화에어로스페이스</t>
+          <t>LG이노텍</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>-524</v>
+        <v>-582</v>
       </c>
       <c r="E48" t="n">
-        <v>-559</v>
+        <v>-195</v>
       </c>
       <c r="F48" t="n">
-        <v>35</v>
+        <v>-386</v>
       </c>
       <c r="G48" t="n">
-        <v>528</v>
+        <v>571</v>
       </c>
       <c r="H48" t="n">
-        <v>146.9</v>
+        <v>563.7</v>
       </c>
       <c r="I48" t="n">
-        <v>11659.9</v>
+        <v>9333.9</v>
       </c>
       <c r="J48" t="n">
-        <v>-434.4</v>
+        <v>-1092.4</v>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="15">
@@ -4040,29 +4048,29 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>알테오젠</t>
+          <t>한화에어로스페이스</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>-511</v>
+        <v>-524</v>
       </c>
       <c r="E49" t="n">
-        <v>132</v>
+        <v>-559</v>
       </c>
       <c r="F49" t="n">
-        <v>-643</v>
+        <v>35</v>
       </c>
       <c r="G49" t="n">
-        <v>559</v>
+        <v>528</v>
       </c>
       <c r="H49" t="n">
-        <v>314.6</v>
+        <v>146.9</v>
       </c>
       <c r="I49" t="n">
-        <v>13946.5</v>
+        <v>11659.9</v>
       </c>
       <c r="J49" t="n">
-        <v>-546.9</v>
+        <v>-434.4</v>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="15">
@@ -4076,29 +4084,29 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>OCI홀딩스</t>
+          <t>알테오젠</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>-478</v>
+        <v>-511</v>
       </c>
       <c r="E50" t="n">
-        <v>-42</v>
+        <v>132</v>
       </c>
       <c r="F50" t="n">
-        <v>-437</v>
+        <v>-643</v>
       </c>
       <c r="G50" t="n">
-        <v>507</v>
+        <v>559</v>
       </c>
       <c r="H50" t="n">
-        <v>37.7</v>
+        <v>314.6</v>
       </c>
       <c r="I50" t="n">
-        <v>3421.8</v>
+        <v>13946.5</v>
       </c>
       <c r="J50" t="n">
-        <v>-191.7</v>
+        <v>-546.9</v>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="15">
@@ -4121,7 +4129,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>주간 순매수 상위 종목이며 대차잔고가 2,044.8억 감소하여 숏커버 여지가 있음.</t>
+          <t>주가 상승에도 대차잔고 감소로 숏커버 여지가 있으며, 외국인과 기관의 순매수가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -4138,7 +4146,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>기관 순매수 2,220억이 집중되었으며 원전 모멘텀이 지속됨.</t>
+          <t>원전 수주 기대감과 함께 기관 순매수 2,220억이 유입됨.</t>
         </is>
       </c>
     </row>
@@ -4150,12 +4158,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>삼성SDI</t>
+          <t>삼성전기</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>주간 순매도 1,568억으로 수급 이탈이 뚜렷함.</t>
+          <t>주가 하락세 속 외국인 -2,520억, 기관 -550억의 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -4172,7 +4180,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>주간 순매도 968억으로 수급이 악화됨.</t>
+          <t>주가 하락세 속 기관 -833억의 순매도가 집중됨.</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4199,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 국면을 연출함.</t>
+          <t>주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 장세가 연출됨.</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4211,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>반도체 및 기계·장비 섹터가 지수 상승을 견인했으나, 주 후반 경기 둔화 우려와 금리 인상 경계감이 부각되며 상승분을 일부 반납함.</t>
+          <t>반도체 섹터로의 수급 쏠림이 극대화되며 삼성전자와 SK하이닉스가 지수 상승을 견인함.</t>
         </is>
       </c>
     </row>
@@ -4215,7 +4223,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 급등이 시장의 밸류에이션 부담을 가중시킴.</t>
+          <t>주 후반 미국발 금리 인상 우려와 국내 2분기 GDP 성장률 0.6% 기록에 따른 경기 둔화 우려가 부각되며 상승분 일부를 반납함.</t>
         </is>
       </c>
     </row>
@@ -4227,7 +4235,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>개인 투자자는 주간 내내 차익 실현 매물을 쏟아내며 외국인·기관의 매수 물량을 받아내는 양상을 보임.</t>
+          <t>개인 투자자의 대규모 차익 실현 매물이 출회되는 가운데, 원/달러 환율은 1,340원대에서 등락하며 변동성이 지속됨.</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4254,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>반도체 및 기계·장비 섹터는 AI 모멘텀과 원전 수주 기대감으로 주간 내내 강세를 유지하며 시장 주도력을 확보함.</t>
+          <t>반도체·AI: 삼성전자와 SK하이닉스 중심의 수급 쏠림이 지속되며 주도 섹터 지위 공고화.</t>
         </is>
       </c>
     </row>
@@ -4258,31 +4266,26 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>음식료·담배 및 부동산 섹터는 환율 하락에 따른 수출 우려와 고금리 부담으로 인해 약세 흐름이 지속됨.</t>
+          <t>건설·원전: 미국 내 대형 원전 8기 건설 협의 및 가덕도 신공항 이슈로 건설 및 기계·장비 섹터가 강한 순환매 흐름 형성.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="15">
       <c r="A64" t="inlineStr">
         <is>
-          <t>10. 촉매 타임라인</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>소비재·IT서비스: 환율 하락에 따른 수출 우려와 차익 실현 매물로 음식료 및 IT 서비스 섹터는 약세 전환.</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="15">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>외국인과 기관의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등</t>
+          <t>10. 촉매 타임라인</t>
         </is>
       </c>
     </row>
@@ -4294,23 +4297,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>네오오토</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D66" t="n">
-        <v>5</v>
-      </c>
-      <c r="E66" t="n">
-        <v>40.59</v>
+          <t>—</t>
+        </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
+          <t>KOSPI 4.61% 급등, 외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -4322,7 +4314,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>필옵틱스</t>
+          <t>네오오토</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -4334,11 +4326,11 @@
         <v>5</v>
       </c>
       <c r="E67" t="n">
-        <v>37.21</v>
+        <v>40.59</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
+          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
         </is>
       </c>
     </row>
@@ -4350,7 +4342,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>나무가</t>
+          <t>필옵틱스</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -4362,11 +4354,11 @@
         <v>5</v>
       </c>
       <c r="E68" t="n">
-        <v>10.23</v>
+        <v>37.21</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
+          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
         </is>
       </c>
     </row>
@@ -4378,23 +4370,23 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>나무가</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>5</v>
       </c>
       <c r="E69" t="n">
-        <v>12.31</v>
+        <v>10.23</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
+          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -4406,7 +4398,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -4415,14 +4407,14 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E70" t="n">
-        <v>15.02</v>
+        <v>12.31</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
+          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -4434,7 +4426,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4446,11 +4438,11 @@
         <v>4</v>
       </c>
       <c r="E71" t="n">
-        <v>13.01</v>
+        <v>15.02</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
+          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4454,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -4474,11 +4466,11 @@
         <v>4</v>
       </c>
       <c r="E72" t="n">
-        <v>8.859999999999999</v>
+        <v>13.01</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
+          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
         </is>
       </c>
     </row>
@@ -4490,7 +4482,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -4502,28 +4494,39 @@
         <v>4</v>
       </c>
       <c r="E73" t="n">
-        <v>5.48</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
+          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1" s="15">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>삼성전자</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>KOSPI</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>4</v>
+      </c>
+      <c r="E74" t="n">
+        <v>5.48</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>2분기 GDP 성장률 0.6%로 둔화 및 국채 금리 급등에 따른 투자 심리 위축으로 KOSPI 0.58% 하락</t>
+          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -4535,23 +4538,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>빛과전자</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>KOSDAQ</t>
-        </is>
-      </c>
-      <c r="D75" t="n">
-        <v>5</v>
-      </c>
-      <c r="E75" t="n">
-        <v>34.07</v>
+          <t>—</t>
+        </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
+          <t>KOSPI 0.58% 하락, 2분기 GDP 성장률 0.6% 발표에 따른 경기 둔화 우려 부각.</t>
         </is>
       </c>
     </row>
@@ -4563,7 +4555,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4575,11 +4567,11 @@
         <v>5</v>
       </c>
       <c r="E76" t="n">
-        <v>39.88</v>
+        <v>34.07</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
+          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
         </is>
       </c>
     </row>
@@ -4591,7 +4583,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>오르비텍</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -4603,11 +4595,11 @@
         <v>5</v>
       </c>
       <c r="E77" t="n">
-        <v>37.07</v>
+        <v>39.88</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -4619,23 +4611,23 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>한전기술</t>
+          <t>서전기전</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D78" t="n">
         <v>5</v>
       </c>
       <c r="E78" t="n">
-        <v>32.53</v>
+        <v>37.07</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
+          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
         </is>
       </c>
     </row>
@@ -4647,7 +4639,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>현대약품</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -4656,14 +4648,14 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E79" t="n">
-        <v>31.32</v>
+        <v>32.53</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
+          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -4675,7 +4667,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>대우건설</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -4687,66 +4679,82 @@
         <v>4</v>
       </c>
       <c r="E80" t="n">
-        <v>18.52</v>
+        <v>31.32</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
+          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="15">
       <c r="A81" t="inlineStr">
         <is>
-          <t>11. 다음 주 프리뷰</t>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>대우건설</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>KOSPI</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>4</v>
+      </c>
+      <c r="E81" t="n">
+        <v>18.52</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="15">
       <c r="A82" t="inlineStr">
         <is>
-          <t>상승 시나리오</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>반도체 및 원전 관련주가 외국인 수급을 유지하면 지수 하방 경직성 확보 및 완만한 상승세 지속</t>
+          <t>11. 다음 주 프리뷰</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="15">
       <c r="A83" t="inlineStr">
         <is>
-          <t>하방 시나리오</t>
+          <t>상승 시나리오</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>미국 물가지표(PPI, CPI)가 예상치를 상회하여 금리 인상 우려가 심화되면 지수 조정 압력 확대</t>
+          <t>반도체 수급이 지속되고 미국 물가 지표가 안정적이면 지수 반등 시도</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="15">
       <c r="A84" t="inlineStr">
         <is>
-          <t>판별 신호</t>
+          <t>하방 시나리오</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>9월 10일 발표되는 미국 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과가 금리 경로에 미칠 영향</t>
+          <t>미국 물가 지표가 예상치를 상회하여 금리 인상 우려가 재점화되면 지수 조정</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="15">
       <c r="A85" t="inlineStr">
         <is>
-          <t>핵심 이벤트</t>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>미국 생산자물가지수(PPI)</t>
+          <t>9월 10일 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
         </is>
       </c>
     </row>
@@ -4758,7 +4766,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>미국 소비자물가지수(CPI)</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -4770,11 +4778,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>국내 무역수지</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15" customHeight="1" s="15"/>
+          <t>미국 소비자물가지수(CPI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="15" customHeight="1" s="15">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>핵심 이벤트</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>한국 무역수지</t>
+        </is>
+      </c>
+    </row>
     <row r="89" ht="15" customHeight="1" s="15"/>
     <row r="90" ht="15" customHeight="1" s="15"/>
     <row r="91" ht="15" customHeight="1" s="15"/>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-09-08 12:56Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-08 21:43 KST</t>
+          <t>2026-09-08 21:56 KST</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>반도체 주도 수급 쏠림과 매크로 불확실성 사이의 줄타기</t>
+          <t>AI 반도체 주도 랠리와 매크로 불확실성 사이의 줄타기</t>
         </is>
       </c>
     </row>
@@ -1303,11 +1303,11 @@
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>미국 필라델피아 반도체 지수 3.37% 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 기대 후퇴로 지수 상단은 제한됨.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1" s="15">
+          <t>필라델피아 반도체 지수의 3.37% 급등과 마이크론 상승세가 국내 반도체 소부장 및 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="44.5" customHeight="1" s="15">
       <c r="A26" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -1336,7 +1336,7 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 0.6% 발표와 맞물려 지수 하락을 견인함.</t>
+          <t>미국 국채금리 급등과 연준의 금리 인상 가능성 제기라는 매크로 악재가 국내 2분기 GDP 성장률 둔화와 맞물리며 지수 하락을 압박함.</t>
         </is>
       </c>
     </row>
@@ -1376,21 +1376,21 @@
     <row r="30" ht="31" customHeight="1" s="15">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>- 매크로 환경은 미국 고용지표가 16만 2천 명 증가하며 견조함을 보였으나, 국내 2분기 GDP 성장률이 0.6%로 이전치 1.8%를 하회하며 경기 둔화 우려가 상존함.</t>
+          <t>- 미국 8월 비농업 고용지수가 16만 2천 명 증가하며 예상치(55.0K)를 상회하는 서프라이즈를 기록했으나, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 매크로 환경의 불확실성을 높임.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="31" customHeight="1" s="15">
       <c r="A31" s="17" t="inlineStr">
         <is>
-          <t>- 수급 구도는 전기·전자 섹터에 외국인 32,305억, 기관 25,821억의 대규모 순매수가 집중되며 반도체 쏠림 현상이 뚜렷했음.</t>
+          <t>- 수급 측면에서는 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되었으며, 삼성전자(45,121억)와 SK하이닉스(29,092억)가 주간 순매수 상위를 독점함.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="31" customHeight="1" s="15">
       <c r="A32" s="17" t="inlineStr">
         <is>
-          <t>- 종합적으로 반도체 중심의 수급 주도력은 강력하나, 매크로 지표의 엇박자와 개인의 차익 실현 매물이 지수 변동성을 키우는 국면임.</t>
+          <t>- 반도체 중심의 수급 쏠림이 지수를 방어하고 있으나, 매크로 지표의 엇갈린 신호와 경기 둔화 우려가 공존하며 시장의 변동성이 확대되는 국면임.</t>
         </is>
       </c>
     </row>
@@ -2237,12 +2237,12 @@
       </c>
       <c r="B59" s="30" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>주가 상승에도 대차잔고 감소로 숏커버 여지가 있으며, 외국인과 기관의 순매수가 집중됨.</t>
+          <t>주간 순매수 45,121억으로 수급 집중도 최상위</t>
         </is>
       </c>
     </row>
@@ -2254,12 +2254,12 @@
       </c>
       <c r="B60" s="30" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>원전 수주 기대감과 함께 기관 순매수 2,220억이 유입됨.</t>
+          <t>주간 순매수 29,092억 및 대차잔고 감소로 숏커버 여지</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>주가 하락세 속 외국인 -2,520억, 기관 -550억의 순매도가 집중됨.</t>
+          <t>주간 순매수 -3,070억으로 수급 이탈 뚜렷</t>
         </is>
       </c>
     </row>
@@ -2288,12 +2288,12 @@
       </c>
       <c r="B62" s="30" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>주가 하락세 속 기관 -833억의 순매도가 집중됨.</t>
+          <t>주간 순매수 -1,568억으로 수급 약세 지속</t>
         </is>
       </c>
     </row>
@@ -2333,28 +2333,28 @@
     <row r="66" ht="31" customHeight="1" s="15">
       <c r="A66" s="17" t="inlineStr">
         <is>
-          <t>- 주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 장세가 연출됨.</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" s="15">
+          <t>- 주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 등 강한 'Risk-On' 국면을 연출함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="31" customHeight="1" s="15">
       <c r="A67" s="17" t="inlineStr">
         <is>
-          <t>- 반도체 섹터로의 수급 쏠림이 극대화되며 삼성전자와 SK하이닉스가 지수 상승을 견인함.</t>
+          <t>- 미국 필라델피아 반도체 지수의 강세가 국내 반도체 대형주로 이어지며 지수 상승을 견인했으나, 주 후반 금리 인상 우려와 국채 금리 급등으로 상승폭을 일부 반납함.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="31" customHeight="1" s="15">
       <c r="A68" s="17" t="inlineStr">
         <is>
-          <t>- 주 후반 미국발 금리 인상 우려와 국내 2분기 GDP 성장률 0.6% 기록에 따른 경기 둔화 우려가 부각되며 상승분 일부를 반납함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="15" customHeight="1" s="15">
+          <t>- 개인 투자자는 주간 내내 대규모 순매도를 기록하며 차익 실현에 집중한 반면, 외국인과 기관은 삼성전자와 SK하이닉스를 중심으로 수급을 집중함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="31" customHeight="1" s="15">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>- 개인 투자자의 대규모 차익 실현 매물이 출회되는 가운데, 원/달러 환율은 1,340원대에서 등락하며 변동성이 지속됨.</t>
+          <t>- 국내 2분기 GDP 성장률이 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각된 점이 시장의 상단을 제한하는 요인으로 작용함.</t>
         </is>
       </c>
     </row>
@@ -2382,21 +2382,21 @@
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>- 반도체·AI: 삼성전자와 SK하이닉스 중심의 수급 쏠림이 지속되며 주도 섹터 지위 공고화.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="31" customHeight="1" s="15">
+          <t>- 전기·전자 및 기계·장비 섹터가 AI 반도체 및 원전 수주 기대감으로 주도주 지위를 공고히 함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="15" customHeight="1" s="15">
       <c r="A73" s="17" t="inlineStr">
         <is>
-          <t>- 건설·원전: 미국 내 대형 원전 8기 건설 협의 및 가덕도 신공항 이슈로 건설 및 기계·장비 섹터가 강한 순환매 흐름 형성.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="15" customHeight="1" s="15">
+          <t>- 건설 섹터는 미국 내 대형 원전 8기 건설 협의 소식에 힘입어 주간 7.86% 상승하며 강한 모멘텀을 보임.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="31" customHeight="1" s="15">
       <c r="A74" s="17" t="inlineStr">
         <is>
-          <t>- 소비재·IT서비스: 환율 하락에 따른 수출 우려와 차익 실현 매물로 음식료 및 IT 서비스 섹터는 약세 전환.</t>
+          <t>- 반면 음식료·담배 및 부동산 섹터는 환율 하락과 고금리 장기화 부담으로 인해 차익 실현 매물이 출회되며 약세를 면치 못함.</t>
         </is>
       </c>
     </row>
@@ -2441,7 +2441,7 @@
       <c r="E77" s="29" t="inlineStr"/>
       <c r="F77" s="17" t="inlineStr">
         <is>
-          <t>KOSPI 4.61% 급등, 외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입.</t>
+          <t>미국 8월 비농업 고용지수 예상치 상회 및 필라델피아 반도체 지수 급등에 따른 국내 반도체 중심의 강세.</t>
         </is>
       </c>
     </row>
@@ -2701,7 +2701,7 @@
       <c r="E86" s="29" t="inlineStr"/>
       <c r="F86" s="17" t="inlineStr">
         <is>
-          <t>KOSPI 0.58% 하락, 2분기 GDP 성장률 0.6% 발표에 따른 경기 둔화 우려 부각.</t>
+          <t>국내 2분기 GDP 성장률 0.6%로 둔화 및 미국 금리 인상 우려 부각에 따른 지수 조정.</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2926,7 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>반도체 수급이 지속되고 미국 물가 지표가 안정적이면 지수 반등 시도</t>
+          <t>반도체 대형주 수급 유지 시 지수 하단 지지</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>미국 물가 지표가 예상치를 상회하여 금리 인상 우려가 재점화되면 지수 조정</t>
+          <t>미국 물가 지표 충격 시 금리 인상 우려 재점화</t>
         </is>
       </c>
     </row>
@@ -2950,7 +2950,7 @@
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>9월 10일 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
+          <t>미국 CPI 및 PPI 발표 결과</t>
         </is>
       </c>
     </row>
@@ -2962,7 +2962,7 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>미국 생산자물가지수(PPI)</t>
+          <t>미국 소비자물가지수(CPI)</t>
         </is>
       </c>
     </row>
@@ -2974,7 +2974,7 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>미국 소비자물가지수(CPI)</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -2986,7 +2986,7 @@
       </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>한국 무역수지</t>
+          <t>국내 무역수지</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-08 21:43 KST</t>
+          <t>2026-09-08 21:56 KST</t>
         </is>
       </c>
     </row>
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>반도체 주도 수급 쏠림과 매크로 불확실성 사이의 줄타기</t>
+          <t>AI 반도체 주도 랠리와 매크로 불확실성 사이의 줄타기</t>
         </is>
       </c>
     </row>
@@ -3319,7 +3319,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>미국 필라델피아 반도체 지수 3.37% 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 기대 후퇴로 지수 상단은 제한됨.</t>
+          <t>필라델피아 반도체 지수의 3.37% 급등과 마이크론 상승세가 국내 반도체 소부장 및 대형주로 이어지며 외국인·기관의 강력한 매수세를 유도함.</t>
         </is>
       </c>
     </row>
@@ -3334,7 +3334,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담으로 작용하며, 2분기 GDP 성장률 0.6% 발표와 맞물려 지수 하락을 견인함.</t>
+          <t>미국 국채금리 급등과 연준의 금리 인상 가능성 제기라는 매크로 악재가 국내 2분기 GDP 성장률 둔화와 맞물리며 지수 하락을 압박함.</t>
         </is>
       </c>
     </row>
@@ -3354,7 +3354,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>매크로 환경은 미국 고용지표가 16만 2천 명 증가하며 견조함을 보였으나, 국내 2분기 GDP 성장률이 0.6%로 이전치 1.8%를 하회하며 경기 둔화 우려가 상존함.</t>
+          <t>미국 8월 비농업 고용지수가 16만 2천 명 증가하며 예상치(55.0K)를 상회하는 서프라이즈를 기록했으나, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 매크로 환경의 불확실성을 높임.</t>
         </is>
       </c>
     </row>
@@ -3366,7 +3366,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>수급 구도는 전기·전자 섹터에 외국인 32,305억, 기관 25,821억의 대규모 순매수가 집중되며 반도체 쏠림 현상이 뚜렷했음.</t>
+          <t>수급 측면에서는 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되었으며, 삼성전자(45,121억)와 SK하이닉스(29,092억)가 주간 순매수 상위를 독점함.</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>종합적으로 반도체 중심의 수급 주도력은 강력하나, 매크로 지표의 엇박자와 개인의 차익 실현 매물이 지수 변동성을 키우는 국면임.</t>
+          <t>반도체 중심의 수급 쏠림이 지수를 방어하고 있으나, 매크로 지표의 엇갈린 신호와 경기 둔화 우려가 공존하며 시장의 변동성이 확대되는 국면임.</t>
         </is>
       </c>
     </row>
@@ -4124,12 +4124,12 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>주가 상승에도 대차잔고 감소로 숏커버 여지가 있으며, 외국인과 기관의 순매수가 집중됨.</t>
+          <t>주간 순매수 45,121억으로 수급 집중도 최상위</t>
         </is>
       </c>
     </row>
@@ -4141,12 +4141,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>원전 수주 기대감과 함께 기관 순매수 2,220억이 유입됨.</t>
+          <t>주간 순매수 29,092억 및 대차잔고 감소로 숏커버 여지</t>
         </is>
       </c>
     </row>
@@ -4163,7 +4163,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>주가 하락세 속 외국인 -2,520억, 기관 -550억의 순매도가 집중됨.</t>
+          <t>주간 순매수 -3,070억으로 수급 이탈 뚜렷</t>
         </is>
       </c>
     </row>
@@ -4175,12 +4175,12 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>삼양식품</t>
+          <t>삼성SDI</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>주가 하락세 속 기관 -833억의 순매도가 집중됨.</t>
+          <t>주간 순매수 -1,568억으로 수급 약세 지속</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 강한 'Risk-On' 장세가 연출됨.</t>
+          <t>주 초반 외국인과 기관의 강력한 동반 매수세가 유입되며 KOSPI가 4.61% 급등하는 등 강한 'Risk-On' 국면을 연출함.</t>
         </is>
       </c>
     </row>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>반도체 섹터로의 수급 쏠림이 극대화되며 삼성전자와 SK하이닉스가 지수 상승을 견인함.</t>
+          <t>미국 필라델피아 반도체 지수의 강세가 국내 반도체 대형주로 이어지며 지수 상승을 견인했으나, 주 후반 금리 인상 우려와 국채 금리 급등으로 상승폭을 일부 반납함.</t>
         </is>
       </c>
     </row>
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>주 후반 미국발 금리 인상 우려와 국내 2분기 GDP 성장률 0.6% 기록에 따른 경기 둔화 우려가 부각되며 상승분 일부를 반납함.</t>
+          <t>개인 투자자는 주간 내내 대규모 순매도를 기록하며 차익 실현에 집중한 반면, 외국인과 기관은 삼성전자와 SK하이닉스를 중심으로 수급을 집중함.</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>개인 투자자의 대규모 차익 실현 매물이 출회되는 가운데, 원/달러 환율은 1,340원대에서 등락하며 변동성이 지속됨.</t>
+          <t>국내 2분기 GDP 성장률이 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각된 점이 시장의 상단을 제한하는 요인으로 작용함.</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4254,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>반도체·AI: 삼성전자와 SK하이닉스 중심의 수급 쏠림이 지속되며 주도 섹터 지위 공고화.</t>
+          <t>전기·전자 및 기계·장비 섹터가 AI 반도체 및 원전 수주 기대감으로 주도주 지위를 공고히 함.</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4266,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>건설·원전: 미국 내 대형 원전 8기 건설 협의 및 가덕도 신공항 이슈로 건설 및 기계·장비 섹터가 강한 순환매 흐름 형성.</t>
+          <t>건설 섹터는 미국 내 대형 원전 8기 건설 협의 소식에 힘입어 주간 7.86% 상승하며 강한 모멘텀을 보임.</t>
         </is>
       </c>
     </row>
@@ -4278,7 +4278,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>소비재·IT서비스: 환율 하락에 따른 수출 우려와 차익 실현 매물로 음식료 및 IT 서비스 섹터는 약세 전환.</t>
+          <t>반면 음식료·담배 및 부동산 섹터는 환율 하락과 고금리 장기화 부담으로 인해 차익 실현 매물이 출회되며 약세를 면치 못함.</t>
         </is>
       </c>
     </row>
@@ -4302,7 +4302,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>KOSPI 4.61% 급등, 외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입.</t>
+          <t>미국 8월 비농업 고용지수 예상치 상회 및 필라델피아 반도체 지수 급등에 따른 국내 반도체 중심의 강세.</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>KOSPI 0.58% 하락, 2분기 GDP 성장률 0.6% 발표에 따른 경기 둔화 우려 부각.</t>
+          <t>국내 2분기 GDP 성장률 0.6%로 둔화 및 미국 금리 인상 우려 부각에 따른 지수 조정.</t>
         </is>
       </c>
     </row>
@@ -4730,7 +4730,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>반도체 수급이 지속되고 미국 물가 지표가 안정적이면 지수 반등 시도</t>
+          <t>반도체 대형주 수급 유지 시 지수 하단 지지</t>
         </is>
       </c>
     </row>
@@ -4742,7 +4742,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>미국 물가 지표가 예상치를 상회하여 금리 인상 우려가 재점화되면 지수 조정</t>
+          <t>미국 물가 지표 충격 시 금리 인상 우려 재점화</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>9월 10일 생산자물가지수(PPI)와 11일 소비자물가지수(CPI) 결과</t>
+          <t>미국 CPI 및 PPI 발표 결과</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>미국 생산자물가지수(PPI)</t>
+          <t>미국 소비자물가지수(CPI)</t>
         </is>
       </c>
     </row>
@@ -4778,7 +4778,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>미국 소비자물가지수(CPI)</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
@@ -4790,7 +4790,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>한국 무역수지</t>
+          <t>국내 무역수지</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-09-09 00:15Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -747,7 +747,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J106"/>
+  <dimension ref="A1:J103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12.9" customWidth="1" style="15" min="1" max="1"/>
@@ -787,7 +787,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-09 08:48 KST</t>
+          <t>2026-09-09 09:14 KST</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="C4" s="27" t="inlineStr">
         <is>
-          <t>반도체와 원전이 주도한 급등 랠리와 고금리 경계감의 공존</t>
+          <t>AI 반도체와 원전 모멘텀이 이끈 주간 상승세</t>
         </is>
       </c>
     </row>
@@ -896,13 +896,13 @@
         </is>
       </c>
       <c r="B8" s="28" t="n">
-        <v>-98706</v>
+        <v>-98067</v>
       </c>
       <c r="C8" s="29" t="n">
-        <v>31848</v>
+        <v>31154</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>32918</v>
+        <v>32584</v>
       </c>
       <c r="E8" s="28" t="n">
         <v>-1.34</v>
@@ -927,13 +927,13 @@
         </is>
       </c>
       <c r="B9" s="29" t="n">
-        <v>3387</v>
-      </c>
-      <c r="C9" s="28" t="n">
-        <v>-99</v>
+        <v>2870</v>
+      </c>
+      <c r="C9" s="29" t="n">
+        <v>542</v>
       </c>
       <c r="D9" s="28" t="n">
-        <v>-3471</v>
+        <v>-3583</v>
       </c>
     </row>
     <row r="10"/>
@@ -1011,17 +1011,17 @@
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>건설 +7.86%</t>
+          <t>건설 +12.14%</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>기계·장비 +7.43%</t>
+          <t>기계·장비 +11.19%</t>
         </is>
       </c>
       <c r="D14" s="30" t="inlineStr">
         <is>
-          <t>전기·전자 +5.93%</t>
+          <t>전기·전자 +7.09%</t>
         </is>
       </c>
     </row>
@@ -1033,17 +1033,17 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>음식료·담배 -3.39%</t>
+          <t>음식료·담배 -3.69%</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>IT 서비스 -1.75%</t>
+          <t>IT 서비스 -2.18%</t>
         </is>
       </c>
       <c r="D15" s="30" t="inlineStr">
         <is>
-          <t>화학 -1.32%</t>
+          <t>섬유·의류 -1.91%</t>
         </is>
       </c>
     </row>
@@ -1342,7 +1342,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="44.5" customHeight="1" s="15">
+    <row r="27" ht="58" customHeight="1" s="15">
       <c r="A27" s="30" t="inlineStr">
         <is>
           <t>2026-09-07</t>
@@ -1371,11 +1371,11 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>미국 반도체 지수 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 경계감이 상단을 제한함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="44.5" customHeight="1" s="15">
+          <t>미국 반도체 지수 3.37% 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 경계감으로 지수 상단이 제한됨.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="58" customHeight="1" s="15">
       <c r="A28" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
@@ -1404,40 +1404,40 @@
       </c>
       <c r="G28" s="17" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담을 가중시키며 지수 하락을 유발함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="44.5" customHeight="1" s="15">
+          <t>미국 국채금리 급등과 금리 인상 우려에도 불구하고, 미국 내 대형 원전 8기 건설 협의 소식이 국내 건설 및 전기·가스 섹터의 강세를 견인함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="58" customHeight="1" s="15">
       <c r="A29" s="30" t="inlineStr">
         <is>
           <t>2026-09-09</t>
         </is>
       </c>
-      <c r="B29" s="30" t="n">
-        <v>0</v>
+      <c r="B29" s="29" t="n">
+        <v>0.79</v>
       </c>
       <c r="C29" s="30" t="inlineStr">
         <is>
-          <t>데이터 없음</t>
-        </is>
-      </c>
-      <c r="D29" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="30" t="inlineStr">
-        <is>
-          <t>데이터 없음</t>
+          <t>436▲/370▼</t>
+        </is>
+      </c>
+      <c r="D29" s="29" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>987▲/561▼ 상한3</t>
         </is>
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>건설, 기계·장비</t>
         </is>
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
-          <t>미국 고용지표 '블로우아웃'에 따른 금리 인상 우려와 중동 지정학적 리스크가 겹치며 시장의 관망세가 짙어짐.</t>
+          <t>미국 고용지표 '블로우아웃'에 따른 금리 인상 우려에도 불구하고, 해외 원전 및 AIDC 수주 기대감이 건설·기계 섹터의 상승을 주도함.</t>
         </is>
       </c>
     </row>
@@ -1477,21 +1477,21 @@
     <row r="33" ht="31" customHeight="1" s="15">
       <c r="A33" s="17" t="inlineStr">
         <is>
-          <t>- 매크로 환경: 미국 비농업고용지수(162K)가 예상치(55K)를 상회하며 고용 호조를 보였으나, 국내 2분기 GDP 성장률(0.6%)은 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>- 매크로 환경은 미국 비농업고용지수가 162K로 예상치를 상회하며 금리 인상 우려를 자극했고, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 공존함.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="31" customHeight="1" s="15">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>- 수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되며 주도권을 형성했으나, 개인은 전 섹터에서 차익 실현 매물을 출회함.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="15">
+          <t>- 수급 구도는 전기·전자 섹터에 외국인 31,234억, 기관 25,529억이 집중되었고, 기계·장비 섹터에도 기관 2,795억이 유입되며 주도 섹터로 자리 잡음.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="31" customHeight="1" s="15">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>- 종합 관점: 반도체와 원전 중심의 수급 쏠림이 뚜렷한 가운데, 매크로 불확실성 확대가 지수 변동성을 키우는 국면임.</t>
+          <t>- 종합적으로 매크로 불확실성에도 불구하고 AI 반도체와 원전이라는 확실한 모멘텀이 수급을 견인하며 시장의 하방을 지지하는 국면임.</t>
         </is>
       </c>
     </row>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>주간 주가 상승률 7.86% 대비 기관 순매수 1,732억이 유입되며 수급 개선세 확인.</t>
+          <t>주간 12.14% 상승하며 기관이 1,743억 순매수함.</t>
         </is>
       </c>
     </row>
@@ -2360,7 +2360,7 @@
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
-          <t>주간 주가 상승률 7.43%와 함께 외국인 528억, 기관 2,736억의 동반 매수세 유입.</t>
+          <t>주간 11.19% 상승하며 기관이 2,795억 순매수함.</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2377,7 @@
       </c>
       <c r="C64" s="17" t="inlineStr">
         <is>
-          <t>주간 주가 하락률 -3.39%에도 불구하고 개인 순매수 1,233억이 집중되어 수급 부담 존재.</t>
+          <t>주간 3.69% 하락하며 기관이 1,083억 순매도함.</t>
         </is>
       </c>
     </row>
@@ -2394,7 +2394,7 @@
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
-          <t>주간 주가 하락률 -1.75%와 함께 기관 순매도 -233억이 지속되며 하방 압력 확인.</t>
+          <t>주간 2.18% 하락하며 기관이 250억 순매도함.</t>
         </is>
       </c>
     </row>
@@ -2434,102 +2434,127 @@
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" s="17" t="inlineStr">
         <is>
-          <t>- KOSPI는 외국인과 기관의 강력한 동반 매수세에 힘입어 주 초반 4.61% 급등하며 강한 상승세를 보임.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="31" customHeight="1" s="15">
+          <t>- 주 초반 미국 반도체 지수 급등에 힘입어 KOSPI가 4.61% 급등하며 7000선에 근접함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="15" customHeight="1" s="15">
       <c r="A70" s="17" t="inlineStr">
         <is>
-          <t>- 미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 상승이 시장 상단을 제한하며 주 후반 지수 하락 및 보합세로 전환.</t>
+          <t>- 미국 고용지표 호조에 따른 금리 인상 우려가 부각되며 주 중반 지수 조정이 발생함.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="15">
       <c r="A71" s="17" t="inlineStr">
         <is>
-          <t>- 반도체와 원전·전력설비 관련주로 수급 쏠림 현상이 뚜렷하게 나타남.</t>
+          <t>- 원전 및 데이터센터 전력 수요 관련 수주 기대감이 건설·기계 섹터의 강세를 견인함.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="15">
       <c r="A72" s="17" t="inlineStr">
         <is>
-          <t>- 개인은 주간 내내 차익 실현 매물을 쏟아내며 지수 하락 압박 요인으로 작용.</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="15" customHeight="1" s="15">
-      <c r="A73" s="17" t="inlineStr">
-        <is>
-          <t>- 중동 지정학적 리스크와 글로벌 경기 둔화 우려가 혼재되며 시장의 관망세가 짙어짐.</t>
-        </is>
-      </c>
-    </row>
-    <row r="74"/>
-    <row r="75">
-      <c r="A75" s="2" t="inlineStr">
+          <t>- 외국인과 기관은 전기·전자 섹터에 각각 31,234억, 25,529억을 순매수하며 수급을 주도함.</t>
+        </is>
+      </c>
+    </row>
+    <row r="73"/>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
         <is>
           <t>09</t>
         </is>
       </c>
-      <c r="B75" s="3" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>섹터·테마 흐름</t>
         </is>
       </c>
-      <c r="C75" s="3" t="inlineStr"/>
-      <c r="D75" s="3" t="inlineStr"/>
-      <c r="E75" s="3" t="inlineStr"/>
-      <c r="F75" s="3" t="inlineStr"/>
-      <c r="G75" s="3" t="inlineStr"/>
-      <c r="H75" s="3" t="inlineStr"/>
-      <c r="I75" s="3" t="inlineStr"/>
-      <c r="J75" s="3" t="inlineStr"/>
+      <c r="C74" s="3" t="inlineStr"/>
+      <c r="D74" s="3" t="inlineStr"/>
+      <c r="E74" s="3" t="inlineStr"/>
+      <c r="F74" s="3" t="inlineStr"/>
+      <c r="G74" s="3" t="inlineStr"/>
+      <c r="H74" s="3" t="inlineStr"/>
+      <c r="I74" s="3" t="inlineStr"/>
+      <c r="J74" s="3" t="inlineStr"/>
+    </row>
+    <row r="75" ht="15" customHeight="1" s="15">
+      <c r="A75" s="17" t="inlineStr">
+        <is>
+          <t>- 전기·전자: AI 반도체 수요 기대감으로 주간 7.09% 상승하며 수급 집중.</t>
+        </is>
+      </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="15">
       <c r="A76" s="17" t="inlineStr">
         <is>
-          <t>- 반도체/AI: 삼성전자, SK하이닉스 중심의 외국인·기관 매수세가 지속되며 시장 주도.</t>
+          <t>- 건설/기계·장비: 원전 및 데이터센터 수주 기대감으로 각각 12.14%, 11.19% 상승하며 주도 섹터로 부상.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="15">
       <c r="A77" s="17" t="inlineStr">
         <is>
-          <t>- 원전/전력설비: 대형 수주 기대감으로 기계·장비 및 건설 섹터가 급등하며 순환매 주도.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="15" customHeight="1" s="15">
-      <c r="A78" s="17" t="inlineStr">
-        <is>
-          <t>- 음식료/소비재: 글로벌 소비 둔화 우려 및 환율 영향으로 약세 전환.</t>
-        </is>
-      </c>
-    </row>
-    <row r="79"/>
+          <t>- 음식료/보험: 규제 및 실적 우려로 각각 3.69%, 0.37% 하락하며 약세 지속.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78"/>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="inlineStr">
+        <is>
+          <t>주간 촉매 타임라인</t>
+        </is>
+      </c>
+      <c r="C79" s="3" t="inlineStr"/>
+      <c r="D79" s="3" t="inlineStr"/>
+      <c r="E79" s="3" t="inlineStr"/>
+      <c r="F79" s="3" t="inlineStr"/>
+      <c r="G79" s="3" t="inlineStr"/>
+      <c r="H79" s="3" t="inlineStr"/>
+      <c r="I79" s="3" t="inlineStr"/>
+      <c r="J79" s="18" t="inlineStr">
+        <is>
+          <t>등락률 = 주간 누적</t>
+        </is>
+      </c>
+    </row>
     <row r="80">
-      <c r="A80" s="2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="B80" s="3" t="inlineStr">
-        <is>
-          <t>주간 촉매 타임라인</t>
-        </is>
-      </c>
-      <c r="C80" s="3" t="inlineStr"/>
-      <c r="D80" s="3" t="inlineStr"/>
-      <c r="E80" s="3" t="inlineStr"/>
-      <c r="F80" s="3" t="inlineStr"/>
-      <c r="G80" s="3" t="inlineStr"/>
-      <c r="H80" s="3" t="inlineStr"/>
-      <c r="I80" s="3" t="inlineStr"/>
-      <c r="J80" s="18" t="inlineStr">
-        <is>
-          <t>등락률 = 주간 누적</t>
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>날짜</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>종목</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>별점</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>등락률(%)</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
+        <is>
+          <t>핵심 촉매</t>
         </is>
       </c>
     </row>
@@ -2539,17 +2564,27 @@
           <t>2026-09-07</t>
         </is>
       </c>
-      <c r="B81" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C81" s="30" t="inlineStr"/>
-      <c r="D81" s="14" t="inlineStr"/>
-      <c r="E81" s="29" t="inlineStr"/>
+      <c r="B81" s="17" t="inlineStr">
+        <is>
+          <t>네오오토 (운송장비·부품)</t>
+        </is>
+      </c>
+      <c r="C81" s="30" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="E81" s="29" t="n">
+        <v>40.59</v>
+      </c>
       <c r="F81" s="17" t="inlineStr">
         <is>
-          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
+          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
         </is>
       </c>
     </row>
@@ -2561,7 +2596,7 @@
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>네오오토 (운송장비·부품)</t>
+          <t>필옵틱스 (기계·장비)</t>
         </is>
       </c>
       <c r="C82" s="30" t="inlineStr">
@@ -2575,11 +2610,11 @@
         </is>
       </c>
       <c r="E82" s="29" t="n">
-        <v>40.59</v>
+        <v>37.21</v>
       </c>
       <c r="F82" s="17" t="inlineStr">
         <is>
-          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
+          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
         </is>
       </c>
     </row>
@@ -2591,7 +2626,7 @@
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>필옵틱스 (기계·장비)</t>
+          <t>나무가 (전기·전자)</t>
         </is>
       </c>
       <c r="C83" s="30" t="inlineStr">
@@ -2605,11 +2640,11 @@
         </is>
       </c>
       <c r="E83" s="29" t="n">
-        <v>37.21</v>
+        <v>10.23</v>
       </c>
       <c r="F83" s="17" t="inlineStr">
         <is>
-          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
+          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -2621,12 +2656,12 @@
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>나무가 (전기·전자)</t>
+          <t>두산퓨얼셀 (전기·전자)</t>
         </is>
       </c>
       <c r="C84" s="30" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D84" s="14" t="inlineStr">
@@ -2635,11 +2670,11 @@
         </is>
       </c>
       <c r="E84" s="29" t="n">
-        <v>10.23</v>
+        <v>12.31</v>
       </c>
       <c r="F84" s="17" t="inlineStr">
         <is>
-          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
+          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -2651,7 +2686,7 @@
       </c>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>두산퓨얼셀 (전기·전자)</t>
+          <t>DB하이텍 (전기·전자)</t>
         </is>
       </c>
       <c r="C85" s="30" t="inlineStr">
@@ -2661,15 +2696,15 @@
       </c>
       <c r="D85" s="14" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="E85" s="29" t="n">
-        <v>12.31</v>
+        <v>15.02</v>
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
-          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
+          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
         </is>
       </c>
     </row>
@@ -2681,7 +2716,7 @@
       </c>
       <c r="B86" s="17" t="inlineStr">
         <is>
-          <t>DB하이텍 (전기·전자)</t>
+          <t>두산에너빌리티 (기계·장비)</t>
         </is>
       </c>
       <c r="C86" s="30" t="inlineStr">
@@ -2695,11 +2730,11 @@
         </is>
       </c>
       <c r="E86" s="29" t="n">
-        <v>15.02</v>
+        <v>13.01</v>
       </c>
       <c r="F86" s="17" t="inlineStr">
         <is>
-          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
+          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
         </is>
       </c>
     </row>
@@ -2711,7 +2746,7 @@
       </c>
       <c r="B87" s="17" t="inlineStr">
         <is>
-          <t>두산에너빌리티 (기계·장비)</t>
+          <t>SK하이닉스 (전기·전자)</t>
         </is>
       </c>
       <c r="C87" s="30" t="inlineStr">
@@ -2725,11 +2760,11 @@
         </is>
       </c>
       <c r="E87" s="29" t="n">
-        <v>13.01</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F87" s="17" t="inlineStr">
         <is>
-          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
+          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2776,7 @@
       </c>
       <c r="B88" s="17" t="inlineStr">
         <is>
-          <t>SK하이닉스 (전기·전자)</t>
+          <t>삼성전자 (전기·전자)</t>
         </is>
       </c>
       <c r="C88" s="30" t="inlineStr">
@@ -2755,41 +2790,41 @@
         </is>
       </c>
       <c r="E88" s="29" t="n">
-        <v>8.859999999999999</v>
+        <v>5.48</v>
       </c>
       <c r="F88" s="17" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
+          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="31" customHeight="1" s="15">
       <c r="A89" s="30" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B89" s="17" t="inlineStr">
         <is>
-          <t>삼성전자 (전기·전자)</t>
+          <t>빛과전자 (전기·전자)</t>
         </is>
       </c>
       <c r="C89" s="30" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D89" s="14" t="inlineStr">
         <is>
-          <t>★★★★</t>
+          <t>★★★★★</t>
         </is>
       </c>
       <c r="E89" s="29" t="n">
-        <v>5.48</v>
+        <v>34.07</v>
       </c>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
+          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
         </is>
       </c>
     </row>
@@ -2799,17 +2834,27 @@
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B90" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C90" s="30" t="inlineStr"/>
-      <c r="D90" s="14" t="inlineStr"/>
-      <c r="E90" s="29" t="inlineStr"/>
+      <c r="B90" s="17" t="inlineStr">
+        <is>
+          <t>오르비텍 (일반서비스)</t>
+        </is>
+      </c>
+      <c r="C90" s="30" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D90" s="14" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="E90" s="29" t="n">
+        <v>39.88</v>
+      </c>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>미국 국채금리 상승 및 국내 2분기 GDP 성장률(0.6%) 둔화로 지수 0.58% 하락.</t>
+          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -2821,7 +2866,7 @@
       </c>
       <c r="B91" s="17" t="inlineStr">
         <is>
-          <t>빛과전자 (전기·전자)</t>
+          <t>서전기전 (전기·전자)</t>
         </is>
       </c>
       <c r="C91" s="30" t="inlineStr">
@@ -2835,28 +2880,28 @@
         </is>
       </c>
       <c r="E91" s="29" t="n">
-        <v>34.07</v>
+        <v>37.07</v>
       </c>
       <c r="F91" s="17" t="inlineStr">
         <is>
-          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15" customHeight="1" s="15">
+          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="31" customHeight="1" s="15">
       <c r="A92" s="30" t="inlineStr">
         <is>
           <t>2026-09-08</t>
         </is>
       </c>
-      <c r="B92" s="30" t="inlineStr">
-        <is>
-          <t>오르비텍</t>
+      <c r="B92" s="17" t="inlineStr">
+        <is>
+          <t>한전기술 (일반서비스)</t>
         </is>
       </c>
       <c r="C92" s="30" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D92" s="14" t="inlineStr">
@@ -2865,11 +2910,11 @@
         </is>
       </c>
       <c r="E92" s="29" t="n">
-        <v>39.88</v>
+        <v>32.53</v>
       </c>
       <c r="F92" s="17" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
+          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -2881,25 +2926,25 @@
       </c>
       <c r="B93" s="17" t="inlineStr">
         <is>
-          <t>서전기전 (전기·전자)</t>
+          <t>현대약품 (제약)</t>
         </is>
       </c>
       <c r="C93" s="30" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D93" s="14" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="E93" s="29" t="n">
-        <v>37.07</v>
+        <v>31.32</v>
       </c>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
         </is>
       </c>
     </row>
@@ -2911,7 +2956,7 @@
       </c>
       <c r="B94" s="17" t="inlineStr">
         <is>
-          <t>한전기술 (일반서비스)</t>
+          <t>대우건설 (건설)</t>
         </is>
       </c>
       <c r="C94" s="30" t="inlineStr">
@@ -2921,205 +2966,126 @@
       </c>
       <c r="D94" s="14" t="inlineStr">
         <is>
-          <t>★★★★★</t>
+          <t>★★★★</t>
         </is>
       </c>
       <c r="E94" s="29" t="n">
-        <v>32.53</v>
+        <v>18.52</v>
       </c>
       <c r="F94" s="17" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="31" customHeight="1" s="15">
-      <c r="A95" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B95" s="17" t="inlineStr">
-        <is>
-          <t>현대약품 (제약)</t>
-        </is>
-      </c>
-      <c r="C95" s="30" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
-        <is>
-          <t>★★★★</t>
-        </is>
-      </c>
-      <c r="E95" s="29" t="n">
-        <v>31.32</v>
-      </c>
-      <c r="F95" s="17" t="inlineStr">
-        <is>
-          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="31" customHeight="1" s="15">
-      <c r="A96" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B96" s="17" t="inlineStr">
-        <is>
-          <t>대우건설 (건설)</t>
-        </is>
-      </c>
-      <c r="C96" s="30" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
-        <is>
-          <t>★★★★</t>
-        </is>
-      </c>
-      <c r="E96" s="29" t="n">
-        <v>18.52</v>
-      </c>
-      <c r="F96" s="17" t="inlineStr">
-        <is>
           <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
         </is>
       </c>
     </row>
-    <row r="97" ht="31" customHeight="1" s="15">
-      <c r="A97" s="30" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B97" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C97" s="30" t="inlineStr"/>
-      <c r="D97" s="14" t="inlineStr"/>
-      <c r="E97" s="29" t="inlineStr"/>
-      <c r="F97" s="17" t="inlineStr">
-        <is>
-          <t>미국 고용지표 호조에 따른 금리 인상 우려와 중동 지정학적 리스크로 관망세 지속.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98"/>
-    <row r="99">
-      <c r="A99" s="2" t="inlineStr">
+    <row r="95"/>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B99" s="3" t="inlineStr">
+      <c r="B96" s="3" t="inlineStr">
         <is>
           <t>다음 주 프리뷰</t>
         </is>
       </c>
-      <c r="C99" s="3" t="inlineStr"/>
-      <c r="D99" s="3" t="inlineStr"/>
-      <c r="E99" s="3" t="inlineStr"/>
-      <c r="F99" s="3" t="inlineStr"/>
-      <c r="G99" s="3" t="inlineStr"/>
-      <c r="H99" s="3" t="inlineStr"/>
-      <c r="I99" s="3" t="inlineStr"/>
-      <c r="J99" s="3" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="4" t="inlineStr">
+      <c r="C96" s="3" t="inlineStr"/>
+      <c r="D96" s="3" t="inlineStr"/>
+      <c r="E96" s="3" t="inlineStr"/>
+      <c r="F96" s="3" t="inlineStr"/>
+      <c r="G96" s="3" t="inlineStr"/>
+      <c r="H96" s="3" t="inlineStr"/>
+      <c r="I96" s="3" t="inlineStr"/>
+      <c r="J96" s="3" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="4" t="inlineStr">
         <is>
           <t>구분</t>
         </is>
       </c>
-      <c r="B100" s="4" t="inlineStr">
+      <c r="B97" s="4" t="inlineStr">
         <is>
           <t>내용</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="31" customHeight="1" s="15">
-      <c r="A101" s="31" t="inlineStr">
+    <row r="98" ht="31" customHeight="1" s="15">
+      <c r="A98" s="31" t="inlineStr">
         <is>
           <t>상승 시나리오</t>
         </is>
       </c>
+      <c r="B98" s="17" t="inlineStr">
+        <is>
+          <t>미국 물가 지표가 안정적으로 확인되면 반도체 및 원전 주도 상승세 지속.</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="31" customHeight="1" s="15">
+      <c r="A99" s="32" t="inlineStr">
+        <is>
+          <t>하방 시나리오</t>
+        </is>
+      </c>
+      <c r="B99" s="17" t="inlineStr">
+        <is>
+          <t>물가 지표가 예상치를 상회하여 금리 인상 우려가 재점화될 경우 조정.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15" customHeight="1" s="15">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>판별 신호</t>
+        </is>
+      </c>
+      <c r="B100" s="17" t="inlineStr">
+        <is>
+          <t>9월 11일 발표되는 미국 소비자물가지수(CPI) 결과가 시장 방향성을 결정할 것.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15" customHeight="1" s="15">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>핵심 이벤트</t>
+        </is>
+      </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>미국 CPI가 예상치를 하회하면 금리 인상 우려 완화로 반도체 중심 상승세 재개</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="31" customHeight="1" s="15">
-      <c r="A102" s="32" t="inlineStr">
-        <is>
-          <t>하방 시나리오</t>
+          <t>미국 소비자물가지수(CPI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15" customHeight="1" s="15">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B102" s="17" t="inlineStr">
         <is>
-          <t>미국 CPI가 예상치를 상회하면 고금리 장기화 우려로 외국인 수급 이탈 및 지수 조정</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="15">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>판별 신호</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B103" s="17" t="inlineStr">
         <is>
-          <t>9월 11일 발표되는 미국 소비자물가지수(CPI)의 전월 대비 상승률 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="15" customHeight="1" s="15">
-      <c r="A104" s="3" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B104" s="17" t="inlineStr">
-        <is>
-          <t>미국 소비자물가지수(CPI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="15" customHeight="1" s="15">
-      <c r="A105" s="3" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B105" s="17" t="inlineStr">
-        <is>
-          <t>한국 무역수지</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15" customHeight="1" s="15">
-      <c r="A106" s="3" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B106" s="17" t="inlineStr">
-        <is>
-          <t>미국 소매판매</t>
+          <t>국내 무역수지</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="51">
+  <mergeCells count="48">
+    <mergeCell ref="B98:J98"/>
     <mergeCell ref="A1:G2"/>
     <mergeCell ref="G26:J26"/>
     <mergeCell ref="F87:J87"/>
@@ -3135,39 +3101,35 @@
     <mergeCell ref="C64:J64"/>
     <mergeCell ref="F83:J83"/>
     <mergeCell ref="B103:J103"/>
-    <mergeCell ref="F95:J95"/>
+    <mergeCell ref="B99:J99"/>
     <mergeCell ref="C63:J63"/>
     <mergeCell ref="C65:J65"/>
     <mergeCell ref="F86:J86"/>
     <mergeCell ref="A77:J77"/>
     <mergeCell ref="A34:J34"/>
+    <mergeCell ref="F80:J80"/>
     <mergeCell ref="F94:J94"/>
-    <mergeCell ref="A73:J73"/>
     <mergeCell ref="F85:J85"/>
     <mergeCell ref="G27:J27"/>
     <mergeCell ref="B68:J68"/>
-    <mergeCell ref="F97:J97"/>
-    <mergeCell ref="B104:J104"/>
     <mergeCell ref="F91:J91"/>
     <mergeCell ref="A70:J70"/>
     <mergeCell ref="F81:J81"/>
     <mergeCell ref="B32:J32"/>
-    <mergeCell ref="A78:J78"/>
     <mergeCell ref="F90:J90"/>
     <mergeCell ref="A69:J69"/>
-    <mergeCell ref="B106:J106"/>
     <mergeCell ref="F93:J93"/>
     <mergeCell ref="C61:J61"/>
+    <mergeCell ref="B97:J97"/>
     <mergeCell ref="I1:J1"/>
-    <mergeCell ref="F96:J96"/>
+    <mergeCell ref="B100:J100"/>
     <mergeCell ref="G28:J28"/>
     <mergeCell ref="A4:B4"/>
-    <mergeCell ref="B100:J100"/>
+    <mergeCell ref="A75:J75"/>
     <mergeCell ref="F92:J92"/>
     <mergeCell ref="A71:J71"/>
     <mergeCell ref="F82:J82"/>
     <mergeCell ref="B102:J102"/>
-    <mergeCell ref="B105:J105"/>
     <mergeCell ref="A76:J76"/>
     <mergeCell ref="A33:J33"/>
     <mergeCell ref="F88:J88"/>
@@ -3182,7 +3144,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J93"/>
+  <dimension ref="A1:J89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5" outlineLevelCol="0"/>
   <cols>
     <col width="30.85546875" customWidth="1" style="15" min="1" max="1"/>
@@ -3214,7 +3176,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-09 08:48 KST</t>
+          <t>2026-09-09 09:14 KST</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3188,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>반도체와 원전이 주도한 급등 랠리와 고금리 경계감의 공존</t>
+          <t>AI 반도체와 원전 모멘텀이 이끈 주간 상승세</t>
         </is>
       </c>
     </row>
@@ -3266,13 +3228,13 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>-98706</v>
+        <v>-98067</v>
       </c>
       <c r="C7" t="n">
-        <v>31848</v>
+        <v>31154</v>
       </c>
       <c r="D7" t="n">
-        <v>32918</v>
+        <v>32584</v>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1" s="15">
@@ -3282,13 +3244,13 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3387</v>
+        <v>2870</v>
       </c>
       <c r="C8" t="n">
-        <v>-99</v>
+        <v>542</v>
       </c>
       <c r="D8" t="n">
-        <v>-3471</v>
+        <v>-3583</v>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1" s="15">
@@ -3495,7 +3457,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>미국 반도체 지수 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 경계감이 상단을 제한함.</t>
+          <t>미국 반도체 지수 3.37% 급등이 국내 반도체 소부장 강세로 이어졌으나, 고용지표 호조에 따른 금리 인하 경계감으로 지수 상단이 제한됨.</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3472,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>미국 국채금리 급등과 연준의 금리 인상 우려가 국내 증시의 밸류에이션 부담을 가중시키며 지수 하락을 유발함.</t>
+          <t>미국 국채금리 급등과 금리 인상 우려에도 불구하고, 미국 내 대형 원전 8기 건설 협의 소식이 국내 건설 및 전기·가스 섹터의 강세를 견인함.</t>
         </is>
       </c>
     </row>
@@ -3521,11 +3483,11 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0</v>
+        <v>0.79</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>미국 고용지표 '블로우아웃'에 따른 금리 인상 우려와 중동 지정학적 리스크가 겹치며 시장의 관망세가 짙어짐.</t>
+          <t>미국 고용지표 '블로우아웃'에 따른 금리 인상 우려에도 불구하고, 해외 원전 및 AIDC 수주 기대감이 건설·기계 섹터의 상승을 주도함.</t>
         </is>
       </c>
     </row>
@@ -3544,7 +3506,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>매크로 환경: 미국 비농업고용지수(162K)가 예상치(55K)를 상회하며 고용 호조를 보였으나, 국내 2분기 GDP 성장률(0.6%)은 이전치(1.8%)를 하회하며 경기 둔화 우려가 부각됨.</t>
+          <t>매크로 환경은 미국 비농업고용지수가 162K로 예상치를 상회하며 금리 인상 우려를 자극했고, 국내 2분기 GDP 성장률은 0.6%로 이전치(1.8%)를 하회하며 경기 둔화 우려가 공존함.</t>
         </is>
       </c>
     </row>
@@ -3556,7 +3518,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>수급 구도: 전기·전자 섹터에 외국인(32,305억)과 기관(25,821억)의 매수세가 집중되며 주도권을 형성했으나, 개인은 전 섹터에서 차익 실현 매물을 출회함.</t>
+          <t>수급 구도는 전기·전자 섹터에 외국인 31,234억, 기관 25,529억이 집중되었고, 기계·장비 섹터에도 기관 2,795억이 유입되며 주도 섹터로 자리 잡음.</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3530,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>종합 관점: 반도체와 원전 중심의 수급 쏠림이 뚜렷한 가운데, 매크로 불확실성 확대가 지수 변동성을 키우는 국면임.</t>
+          <t>종합적으로 매크로 불확실성에도 불구하고 AI 반도체와 원전이라는 확실한 모멘텀이 수급을 견인하며 시장의 하방을 지지하는 국면임.</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4281,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>주간 주가 상승률 7.86% 대비 기관 순매수 1,732억이 유입되며 수급 개선세 확인.</t>
+          <t>주간 12.14% 상승하며 기관이 1,743억 순매수함.</t>
         </is>
       </c>
     </row>
@@ -4336,7 +4298,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>주간 주가 상승률 7.43%와 함께 외국인 528억, 기관 2,736억의 동반 매수세 유입.</t>
+          <t>주간 11.19% 상승하며 기관이 2,795억 순매수함.</t>
         </is>
       </c>
     </row>
@@ -4353,7 +4315,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>주간 주가 하락률 -3.39%에도 불구하고 개인 순매수 1,233억이 집중되어 수급 부담 존재.</t>
+          <t>주간 3.69% 하락하며 기관이 1,083억 순매도함.</t>
         </is>
       </c>
     </row>
@@ -4370,7 +4332,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>주간 주가 하락률 -1.75%와 함께 기관 순매도 -233억이 지속되며 하방 압력 확인.</t>
+          <t>주간 2.18% 하락하며 기관이 250억 순매도함.</t>
         </is>
       </c>
     </row>
@@ -4389,7 +4351,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KOSPI는 외국인과 기관의 강력한 동반 매수세에 힘입어 주 초반 4.61% 급등하며 강한 상승세를 보임.</t>
+          <t>주 초반 미국 반도체 지수 급등에 힘입어 KOSPI가 4.61% 급등하며 7000선에 근접함.</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4363,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>미국 고용지표 호조에 따른 금리 인하 기대감 후퇴와 국채 금리 상승이 시장 상단을 제한하며 주 후반 지수 하락 및 보합세로 전환.</t>
+          <t>미국 고용지표 호조에 따른 금리 인상 우려가 부각되며 주 중반 지수 조정이 발생함.</t>
         </is>
       </c>
     </row>
@@ -4413,7 +4375,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>반도체와 원전·전력설비 관련주로 수급 쏠림 현상이 뚜렷하게 나타남.</t>
+          <t>원전 및 데이터센터 전력 수요 관련 수주 기대감이 건설·기계 섹터의 강세를 견인함.</t>
         </is>
       </c>
     </row>
@@ -4425,26 +4387,26 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>개인은 주간 내내 차익 실현 매물을 쏟아내며 지수 하락 압박 요인으로 작용.</t>
+          <t>외국인과 기관은 전기·전자 섹터에 각각 31,234억, 25,529억을 순매수하며 수급을 주도함.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="15">
       <c r="A64" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>중동 지정학적 리스크와 글로벌 경기 둔화 우려가 혼재되며 시장의 관망세가 짙어짐.</t>
+          <t>9. 섹터·테마 흐름</t>
         </is>
       </c>
     </row>
     <row r="65" ht="15" customHeight="1" s="15">
       <c r="A65" t="inlineStr">
         <is>
-          <t>9. 섹터·테마 흐름</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>전기·전자: AI 반도체 수요 기대감으로 주간 7.09% 상승하며 수급 집중.</t>
         </is>
       </c>
     </row>
@@ -4456,7 +4418,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>반도체/AI: 삼성전자, SK하이닉스 중심의 외국인·기관 매수세가 지속되며 시장 주도.</t>
+          <t>건설/기계·장비: 원전 및 데이터센터 수주 기대감으로 각각 12.14%, 11.19% 상승하며 주도 섹터로 부상.</t>
         </is>
       </c>
     </row>
@@ -4468,26 +4430,42 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>원전/전력설비: 대형 수주 기대감으로 기계·장비 및 건설 섹터가 급등하며 순환매 주도.</t>
+          <t>음식료/보험: 규제 및 실적 우려로 각각 3.69%, 0.37% 하락하며 약세 지속.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>음식료/소비재: 글로벌 소비 둔화 우려 및 환율 영향으로 약세 전환.</t>
+          <t>10. 촉매 타임라인</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="15">
       <c r="A69" t="inlineStr">
         <is>
-          <t>10. 촉매 타임라인</t>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>네오오토</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>5</v>
+      </c>
+      <c r="E69" t="n">
+        <v>40.59</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4477,23 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>필옵틱스</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>5</v>
+      </c>
+      <c r="E70" t="n">
+        <v>37.21</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>외국인(+25,532억)과 기관(+26,491억)의 강력한 동반 매수세 유입으로 KOSPI 4.61% 급등.</t>
+          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
         </is>
       </c>
     </row>
@@ -4516,7 +4505,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>네오오토</t>
+          <t>나무가</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -4528,11 +4517,11 @@
         <v>5</v>
       </c>
       <c r="E71" t="n">
-        <v>40.59</v>
+        <v>10.23</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>계열사 오토인더스트리를 완전 자회사로 편입한다는 결정에 상한가 기록.</t>
+          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -4544,23 +4533,23 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>필옵틱스</t>
+          <t>두산퓨얼셀</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>5</v>
       </c>
       <c r="E72" t="n">
-        <v>37.21</v>
+        <v>12.31</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>차세대 반도체 패키지용 유리기판 실물 공개 및 해외 고객사 수주 가시화.</t>
+          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
         </is>
       </c>
     </row>
@@ -4572,23 +4561,23 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>나무가</t>
+          <t>DB하이텍</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E73" t="n">
-        <v>10.23</v>
+        <v>15.02</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>북미 휴머노이드 로봇 기업에 3D 카메라 모듈 단독 공급 계약 체결.</t>
+          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
         </is>
       </c>
     </row>
@@ -4600,7 +4589,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>두산퓨얼셀</t>
+          <t>두산에너빌리티</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -4609,14 +4598,14 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E74" t="n">
-        <v>12.31</v>
+        <v>13.01</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>미국 AI 데이터센터용 5,000억원대 대규모 연료전지 공급 계약 체결.</t>
+          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
         </is>
       </c>
     </row>
@@ -4628,7 +4617,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>DB하이텍</t>
+          <t>SK하이닉스</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4640,11 +4629,11 @@
         <v>4</v>
       </c>
       <c r="E75" t="n">
-        <v>15.02</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>차세대 전력반도체 양산 체제 구축 및 AI 모델 공개에 따른 파운드리 수혜 기대감.</t>
+          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
         </is>
       </c>
     </row>
@@ -4656,7 +4645,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>두산에너빌리티</t>
+          <t>삼성전자</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -4668,67 +4657,67 @@
         <v>4</v>
       </c>
       <c r="E76" t="n">
-        <v>13.01</v>
+        <v>5.48</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>원전 및 가스터빈 수주 기대감과 SMR 생산거점 육성 이슈 부각.</t>
+          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="15">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SK하이닉스</t>
+          <t>빛과전자</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E77" t="n">
-        <v>8.859999999999999</v>
+        <v>34.07</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 및 반도체 업황 회복 기대감에 따른 외국인·기관 매수세 유입.</t>
+          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="15">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>삼성전자</t>
+          <t>오르비텍</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>KOSPI</t>
+          <t>KOSDAQ</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E78" t="n">
-        <v>5.48</v>
+        <v>39.88</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>AI 메모리 수요 확대 기대감과 외국인·기관의 대규모 순매수세 유입.</t>
+          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -4740,12 +4729,23 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
+          <t>서전기전</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>KOSDAQ</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>5</v>
+      </c>
+      <c r="E79" t="n">
+        <v>37.07</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>미국 국채금리 상승 및 국내 2분기 GDP 성장률(0.6%) 둔화로 지수 0.58% 하락.</t>
+          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
         </is>
       </c>
     </row>
@@ -4757,23 +4757,23 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>빛과전자</t>
+          <t>한전기술</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D80" t="n">
         <v>5</v>
       </c>
       <c r="E80" t="n">
-        <v>34.07</v>
+        <v>32.53</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>차세대 광통신 부품 국산화 국책 사업 수행기관 선정.</t>
+          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
         </is>
       </c>
     </row>
@@ -4785,23 +4785,23 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>오르비텍</t>
+          <t>현대약품</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E81" t="n">
-        <v>39.88</v>
+        <v>31.32</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>미국 내 대형 원전 8기 건설 추진 기대감에 따른 수주 기대.</t>
+          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
         </is>
       </c>
     </row>
@@ -4813,206 +4813,108 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>서전기전</t>
+          <t>대우건설</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>KOSDAQ</t>
+          <t>KOSPI</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E82" t="n">
-        <v>37.07</v>
+        <v>18.52</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>한미 원전 협력 가시화 및 대미 투자 프로젝트 내 원전 건설 기대.</t>
+          <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="15">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>한전기술</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
-        <v>5</v>
-      </c>
-      <c r="E83" t="n">
-        <v>32.53</v>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>미국 내 대형 원전 8기 건설 협의 소식에 따른 수주 기대.</t>
+          <t>11. 다음 주 프리뷰</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="15">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>상승 시나리오</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>현대약품</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>4</v>
-      </c>
-      <c r="E84" t="n">
-        <v>31.32</v>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>임신중지약 미프진의 연내 출시 기대감 및 탈모 치료제 성장.</t>
+          <t>미국 물가 지표가 안정적으로 확인되면 반도체 및 원전 주도 상승세 지속.</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="15">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>하방 시나리오</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>대우건설</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>KOSPI</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>4</v>
-      </c>
-      <c r="E85" t="n">
-        <v>18.52</v>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>가덕도 신공항 기본설계 제출 및 미국 원전 건설 기대감.</t>
+          <t>물가 지표가 예상치를 상회하여 금리 인상 우려가 재점화될 경우 조정.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="15">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>판별 신호</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F86" t="inlineStr">
-        <is>
-          <t>미국 고용지표 호조에 따른 금리 인상 우려와 중동 지정학적 리스크로 관망세 지속.</t>
+          <t>9월 11일 발표되는 미국 소비자물가지수(CPI) 결과가 시장 방향성을 결정할 것.</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="15">
       <c r="A87" t="inlineStr">
         <is>
-          <t>11. 다음 주 프리뷰</t>
+          <t>핵심 이벤트</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>미국 소비자물가지수(CPI)</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="15">
       <c r="A88" t="inlineStr">
         <is>
-          <t>상승 시나리오</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>미국 CPI가 예상치를 하회하면 금리 인상 우려 완화로 반도체 중심 상승세 재개</t>
+          <t>미국 생산자물가지수(PPI)</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="15">
       <c r="A89" t="inlineStr">
         <is>
-          <t>하방 시나리오</t>
+          <t>핵심 이벤트</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>미국 CPI가 예상치를 상회하면 고금리 장기화 우려로 외국인 수급 이탈 및 지수 조정</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="15" customHeight="1" s="15">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>판별 신호</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>9월 11일 발표되는 미국 소비자물가지수(CPI)의 전월 대비 상승률 확인</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="15" customHeight="1" s="15">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>미국 소비자물가지수(CPI)</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>한국 무역수지</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="15" customHeight="1" s="15">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>핵심 이벤트</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>미국 소매판매</t>
-        </is>
-      </c>
-    </row>
+          <t>국내 무역수지</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="15" customHeight="1" s="15"/>
+    <row r="91" ht="15" customHeight="1" s="15"/>
+    <row r="93" ht="15" customHeight="1" s="15"/>
     <row r="94" ht="15" customHeight="1" s="15"/>
     <row r="95" ht="15" customHeight="1" s="15"/>
     <row r="96" ht="15" customHeight="1" s="15"/>

</xml_diff>

<commit_message>
chore: weekly briefing 2026-09-09 00:21Z [skip railway]
</commit_message>
<xml_diff>
--- a/public/reports/weekly_briefing/2026-09-07.xlsx
+++ b/public/reports/weekly_briefing/2026-09-07.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="I2" s="25" t="inlineStr">
         <is>
-          <t>2026-09-09 09:14 KST</t>
+          <t>2026-09-09 09:21 KST</t>
         </is>
       </c>
     </row>
@@ -2580,7 +2580,7 @@
         </is>
       </c>
       <c r="E81" s="29" t="n">
-        <v>40.59</v>
+        <v>40.81</v>
       </c>
       <c r="F81" s="17" t="inlineStr">
         <is>
@@ -2610,7 +2610,7 @@
         </is>
       </c>
       <c r="E82" s="29" t="n">
-        <v>37.21</v>
+        <v>37.02</v>
       </c>
       <c r="F82" s="17" t="inlineStr">
         <is>
@@ -2640,7 +2640,7 @@
         </is>
       </c>
       <c r="E83" s="29" t="n">
-        <v>10.23</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F83" s="17" t="inlineStr">
         <is>
@@ -2670,7 +2670,7 @@
         </is>
       </c>
       <c r="E84" s="29" t="n">
-        <v>12.31</v>
+        <v>19.5</v>
       </c>
       <c r="F84" s="17" t="inlineStr">
         <is>
@@ -2700,7 +2700,7 @@
         </is>
       </c>
       <c r="E85" s="29" t="n">
-        <v>15.02</v>
+        <v>24.36</v>
       </c>
       <c r="F85" s="17" t="inlineStr">
         <is>
@@ -2730,7 +2730,7 @@
         </is>
       </c>
       <c r="E86" s="29" t="n">
-        <v>13.01</v>
+        <v>16.16</v>
       </c>
       <c r="F86" s="17" t="inlineStr">
         <is>
@@ -2760,7 +2760,7 @@
         </is>
       </c>
       <c r="E87" s="29" t="n">
-        <v>8.859999999999999</v>
+        <v>10.14</v>
       </c>
       <c r="F87" s="17" t="inlineStr">
         <is>
@@ -2790,7 +2790,7 @@
         </is>
       </c>
       <c r="E88" s="29" t="n">
-        <v>5.48</v>
+        <v>5.58</v>
       </c>
       <c r="F88" s="17" t="inlineStr">
         <is>
@@ -2820,7 +2820,7 @@
         </is>
       </c>
       <c r="E89" s="29" t="n">
-        <v>34.07</v>
+        <v>42.17</v>
       </c>
       <c r="F89" s="17" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
         </is>
       </c>
       <c r="E90" s="29" t="n">
-        <v>39.88</v>
+        <v>43.82</v>
       </c>
       <c r="F90" s="17" t="inlineStr">
         <is>
@@ -2880,7 +2880,7 @@
         </is>
       </c>
       <c r="E91" s="29" t="n">
-        <v>37.07</v>
+        <v>35.64</v>
       </c>
       <c r="F91" s="17" t="inlineStr">
         <is>
@@ -2910,7 +2910,7 @@
         </is>
       </c>
       <c r="E92" s="29" t="n">
-        <v>32.53</v>
+        <v>40.52</v>
       </c>
       <c r="F92" s="17" t="inlineStr">
         <is>
@@ -2940,7 +2940,7 @@
         </is>
       </c>
       <c r="E93" s="29" t="n">
-        <v>31.32</v>
+        <v>28.43</v>
       </c>
       <c r="F93" s="17" t="inlineStr">
         <is>
@@ -2970,7 +2970,7 @@
         </is>
       </c>
       <c r="E94" s="29" t="n">
-        <v>18.52</v>
+        <v>20.77</v>
       </c>
       <c r="F94" s="17" t="inlineStr">
         <is>
@@ -3176,7 +3176,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-09-09 09:14 KST</t>
+          <t>2026-09-09 09:21 KST</t>
         </is>
       </c>
     </row>
@@ -4461,7 +4461,7 @@
         <v>5</v>
       </c>
       <c r="E69" t="n">
-        <v>40.59</v>
+        <v>40.81</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -4489,7 +4489,7 @@
         <v>5</v>
       </c>
       <c r="E70" t="n">
-        <v>37.21</v>
+        <v>37.02</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>5</v>
       </c>
       <c r="E71" t="n">
-        <v>10.23</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -4545,7 +4545,7 @@
         <v>5</v>
       </c>
       <c r="E72" t="n">
-        <v>12.31</v>
+        <v>19.5</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         <v>4</v>
       </c>
       <c r="E73" t="n">
-        <v>15.02</v>
+        <v>24.36</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -4601,7 +4601,7 @@
         <v>4</v>
       </c>
       <c r="E74" t="n">
-        <v>13.01</v>
+        <v>16.16</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -4629,7 +4629,7 @@
         <v>4</v>
       </c>
       <c r="E75" t="n">
-        <v>8.859999999999999</v>
+        <v>10.14</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -4657,7 +4657,7 @@
         <v>4</v>
       </c>
       <c r="E76" t="n">
-        <v>5.48</v>
+        <v>5.58</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -4685,7 +4685,7 @@
         <v>5</v>
       </c>
       <c r="E77" t="n">
-        <v>34.07</v>
+        <v>42.17</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -4713,7 +4713,7 @@
         <v>5</v>
       </c>
       <c r="E78" t="n">
-        <v>39.88</v>
+        <v>43.82</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -4741,7 +4741,7 @@
         <v>5</v>
       </c>
       <c r="E79" t="n">
-        <v>37.07</v>
+        <v>35.64</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -4769,7 +4769,7 @@
         <v>5</v>
       </c>
       <c r="E80" t="n">
-        <v>32.53</v>
+        <v>40.52</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -4797,7 +4797,7 @@
         <v>4</v>
       </c>
       <c r="E81" t="n">
-        <v>31.32</v>
+        <v>28.43</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
         <v>4</v>
       </c>
       <c r="E82" t="n">
-        <v>18.52</v>
+        <v>20.77</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>

</xml_diff>